<commit_message>
Mise a jour tresorerie juillet 2026
</commit_message>
<xml_diff>
--- a/Tresorerie_2026_Bely_v2.xlsx
+++ b/Tresorerie_2026_Bely_v2.xlsx
@@ -52,7 +52,7 @@
     <t xml:space="preserve">Juin ✅ réel</t>
   </si>
   <si>
-    <t xml:space="preserve">Juil 🔮 prévi</t>
+    <t xml:space="preserve">Juil ✅ réel</t>
   </si>
   <si>
     <t xml:space="preserve">Août 🔮 prévi</t>
@@ -409,8 +409,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -721,1876 +725,1882 @@
   <dimension ref="A1:P44"/>
   <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="59.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="59.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="O4" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <v>2200</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
         <v>2200</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="8" t="n">
         <v>2200</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="8" t="n">
         <v>2200</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="9" t="n">
         <v>3240</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="8" t="n">
         <v>2200</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="8" t="n">
         <v>2700</v>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="J6" s="8" t="n">
         <v>2700</v>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="K6" s="8" t="n">
         <v>2700</v>
       </c>
-      <c r="K6" s="7" t="n">
+      <c r="L6" s="8" t="n">
         <v>2700</v>
       </c>
-      <c r="L6" s="7" t="n">
+      <c r="M6" s="8" t="n">
         <v>2700</v>
       </c>
-      <c r="M6" s="7" t="n">
-        <v>2700</v>
-      </c>
-      <c r="N6" s="7" t="n">
+      <c r="N6" s="8" t="n">
         <f aca="false">SUM(B6:M6)</f>
-        <v>30440</v>
-      </c>
-      <c r="O6" s="7" t="n">
+        <v>27740</v>
+      </c>
+      <c r="O6" s="8" t="n">
         <f aca="false">IFERROR(N6/12,0)</f>
-        <v>2536.66666666667</v>
+        <v>2311.66666666667</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="8" t="n">
         <v>920</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="8" t="n">
         <v>920</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="8" t="n">
         <v>920</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="8" t="n">
         <v>920</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="9" t="n">
         <v>920</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G7" s="8" t="n">
         <v>920</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="8" t="n">
         <v>920</v>
       </c>
-      <c r="I7" s="7" t="n">
+      <c r="J7" s="8" t="n">
         <v>920</v>
       </c>
-      <c r="J7" s="7" t="n">
+      <c r="K7" s="8" t="n">
         <v>920</v>
       </c>
-      <c r="K7" s="7" t="n">
+      <c r="L7" s="8" t="n">
         <v>920</v>
       </c>
-      <c r="L7" s="7" t="n">
+      <c r="M7" s="8" t="n">
         <v>920</v>
       </c>
-      <c r="M7" s="7" t="n">
-        <v>920</v>
-      </c>
-      <c r="N7" s="7" t="n">
+      <c r="N7" s="8" t="n">
         <f aca="false">SUM(B7:M7)</f>
-        <v>11040</v>
-      </c>
-      <c r="O7" s="7" t="n">
+        <v>10120</v>
+      </c>
+      <c r="O7" s="8" t="n">
         <f aca="false">IFERROR(N7/12,0)</f>
-        <v>920</v>
+        <v>843.333333333333</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="9" t="n">
         <v>600</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="I8" s="7" t="n">
+      <c r="I8" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="J8" s="7" t="n">
+      <c r="J8" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="K8" s="7" t="n">
+      <c r="K8" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="L8" s="7" t="n">
+      <c r="L8" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="M8" s="7" t="n">
+      <c r="M8" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="N8" s="7" t="n">
+      <c r="N8" s="8" t="n">
         <f aca="false">SUM(B8:M8)</f>
         <v>7200</v>
       </c>
-      <c r="O8" s="7" t="n">
+      <c r="O8" s="8" t="n">
         <f aca="false">IFERROR(N8/12,0)</f>
         <v>600</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="8" t="n">
         <v>151</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="8" t="n">
         <v>151</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="8" t="n">
         <v>151</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="8" t="n">
         <v>151</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="9" t="n">
         <v>152</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="G9" s="8" t="n">
         <v>152</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="H9" s="8" t="n">
+        <v>152</v>
+      </c>
+      <c r="I9" s="8" t="n">
         <v>151</v>
       </c>
-      <c r="I9" s="7" t="n">
+      <c r="J9" s="8" t="n">
         <v>151</v>
       </c>
-      <c r="J9" s="7" t="n">
+      <c r="K9" s="8" t="n">
         <v>151</v>
       </c>
-      <c r="K9" s="7" t="n">
+      <c r="L9" s="8" t="n">
         <v>151</v>
       </c>
-      <c r="L9" s="7" t="n">
+      <c r="M9" s="8" t="n">
         <v>151</v>
       </c>
-      <c r="M9" s="7" t="n">
-        <v>151</v>
-      </c>
-      <c r="N9" s="7" t="n">
+      <c r="N9" s="8" t="n">
         <f aca="false">SUM(B9:M9)</f>
-        <v>1814</v>
-      </c>
-      <c r="O9" s="7" t="n">
+        <v>1815</v>
+      </c>
+      <c r="O9" s="8" t="n">
         <f aca="false">IFERROR(N9/12,0)</f>
-        <v>151.166666666667</v>
+        <v>151.25</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7" t="n">
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="I10" s="7" t="n">
+      <c r="J10" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="J10" s="7" t="n">
+      <c r="K10" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="K10" s="7" t="n">
+      <c r="L10" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="L10" s="7" t="n">
+      <c r="M10" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="M10" s="7" t="n">
-        <v>600</v>
-      </c>
-      <c r="N10" s="7" t="n">
+      <c r="N10" s="8" t="n">
         <f aca="false">SUM(B10:M10)</f>
-        <v>3600</v>
-      </c>
-      <c r="O10" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="O10" s="8" t="n">
         <f aca="false">IFERROR(N10/12,0)</f>
-        <v>300</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="8" t="n">
         <v>725</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="8" t="n">
         <v>1743</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="8" t="n">
         <v>1443</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="8" t="n">
         <v>812</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="9" t="n">
         <v>309</v>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="G11" s="8" t="n">
         <v>1595</v>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="H11" s="8" t="n">
+        <v>555</v>
+      </c>
+      <c r="I11" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="I11" s="7" t="n">
+      <c r="J11" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="J11" s="7" t="n">
+      <c r="K11" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="K11" s="7" t="n">
+      <c r="L11" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="L11" s="7" t="n">
+      <c r="M11" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="M11" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="N11" s="7" t="n">
+      <c r="N11" s="8" t="n">
         <f aca="false">SUM(B11:M11)</f>
-        <v>9027</v>
-      </c>
-      <c r="O11" s="7" t="n">
+        <v>9182</v>
+      </c>
+      <c r="O11" s="8" t="n">
         <f aca="false">IFERROR(N11/12,0)</f>
-        <v>752.25</v>
+        <v>765.166666666667</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="10" t="n">
         <f aca="false">SUM(B6:B11)</f>
         <v>4596</v>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="10" t="n">
         <f aca="false">SUM(C6:C11)</f>
         <v>5614</v>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="10" t="n">
         <f aca="false">SUM(D6:D11)</f>
         <v>5314</v>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="E12" s="10" t="n">
         <f aca="false">SUM(E6:E11)</f>
         <v>4683</v>
       </c>
-      <c r="F12" s="10" t="n">
+      <c r="F12" s="11" t="n">
         <f aca="false">SUM(F6:F11)</f>
         <v>5221</v>
       </c>
-      <c r="G12" s="9" t="n">
+      <c r="G12" s="10" t="n">
         <f aca="false">SUM(G6:G11)</f>
         <v>5467</v>
       </c>
-      <c r="H12" s="9" t="n">
+      <c r="H12" s="10" t="n">
         <f aca="false">SUM(H6:H11)</f>
-        <v>5371</v>
-      </c>
-      <c r="I12" s="9" t="n">
+        <v>1307</v>
+      </c>
+      <c r="I12" s="10" t="n">
         <f aca="false">SUM(I6:I11)</f>
         <v>5371</v>
       </c>
-      <c r="J12" s="9" t="n">
+      <c r="J12" s="10" t="n">
         <f aca="false">SUM(J6:J11)</f>
         <v>5371</v>
       </c>
-      <c r="K12" s="9" t="n">
+      <c r="K12" s="10" t="n">
         <f aca="false">SUM(K6:K11)</f>
         <v>5371</v>
       </c>
-      <c r="L12" s="9" t="n">
+      <c r="L12" s="10" t="n">
         <f aca="false">SUM(L6:L11)</f>
         <v>5371</v>
       </c>
-      <c r="M12" s="9" t="n">
+      <c r="M12" s="10" t="n">
         <f aca="false">SUM(M6:M11)</f>
         <v>5371</v>
       </c>
-      <c r="N12" s="9" t="n">
+      <c r="N12" s="10" t="n">
         <f aca="false">SUM(N6:N11)</f>
-        <v>63121</v>
-      </c>
-      <c r="O12" s="9" t="n">
+        <v>59057</v>
+      </c>
+      <c r="O12" s="10" t="n">
         <f aca="false">IFERROR(N12/12,0)</f>
-        <v>5260.08333333333</v>
+        <v>4921.41666666667</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="8" t="n">
         <v>154</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="8" t="n">
         <v>141</v>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="8" t="n">
         <v>141</v>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="E14" s="8" t="n">
         <v>142</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="9" t="n">
         <v>142</v>
       </c>
-      <c r="G14" s="7" t="n">
+      <c r="G14" s="8" t="n">
         <v>162</v>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="H14" s="8" t="n">
+        <v>142</v>
+      </c>
+      <c r="I14" s="8" t="n">
         <v>134</v>
       </c>
-      <c r="I14" s="7" t="n">
+      <c r="J14" s="8" t="n">
         <v>134</v>
       </c>
-      <c r="J14" s="7" t="n">
+      <c r="K14" s="8" t="n">
         <v>134</v>
       </c>
-      <c r="K14" s="7" t="n">
+      <c r="L14" s="8" t="n">
         <v>134</v>
       </c>
-      <c r="L14" s="7" t="n">
+      <c r="M14" s="8" t="n">
         <v>134</v>
       </c>
-      <c r="M14" s="7" t="n">
-        <v>134</v>
-      </c>
-      <c r="N14" s="7" t="n">
+      <c r="N14" s="8" t="n">
         <f aca="false">SUM(B14:M14)</f>
-        <v>1686</v>
-      </c>
-      <c r="O14" s="7" t="n">
+        <v>1694</v>
+      </c>
+      <c r="O14" s="8" t="n">
         <f aca="false">IFERROR(N14/12,0)</f>
-        <v>140.5</v>
+        <v>141.166666666667</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="9" t="n">
         <v>35</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="G15" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="I15" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="I15" s="7" t="n">
+      <c r="J15" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="J15" s="7" t="n">
+      <c r="K15" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="K15" s="7" t="n">
+      <c r="L15" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="L15" s="7" t="n">
+      <c r="M15" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="M15" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="N15" s="7" t="n">
+      <c r="N15" s="8" t="n">
         <f aca="false">SUM(B15:M15)</f>
-        <v>420</v>
-      </c>
-      <c r="O15" s="7" t="n">
+        <v>423</v>
+      </c>
+      <c r="O15" s="8" t="n">
         <f aca="false">IFERROR(N15/12,0)</f>
-        <v>35</v>
+        <v>35.25</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="E16" s="7"/>
-      <c r="F16" s="8" t="n">
+      <c r="E16" s="8"/>
+      <c r="F16" s="9" t="n">
         <v>81</v>
       </c>
-      <c r="G16" s="7" t="n">
+      <c r="G16" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="H16" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="I16" s="7" t="n">
+      <c r="I16" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="J16" s="7" t="n">
+      <c r="J16" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="K16" s="7" t="n">
+      <c r="K16" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="L16" s="7" t="n">
+      <c r="L16" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="M16" s="7" t="n">
+      <c r="M16" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="N16" s="7" t="n">
+      <c r="N16" s="8" t="n">
         <f aca="false">SUM(B16:M16)</f>
         <v>891</v>
       </c>
-      <c r="O16" s="7" t="n">
+      <c r="O16" s="8" t="n">
         <f aca="false">IFERROR(N16/12,0)</f>
         <v>74.25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="7" t="n">
+      <c r="B17" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E17" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="F17" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="G17" s="7" t="n">
+      <c r="G17" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="H17" s="7" t="n">
+      <c r="H17" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="I17" s="7" t="n">
+      <c r="I17" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="J17" s="7" t="n">
+      <c r="J17" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="K17" s="7" t="n">
+      <c r="K17" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="L17" s="7" t="n">
+      <c r="L17" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="M17" s="7" t="n">
+      <c r="M17" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="N17" s="7" t="n">
+      <c r="N17" s="8" t="n">
         <f aca="false">SUM(B17:M17)</f>
         <v>725</v>
       </c>
-      <c r="O17" s="7" t="n">
+      <c r="O17" s="8" t="n">
         <f aca="false">IFERROR(N17/12,0)</f>
         <v>60.4166666666667</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B18" s="8" t="n">
         <v>74</v>
       </c>
-      <c r="C18" s="7" t="n">
+      <c r="C18" s="8" t="n">
         <v>64</v>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D18" s="8" t="n">
         <v>64</v>
       </c>
-      <c r="E18" s="7" t="n">
+      <c r="E18" s="8" t="n">
         <v>70</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F18" s="9" t="n">
         <v>92</v>
       </c>
-      <c r="G18" s="7" t="n">
+      <c r="G18" s="8" t="n">
         <v>86</v>
       </c>
-      <c r="H18" s="7" t="n">
+      <c r="H18" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="I18" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="I18" s="7" t="n">
+      <c r="J18" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="J18" s="7" t="n">
+      <c r="K18" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="K18" s="7" t="n">
+      <c r="L18" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="L18" s="7" t="n">
+      <c r="M18" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="M18" s="7" t="n">
-        <v>66</v>
-      </c>
-      <c r="N18" s="7" t="n">
+      <c r="N18" s="8" t="n">
         <f aca="false">SUM(B18:M18)</f>
-        <v>846</v>
-      </c>
-      <c r="O18" s="7" t="n">
+        <v>872</v>
+      </c>
+      <c r="O18" s="8" t="n">
         <f aca="false">IFERROR(N18/12,0)</f>
-        <v>70.5</v>
+        <v>72.6666666666667</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7" t="n">
+      <c r="B19" s="8"/>
+      <c r="C19" s="8" t="n">
         <v>561</v>
       </c>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7" t="n">
+      <c r="D19" s="8"/>
+      <c r="E19" s="8" t="n">
         <v>377</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="F19" s="9" t="n">
         <v>173</v>
       </c>
-      <c r="G19" s="7" t="n">
+      <c r="G19" s="8" t="n">
         <v>159</v>
       </c>
-      <c r="H19" s="7" t="n">
+      <c r="H19" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="I19" s="8" t="n">
         <v>235</v>
       </c>
-      <c r="I19" s="7" t="n">
+      <c r="J19" s="8" t="n">
         <v>235</v>
       </c>
-      <c r="J19" s="7" t="n">
+      <c r="K19" s="8" t="n">
         <v>235</v>
       </c>
-      <c r="K19" s="7" t="n">
+      <c r="L19" s="8" t="n">
         <v>235</v>
       </c>
-      <c r="L19" s="7" t="n">
+      <c r="M19" s="8" t="n">
         <v>235</v>
       </c>
-      <c r="M19" s="7" t="n">
-        <v>235</v>
-      </c>
-      <c r="N19" s="7" t="n">
+      <c r="N19" s="8" t="n">
         <f aca="false">SUM(B19:M19)</f>
-        <v>2680</v>
-      </c>
-      <c r="O19" s="7" t="n">
+        <v>2651</v>
+      </c>
+      <c r="O19" s="8" t="n">
         <f aca="false">IFERROR(N19/12,0)</f>
-        <v>223.333333333333</v>
+        <v>220.916666666667</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="7" t="n">
+      <c r="B20" s="8" t="n">
         <v>254</v>
       </c>
-      <c r="C20" s="7" t="n">
+      <c r="C20" s="8" t="n">
         <v>254</v>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D20" s="8" t="n">
         <v>254</v>
       </c>
-      <c r="E20" s="7" t="n">
+      <c r="E20" s="8" t="n">
         <v>254</v>
       </c>
-      <c r="F20" s="8" t="n">
+      <c r="F20" s="9" t="n">
         <v>254</v>
       </c>
-      <c r="G20" s="7" t="n">
+      <c r="G20" s="8" t="n">
         <v>254</v>
       </c>
-      <c r="H20" s="7" t="n">
+      <c r="H20" s="8" t="n">
         <v>254</v>
       </c>
-      <c r="I20" s="7" t="n">
+      <c r="I20" s="8" t="n">
         <v>254</v>
       </c>
-      <c r="J20" s="7" t="n">
+      <c r="J20" s="8" t="n">
         <v>254</v>
       </c>
-      <c r="K20" s="7" t="n">
+      <c r="K20" s="8" t="n">
         <v>254</v>
       </c>
-      <c r="L20" s="7" t="n">
+      <c r="L20" s="8" t="n">
         <v>254</v>
       </c>
-      <c r="M20" s="7" t="n">
+      <c r="M20" s="8" t="n">
         <v>254</v>
       </c>
-      <c r="N20" s="7" t="n">
+      <c r="N20" s="8" t="n">
         <f aca="false">SUM(B20:M20)</f>
         <v>3048</v>
       </c>
-      <c r="O20" s="7" t="n">
+      <c r="O20" s="8" t="n">
         <f aca="false">IFERROR(N20/12,0)</f>
         <v>254</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="7" t="n">
+      <c r="B21" s="8" t="n">
         <v>147</v>
       </c>
-      <c r="C21" s="7" t="n">
+      <c r="C21" s="8" t="n">
         <v>147</v>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D21" s="8" t="n">
         <v>147</v>
       </c>
-      <c r="E21" s="7" t="n">
+      <c r="E21" s="8" t="n">
         <v>147</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="F21" s="9" t="n">
         <v>147</v>
       </c>
-      <c r="G21" s="7" t="n">
+      <c r="G21" s="8" t="n">
         <v>147</v>
       </c>
-      <c r="H21" s="7" t="n">
+      <c r="H21" s="8" t="n">
         <v>147</v>
       </c>
-      <c r="I21" s="7" t="n">
+      <c r="I21" s="8" t="n">
         <v>147</v>
       </c>
-      <c r="J21" s="7" t="n">
+      <c r="J21" s="8" t="n">
         <v>147</v>
       </c>
-      <c r="K21" s="7" t="n">
+      <c r="K21" s="8" t="n">
         <v>147</v>
       </c>
-      <c r="L21" s="7" t="n">
+      <c r="L21" s="8" t="n">
         <v>147</v>
       </c>
-      <c r="M21" s="7" t="n">
+      <c r="M21" s="8" t="n">
         <v>147</v>
       </c>
-      <c r="N21" s="7" t="n">
+      <c r="N21" s="8" t="n">
         <f aca="false">SUM(B21:M21)</f>
         <v>1764</v>
       </c>
-      <c r="O21" s="7" t="n">
+      <c r="O21" s="8" t="n">
         <f aca="false">IFERROR(N21/12,0)</f>
         <v>147</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="7" t="n">
+      <c r="B22" s="8" t="n">
         <v>164</v>
       </c>
-      <c r="C22" s="7" t="n">
+      <c r="C22" s="8" t="n">
         <v>282</v>
       </c>
-      <c r="D22" s="7" t="n">
+      <c r="D22" s="8" t="n">
         <v>282</v>
       </c>
-      <c r="E22" s="7" t="n">
+      <c r="E22" s="8" t="n">
         <v>282</v>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="F22" s="9" t="n">
         <v>283</v>
       </c>
-      <c r="G22" s="7" t="n">
+      <c r="G22" s="8" t="n">
         <v>282</v>
       </c>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7" t="n">
+      <c r="H22" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8" t="n">
         <v>282</v>
       </c>
-      <c r="K22" s="7" t="n">
+      <c r="K22" s="8" t="n">
         <v>282</v>
       </c>
-      <c r="L22" s="7" t="n">
+      <c r="L22" s="8" t="n">
         <v>282</v>
       </c>
-      <c r="M22" s="7" t="n">
+      <c r="M22" s="8" t="n">
         <v>282</v>
       </c>
-      <c r="N22" s="7" t="n">
+      <c r="N22" s="8" t="n">
         <f aca="false">SUM(B22:M22)</f>
-        <v>2703</v>
-      </c>
-      <c r="O22" s="7" t="n">
+        <v>2806</v>
+      </c>
+      <c r="O22" s="8" t="n">
         <f aca="false">IFERROR(N22/12,0)</f>
-        <v>225.25</v>
+        <v>233.833333333333</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="7" t="n">
+      <c r="B23" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="C23" s="7" t="n">
+      <c r="C23" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="D23" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="E23" s="7" t="n">
+      <c r="E23" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F23" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="G23" s="7" t="n">
+      <c r="G23" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7" t="n">
+      <c r="H23" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="K23" s="7" t="n">
+      <c r="I23" s="8"/>
+      <c r="J23" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="L23" s="7" t="n">
+      <c r="K23" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="M23" s="7" t="n">
+      <c r="L23" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="N23" s="7" t="n">
+      <c r="M23" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="N23" s="8" t="n">
         <f aca="false">SUM(B23:M23)</f>
-        <v>600</v>
-      </c>
-      <c r="O23" s="7" t="n">
+        <v>660</v>
+      </c>
+      <c r="O23" s="8" t="n">
         <f aca="false">IFERROR(N23/12,0)</f>
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="7" t="n">
+      <c r="B24" s="8" t="n">
         <v>219</v>
       </c>
-      <c r="C24" s="7" t="n">
+      <c r="C24" s="8" t="n">
         <v>157</v>
       </c>
-      <c r="D24" s="7" t="n">
+      <c r="D24" s="8" t="n">
         <v>131</v>
       </c>
-      <c r="E24" s="7" t="n">
+      <c r="E24" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="F24" s="8" t="n">
+      <c r="F24" s="9" t="n">
         <v>190</v>
       </c>
-      <c r="G24" s="7" t="n">
+      <c r="G24" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="H24" s="7" t="n">
+      <c r="H24" s="8" t="n">
+        <v>123</v>
+      </c>
+      <c r="I24" s="8" t="n">
         <v>130</v>
       </c>
-      <c r="I24" s="7" t="n">
+      <c r="J24" s="8" t="n">
         <v>130</v>
       </c>
-      <c r="J24" s="7" t="n">
+      <c r="K24" s="8" t="n">
         <v>130</v>
       </c>
-      <c r="K24" s="7" t="n">
+      <c r="L24" s="8" t="n">
         <v>130</v>
       </c>
-      <c r="L24" s="7" t="n">
+      <c r="M24" s="8" t="n">
         <v>130</v>
       </c>
-      <c r="M24" s="7" t="n">
-        <v>130</v>
-      </c>
-      <c r="N24" s="7" t="n">
+      <c r="N24" s="8" t="n">
         <f aca="false">SUM(B24:M24)</f>
-        <v>1534</v>
-      </c>
-      <c r="O24" s="7" t="n">
+        <v>1527</v>
+      </c>
+      <c r="O24" s="8" t="n">
         <f aca="false">IFERROR(N24/12,0)</f>
-        <v>127.833333333333</v>
+        <v>127.25</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="7" t="n">
+      <c r="B25" s="8" t="n">
         <v>700</v>
       </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7" t="n">
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8" t="n">
         <v>1400</v>
       </c>
-      <c r="F25" s="8"/>
-      <c r="G25" s="7" t="n">
+      <c r="F25" s="9"/>
+      <c r="G25" s="8" t="n">
         <v>1000</v>
       </c>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7"/>
-      <c r="M25" s="7"/>
-      <c r="N25" s="7" t="n">
+      <c r="H25" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="8"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8" t="n">
         <f aca="false">SUM(B25:M25)</f>
-        <v>3100</v>
-      </c>
-      <c r="O25" s="7" t="n">
+        <v>3104</v>
+      </c>
+      <c r="O25" s="8" t="n">
         <f aca="false">IFERROR(N25/12,0)</f>
-        <v>258.333333333333</v>
+        <v>258.666666666667</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7" t="n">
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8" t="n">
         <v>494</v>
       </c>
-      <c r="F26" s="8"/>
-      <c r="G26" s="7" t="n">
+      <c r="F26" s="9"/>
+      <c r="G26" s="8" t="n">
         <v>466</v>
       </c>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7" t="n">
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8" t="n">
         <v>165</v>
       </c>
-      <c r="K26" s="7" t="n">
+      <c r="K26" s="8" t="n">
         <v>165</v>
       </c>
-      <c r="L26" s="7" t="n">
+      <c r="L26" s="8" t="n">
         <v>165</v>
       </c>
-      <c r="M26" s="7" t="n">
+      <c r="M26" s="8" t="n">
         <v>165</v>
       </c>
-      <c r="N26" s="7" t="n">
+      <c r="N26" s="8" t="n">
         <f aca="false">SUM(B26:M26)</f>
         <v>1620</v>
       </c>
-      <c r="O26" s="7" t="n">
+      <c r="O26" s="8" t="n">
         <f aca="false">IFERROR(N26/12,0)</f>
         <v>135</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7" t="n">
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8" t="n">
         <v>1500</v>
       </c>
-      <c r="F27" s="8" t="n">
+      <c r="F27" s="9" t="n">
         <v>200</v>
       </c>
-      <c r="G27" s="7" t="n">
+      <c r="G27" s="8" t="n">
         <v>500</v>
       </c>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
-      <c r="L27" s="7"/>
-      <c r="M27" s="7"/>
-      <c r="N27" s="7" t="n">
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8" t="n">
         <f aca="false">SUM(B27:M27)</f>
         <v>2200</v>
       </c>
-      <c r="O27" s="7" t="n">
+      <c r="O27" s="8" t="n">
         <f aca="false">IFERROR(N27/12,0)</f>
         <v>183.333333333333</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B28" s="9" t="n">
+      <c r="B28" s="10" t="n">
         <f aca="false">SUM(B14:B27)</f>
         <v>1948</v>
       </c>
-      <c r="C28" s="9" t="n">
+      <c r="C28" s="10" t="n">
         <f aca="false">SUM(C14:C27)</f>
         <v>1847</v>
       </c>
-      <c r="D28" s="9" t="n">
+      <c r="D28" s="10" t="n">
         <f aca="false">SUM(D14:D27)</f>
         <v>1255</v>
       </c>
-      <c r="E28" s="9" t="n">
+      <c r="E28" s="10" t="n">
         <f aca="false">SUM(E14:E27)</f>
         <v>4835</v>
       </c>
-      <c r="F28" s="10" t="n">
+      <c r="F28" s="11" t="n">
         <f aca="false">SUM(F14:F27)</f>
         <v>1717</v>
       </c>
-      <c r="G28" s="9" t="n">
+      <c r="G28" s="10" t="n">
         <f aca="false">SUM(G14:G27)</f>
         <v>3335</v>
       </c>
-      <c r="H28" s="9" t="n">
+      <c r="H28" s="10" t="n">
         <f aca="false">SUM(H14:H27)</f>
-        <v>1142</v>
-      </c>
-      <c r="I28" s="9" t="n">
+        <v>1310</v>
+      </c>
+      <c r="I28" s="10" t="n">
         <f aca="false">SUM(I14:I27)</f>
         <v>1142</v>
       </c>
-      <c r="J28" s="9" t="n">
+      <c r="J28" s="10" t="n">
         <f aca="false">SUM(J14:J27)</f>
         <v>1649</v>
       </c>
-      <c r="K28" s="9" t="n">
+      <c r="K28" s="10" t="n">
         <f aca="false">SUM(K14:K27)</f>
         <v>1649</v>
       </c>
-      <c r="L28" s="9" t="n">
+      <c r="L28" s="10" t="n">
         <f aca="false">SUM(L14:L27)</f>
         <v>1649</v>
       </c>
-      <c r="M28" s="9" t="n">
+      <c r="M28" s="10" t="n">
         <f aca="false">SUM(M14:M27)</f>
         <v>1649</v>
       </c>
-      <c r="N28" s="9" t="n">
+      <c r="N28" s="10" t="n">
         <f aca="false">SUM(N14:N27)</f>
-        <v>23817</v>
-      </c>
-      <c r="O28" s="9" t="n">
+        <v>23985</v>
+      </c>
+      <c r="O28" s="10" t="n">
         <f aca="false">IFERROR(N28/12,0)</f>
-        <v>1984.75</v>
+        <v>1998.75</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
-      <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="6"/>
+      <c r="K29" s="6"/>
+      <c r="L29" s="6"/>
+      <c r="M29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B30" s="7" t="n">
+      <c r="B30" s="8" t="n">
         <v>250</v>
       </c>
-      <c r="C30" s="7" t="n">
+      <c r="C30" s="8" t="n">
         <v>230</v>
       </c>
-      <c r="D30" s="7" t="n">
+      <c r="D30" s="8" t="n">
         <v>260</v>
       </c>
-      <c r="E30" s="7" t="n">
+      <c r="E30" s="8" t="n">
         <v>200</v>
       </c>
-      <c r="F30" s="8" t="n">
+      <c r="F30" s="9" t="n">
         <v>834</v>
       </c>
-      <c r="G30" s="7" t="n">
+      <c r="G30" s="8" t="n">
         <v>569</v>
       </c>
-      <c r="H30" s="7" t="n">
+      <c r="H30" s="8" t="n">
+        <v>801</v>
+      </c>
+      <c r="I30" s="8" t="n">
         <v>235</v>
       </c>
-      <c r="I30" s="7" t="n">
+      <c r="J30" s="8" t="n">
         <v>235</v>
       </c>
-      <c r="J30" s="7" t="n">
+      <c r="K30" s="8" t="n">
         <v>235</v>
       </c>
-      <c r="K30" s="7" t="n">
+      <c r="L30" s="8" t="n">
         <v>235</v>
       </c>
-      <c r="L30" s="7" t="n">
+      <c r="M30" s="8" t="n">
         <v>235</v>
       </c>
-      <c r="M30" s="7" t="n">
-        <v>235</v>
-      </c>
-      <c r="N30" s="7" t="n">
+      <c r="N30" s="8" t="n">
         <f aca="false">SUM(B30:M30)</f>
-        <v>3753</v>
-      </c>
-      <c r="O30" s="7" t="n">
+        <v>4319</v>
+      </c>
+      <c r="O30" s="8" t="n">
         <f aca="false">IFERROR(N30/12,0)</f>
-        <v>312.75</v>
+        <v>359.916666666667</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B31" s="7" t="n">
+      <c r="B31" s="8" t="n">
         <v>450</v>
       </c>
-      <c r="C31" s="7" t="n">
+      <c r="C31" s="8" t="n">
         <v>380</v>
       </c>
-      <c r="D31" s="7" t="n">
+      <c r="D31" s="8" t="n">
         <v>480</v>
       </c>
-      <c r="E31" s="7" t="n">
+      <c r="E31" s="8" t="n">
         <v>500</v>
       </c>
-      <c r="F31" s="8" t="n">
+      <c r="F31" s="9" t="n">
         <v>312</v>
       </c>
-      <c r="G31" s="7" t="n">
+      <c r="G31" s="8" t="n">
         <v>347</v>
       </c>
-      <c r="H31" s="7" t="n">
+      <c r="H31" s="8" t="n">
+        <v>579</v>
+      </c>
+      <c r="I31" s="8" t="n">
         <v>453</v>
       </c>
-      <c r="I31" s="7" t="n">
+      <c r="J31" s="8" t="n">
         <v>453</v>
       </c>
-      <c r="J31" s="7" t="n">
+      <c r="K31" s="8" t="n">
         <v>453</v>
       </c>
-      <c r="K31" s="7" t="n">
+      <c r="L31" s="8" t="n">
         <v>453</v>
       </c>
-      <c r="L31" s="7" t="n">
+      <c r="M31" s="8" t="n">
         <v>453</v>
       </c>
-      <c r="M31" s="7" t="n">
-        <v>453</v>
-      </c>
-      <c r="N31" s="7" t="n">
+      <c r="N31" s="8" t="n">
         <f aca="false">SUM(B31:M31)</f>
-        <v>5187</v>
-      </c>
-      <c r="O31" s="7" t="n">
+        <v>5313</v>
+      </c>
+      <c r="O31" s="8" t="n">
         <f aca="false">IFERROR(N31/12,0)</f>
-        <v>432.25</v>
+        <v>442.75</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B32" s="7" t="n">
+      <c r="B32" s="8" t="n">
         <v>850</v>
       </c>
-      <c r="C32" s="7" t="n">
+      <c r="C32" s="8" t="n">
         <v>520</v>
       </c>
-      <c r="D32" s="7" t="n">
+      <c r="D32" s="8" t="n">
         <v>380</v>
       </c>
-      <c r="E32" s="7" t="n">
+      <c r="E32" s="8" t="n">
         <v>620</v>
       </c>
-      <c r="F32" s="8" t="n">
+      <c r="F32" s="9" t="n">
         <v>632</v>
       </c>
-      <c r="G32" s="7" t="n">
+      <c r="G32" s="8" t="n">
         <v>546</v>
       </c>
-      <c r="H32" s="7" t="n">
+      <c r="H32" s="8" t="n">
+        <v>876</v>
+      </c>
+      <c r="I32" s="8" t="n">
         <v>593</v>
       </c>
-      <c r="I32" s="7" t="n">
+      <c r="J32" s="8" t="n">
         <v>593</v>
       </c>
-      <c r="J32" s="7" t="n">
+      <c r="K32" s="8" t="n">
         <v>593</v>
       </c>
-      <c r="K32" s="7" t="n">
+      <c r="L32" s="8" t="n">
         <v>593</v>
       </c>
-      <c r="L32" s="7" t="n">
+      <c r="M32" s="8" t="n">
         <v>593</v>
       </c>
-      <c r="M32" s="7" t="n">
-        <v>593</v>
-      </c>
-      <c r="N32" s="7" t="n">
+      <c r="N32" s="8" t="n">
         <f aca="false">SUM(B32:M32)</f>
-        <v>7106</v>
-      </c>
-      <c r="O32" s="7" t="n">
+        <v>7389</v>
+      </c>
+      <c r="O32" s="8" t="n">
         <f aca="false">IFERROR(N32/12,0)</f>
-        <v>592.166666666667</v>
+        <v>615.75</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="6" t="s">
+      <c r="A33" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B33" s="7" t="n">
+      <c r="B33" s="8" t="n">
         <v>200</v>
       </c>
-      <c r="C33" s="7" t="n">
+      <c r="C33" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="D33" s="7" t="n">
+      <c r="D33" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="E33" s="7" t="n">
+      <c r="E33" s="8" t="n">
         <v>120</v>
       </c>
-      <c r="F33" s="8" t="n">
+      <c r="F33" s="9" t="n">
         <v>190</v>
       </c>
-      <c r="G33" s="7" t="n">
+      <c r="G33" s="8" t="n">
         <v>66</v>
       </c>
-      <c r="H33" s="7" t="n">
+      <c r="H33" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="I33" s="8" t="n">
         <v>111</v>
       </c>
-      <c r="I33" s="7" t="n">
+      <c r="J33" s="8" t="n">
         <v>111</v>
       </c>
-      <c r="J33" s="7" t="n">
+      <c r="K33" s="8" t="n">
         <v>111</v>
       </c>
-      <c r="K33" s="7" t="n">
+      <c r="L33" s="8" t="n">
         <v>111</v>
       </c>
-      <c r="L33" s="7" t="n">
+      <c r="M33" s="8" t="n">
         <v>111</v>
       </c>
-      <c r="M33" s="7" t="n">
-        <v>111</v>
-      </c>
-      <c r="N33" s="7" t="n">
+      <c r="N33" s="8" t="n">
         <f aca="false">SUM(B33:M33)</f>
-        <v>1367</v>
-      </c>
-      <c r="O33" s="7" t="n">
+        <v>1300</v>
+      </c>
+      <c r="O33" s="8" t="n">
         <f aca="false">IFERROR(N33/12,0)</f>
-        <v>113.916666666667</v>
+        <v>108.333333333333</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B34" s="7" t="n">
+      <c r="B34" s="8" t="n">
         <v>200</v>
       </c>
-      <c r="C34" s="7" t="n">
+      <c r="C34" s="8" t="n">
         <v>280</v>
       </c>
-      <c r="D34" s="7" t="n">
+      <c r="D34" s="8" t="n">
         <v>480</v>
       </c>
-      <c r="E34" s="7" t="n">
+      <c r="E34" s="8" t="n">
         <v>380</v>
       </c>
-      <c r="F34" s="8" t="n">
+      <c r="F34" s="9" t="n">
         <v>432</v>
       </c>
-      <c r="G34" s="7" t="n">
+      <c r="G34" s="8" t="n">
         <v>251</v>
       </c>
-      <c r="H34" s="7" t="n">
+      <c r="H34" s="8" t="n">
+        <v>559</v>
+      </c>
+      <c r="I34" s="8" t="n">
         <v>335</v>
       </c>
-      <c r="I34" s="7" t="n">
+      <c r="J34" s="8" t="n">
         <v>335</v>
       </c>
-      <c r="J34" s="7" t="n">
+      <c r="K34" s="8" t="n">
         <v>335</v>
       </c>
-      <c r="K34" s="7" t="n">
+      <c r="L34" s="8" t="n">
         <v>335</v>
       </c>
-      <c r="L34" s="7" t="n">
+      <c r="M34" s="8" t="n">
         <v>335</v>
       </c>
-      <c r="M34" s="7" t="n">
-        <v>335</v>
-      </c>
-      <c r="N34" s="7" t="n">
+      <c r="N34" s="8" t="n">
         <f aca="false">SUM(B34:M34)</f>
-        <v>4033</v>
-      </c>
-      <c r="O34" s="7" t="n">
+        <v>4257</v>
+      </c>
+      <c r="O34" s="8" t="n">
         <f aca="false">IFERROR(N34/12,0)</f>
-        <v>336.083333333333</v>
+        <v>354.75</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="s">
+      <c r="A35" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B35" s="7" t="n">
+      <c r="B35" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="C35" s="7" t="n">
+      <c r="C35" s="8" t="n">
         <v>290</v>
       </c>
-      <c r="D35" s="7" t="n">
+      <c r="D35" s="8" t="n">
         <v>245</v>
       </c>
-      <c r="E35" s="7" t="n">
+      <c r="E35" s="8" t="n">
         <v>85</v>
       </c>
-      <c r="F35" s="8" t="n">
+      <c r="F35" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="G35" s="7" t="n">
+      <c r="G35" s="8" t="n">
         <v>1500</v>
       </c>
-      <c r="H35" s="7" t="n">
-        <v>800</v>
-      </c>
-      <c r="I35" s="7" t="n">
+      <c r="H35" s="8" t="n">
+        <v>395</v>
+      </c>
+      <c r="I35" s="8" t="n">
         <v>1500</v>
       </c>
-      <c r="J35" s="7"/>
-      <c r="K35" s="7"/>
-      <c r="L35" s="7"/>
-      <c r="M35" s="7"/>
-      <c r="N35" s="7" t="n">
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
+      <c r="N35" s="8" t="n">
         <f aca="false">SUM(B35:M35)</f>
-        <v>4520</v>
-      </c>
-      <c r="O35" s="7" t="n">
+        <v>4115</v>
+      </c>
+      <c r="O35" s="8" t="n">
         <f aca="false">IFERROR(N35/12,0)</f>
-        <v>376.666666666667</v>
+        <v>342.916666666667</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
+      <c r="A36" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="7" t="n">
+      <c r="B36" s="8" t="n">
         <v>396</v>
       </c>
-      <c r="C36" s="7" t="n">
+      <c r="C36" s="8" t="n">
         <v>375</v>
       </c>
-      <c r="D36" s="7" t="n">
+      <c r="D36" s="8" t="n">
         <v>851</v>
       </c>
-      <c r="E36" s="7" t="n">
+      <c r="E36" s="8" t="n">
         <v>1276</v>
       </c>
-      <c r="F36" s="8" t="n">
+      <c r="F36" s="9" t="n">
         <v>401</v>
       </c>
-      <c r="G36" s="7" t="n">
+      <c r="G36" s="8" t="n">
         <v>1542</v>
       </c>
-      <c r="H36" s="7" t="n">
+      <c r="H36" s="8" t="n">
+        <v>1528</v>
+      </c>
+      <c r="I36" s="8" t="n">
         <v>725</v>
       </c>
-      <c r="I36" s="7" t="n">
+      <c r="J36" s="8" t="n">
         <v>725</v>
       </c>
-      <c r="J36" s="7" t="n">
+      <c r="K36" s="8" t="n">
         <v>725</v>
       </c>
-      <c r="K36" s="7" t="n">
+      <c r="L36" s="8" t="n">
         <v>725</v>
       </c>
-      <c r="L36" s="7" t="n">
+      <c r="M36" s="8" t="n">
         <v>725</v>
       </c>
-      <c r="M36" s="7" t="n">
-        <v>725</v>
-      </c>
-      <c r="N36" s="7" t="n">
+      <c r="N36" s="8" t="n">
         <f aca="false">SUM(B36:M36)</f>
-        <v>9191</v>
-      </c>
-      <c r="O36" s="7" t="n">
+        <v>9994</v>
+      </c>
+      <c r="O36" s="8" t="n">
         <f aca="false">IFERROR(N36/12,0)</f>
-        <v>765.916666666667</v>
+        <v>832.833333333333</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B37" s="9" t="n">
+      <c r="B37" s="10" t="n">
         <f aca="false">SUM(B30:B36)</f>
         <v>2426</v>
       </c>
-      <c r="C37" s="9" t="n">
+      <c r="C37" s="10" t="n">
         <f aca="false">SUM(C30:C36)</f>
         <v>2155</v>
       </c>
-      <c r="D37" s="9" t="n">
+      <c r="D37" s="10" t="n">
         <f aca="false">SUM(D30:D36)</f>
         <v>2741</v>
       </c>
-      <c r="E37" s="9" t="n">
+      <c r="E37" s="10" t="n">
         <f aca="false">SUM(E30:E36)</f>
         <v>3181</v>
       </c>
-      <c r="F37" s="10" t="n">
+      <c r="F37" s="11" t="n">
         <f aca="false">SUM(F30:F36)</f>
         <v>2821</v>
       </c>
-      <c r="G37" s="9" t="n">
+      <c r="G37" s="10" t="n">
         <f aca="false">SUM(G30:G36)</f>
         <v>4821</v>
       </c>
-      <c r="H37" s="9" t="n">
+      <c r="H37" s="10" t="n">
         <f aca="false">SUM(H30:H36)</f>
-        <v>3252</v>
-      </c>
-      <c r="I37" s="9" t="n">
+        <v>4782</v>
+      </c>
+      <c r="I37" s="10" t="n">
         <f aca="false">SUM(I30:I36)</f>
         <v>3952</v>
       </c>
-      <c r="J37" s="9" t="n">
+      <c r="J37" s="10" t="n">
         <f aca="false">SUM(J30:J36)</f>
         <v>2452</v>
       </c>
-      <c r="K37" s="9" t="n">
+      <c r="K37" s="10" t="n">
         <f aca="false">SUM(K30:K36)</f>
         <v>2452</v>
       </c>
-      <c r="L37" s="9" t="n">
+      <c r="L37" s="10" t="n">
         <f aca="false">SUM(L30:L36)</f>
         <v>2452</v>
       </c>
-      <c r="M37" s="9" t="n">
+      <c r="M37" s="10" t="n">
         <f aca="false">SUM(M30:M36)</f>
         <v>2452</v>
       </c>
-      <c r="N37" s="9" t="n">
+      <c r="N37" s="10" t="n">
         <f aca="false">SUM(N30:N36)</f>
-        <v>35157</v>
-      </c>
-      <c r="O37" s="9" t="n">
+        <v>36687</v>
+      </c>
+      <c r="O37" s="10" t="n">
         <f aca="false">IFERROR(N37/12,0)</f>
-        <v>2929.75</v>
+        <v>3057.25</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="11" t="s">
+      <c r="A38" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B38" s="11" t="n">
+      <c r="B38" s="12" t="n">
         <f aca="false">B28+B37</f>
         <v>4374</v>
       </c>
-      <c r="C38" s="11" t="n">
+      <c r="C38" s="12" t="n">
         <f aca="false">C28+C37</f>
         <v>4002</v>
       </c>
-      <c r="D38" s="11" t="n">
+      <c r="D38" s="12" t="n">
         <f aca="false">D28+D37</f>
         <v>3996</v>
       </c>
-      <c r="E38" s="11" t="n">
+      <c r="E38" s="12" t="n">
         <f aca="false">E28+E37</f>
         <v>8016</v>
       </c>
-      <c r="F38" s="11" t="n">
+      <c r="F38" s="12" t="n">
         <f aca="false">F28+F37</f>
         <v>4538</v>
       </c>
-      <c r="G38" s="11" t="n">
+      <c r="G38" s="12" t="n">
         <f aca="false">G28+G37</f>
         <v>8156</v>
       </c>
-      <c r="H38" s="11" t="n">
+      <c r="H38" s="12" t="n">
         <f aca="false">H28+H37</f>
-        <v>4394</v>
-      </c>
-      <c r="I38" s="11" t="n">
+        <v>6092</v>
+      </c>
+      <c r="I38" s="12" t="n">
         <f aca="false">I28+I37</f>
         <v>5094</v>
       </c>
-      <c r="J38" s="11" t="n">
+      <c r="J38" s="12" t="n">
         <f aca="false">J28+J37</f>
         <v>4101</v>
       </c>
-      <c r="K38" s="11" t="n">
+      <c r="K38" s="12" t="n">
         <f aca="false">K28+K37</f>
         <v>4101</v>
       </c>
-      <c r="L38" s="11" t="n">
+      <c r="L38" s="12" t="n">
         <f aca="false">L28+L37</f>
         <v>4101</v>
       </c>
-      <c r="M38" s="11" t="n">
+      <c r="M38" s="12" t="n">
         <f aca="false">M28+M37</f>
         <v>4101</v>
       </c>
-      <c r="N38" s="11" t="n">
+      <c r="N38" s="12" t="n">
         <f aca="false">N28+N37</f>
-        <v>58974</v>
-      </c>
-      <c r="O38" s="11" t="n">
+        <v>60672</v>
+      </c>
+      <c r="O38" s="12" t="n">
         <f aca="false">IFERROR(N38/12,0)</f>
-        <v>4914.5</v>
+        <v>5056</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="12" t="s">
+      <c r="A39" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B39" s="12" t="n">
+      <c r="B39" s="13" t="n">
         <f aca="false">B12-B28-B37</f>
         <v>222</v>
       </c>
-      <c r="C39" s="12" t="n">
+      <c r="C39" s="13" t="n">
         <f aca="false">C12-C28-C37</f>
         <v>1612</v>
       </c>
-      <c r="D39" s="12" t="n">
+      <c r="D39" s="13" t="n">
         <f aca="false">D12-D28-D37</f>
         <v>1318</v>
       </c>
-      <c r="E39" s="12" t="n">
+      <c r="E39" s="13" t="n">
         <f aca="false">E12-E28-E37</f>
         <v>-3333</v>
       </c>
-      <c r="F39" s="12" t="n">
+      <c r="F39" s="13" t="n">
         <f aca="false">F12-F28-F37</f>
         <v>683</v>
       </c>
-      <c r="G39" s="12" t="n">
+      <c r="G39" s="13" t="n">
         <f aca="false">G12-G28-G37</f>
         <v>-2689</v>
       </c>
-      <c r="H39" s="12" t="n">
+      <c r="H39" s="13" t="n">
         <f aca="false">H12-H28-H37</f>
-        <v>977</v>
-      </c>
-      <c r="I39" s="12" t="n">
+        <v>-4785</v>
+      </c>
+      <c r="I39" s="13" t="n">
         <f aca="false">I12-I28-I37</f>
         <v>277</v>
       </c>
-      <c r="J39" s="12" t="n">
+      <c r="J39" s="13" t="n">
         <f aca="false">J12-J28-J37</f>
         <v>1270</v>
       </c>
-      <c r="K39" s="12" t="n">
+      <c r="K39" s="13" t="n">
         <f aca="false">K12-K28-K37</f>
         <v>1270</v>
       </c>
-      <c r="L39" s="12" t="n">
+      <c r="L39" s="13" t="n">
         <f aca="false">L12-L28-L37</f>
         <v>1270</v>
       </c>
-      <c r="M39" s="12" t="n">
+      <c r="M39" s="13" t="n">
         <f aca="false">M12-M28-M37</f>
         <v>1270</v>
       </c>
-      <c r="N39" s="12" t="n">
+      <c r="N39" s="13" t="n">
         <f aca="false">N12-N28-N37</f>
-        <v>4147</v>
-      </c>
-      <c r="O39" s="12" t="n">
+        <v>-1615</v>
+      </c>
+      <c r="O39" s="13" t="n">
         <f aca="false">IFERROR(N39/12,0)</f>
-        <v>345.583333333333</v>
+        <v>-134.583333333333</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="12" t="s">
+      <c r="A40" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="B40" s="12" t="n">
+      <c r="B40" s="13" t="n">
         <v>-29</v>
       </c>
-      <c r="C40" s="12" t="n">
+      <c r="C40" s="13" t="n">
         <v>1540</v>
       </c>
-      <c r="D40" s="12" t="n">
+      <c r="D40" s="13" t="n">
         <v>2525</v>
       </c>
-      <c r="E40" s="12" t="n">
+      <c r="E40" s="13" t="n">
         <v>729</v>
       </c>
-      <c r="F40" s="12" t="n">
+      <c r="F40" s="13" t="n">
         <v>934</v>
       </c>
-      <c r="G40" s="12" t="n">
+      <c r="G40" s="13" t="n">
         <v>4978</v>
       </c>
-      <c r="H40" s="12" t="n">
-        <v>-34</v>
-      </c>
-      <c r="I40" s="12" t="n">
-        <v>245</v>
-      </c>
-      <c r="J40" s="12" t="n">
-        <v>1517</v>
-      </c>
-      <c r="K40" s="12" t="n">
-        <v>2788</v>
-      </c>
-      <c r="L40" s="12" t="n">
-        <v>4060</v>
-      </c>
-      <c r="M40" s="12" t="n">
-        <v>5331</v>
+      <c r="H40" s="13" t="n">
+        <v>2355</v>
+      </c>
+      <c r="I40" s="13" t="n">
+        <v>2632</v>
+      </c>
+      <c r="J40" s="13" t="n">
+        <v>3902</v>
+      </c>
+      <c r="K40" s="13" t="n">
+        <v>5172</v>
+      </c>
+      <c r="L40" s="13" t="n">
+        <v>6442</v>
+      </c>
+      <c r="M40" s="13" t="n">
+        <v>7712</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="B42" s="13"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="13"/>
-      <c r="G42" s="13"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="13"/>
-      <c r="J42" s="13"/>
-      <c r="K42" s="13"/>
-      <c r="L42" s="13"/>
-      <c r="M42" s="13"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="12" t="s">
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="14"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="14"/>
+      <c r="J42" s="14"/>
+      <c r="K42" s="14"/>
+      <c r="L42" s="14"/>
+      <c r="M42" s="14"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B43" s="12" t="n">
+      <c r="B43" s="13" t="n">
         <f aca="false">B12-B28</f>
         <v>2648</v>
       </c>
-      <c r="C43" s="12" t="n">
+      <c r="C43" s="13" t="n">
         <f aca="false">C12-C28</f>
         <v>3767</v>
       </c>
-      <c r="D43" s="12" t="n">
+      <c r="D43" s="13" t="n">
         <f aca="false">D12-D28</f>
         <v>4059</v>
       </c>
-      <c r="E43" s="12" t="n">
+      <c r="E43" s="13" t="n">
         <f aca="false">E12-E28</f>
         <v>-152</v>
       </c>
-      <c r="F43" s="12" t="n">
+      <c r="F43" s="13" t="n">
         <f aca="false">F12-F28</f>
         <v>3504</v>
       </c>
-      <c r="G43" s="12" t="n">
+      <c r="G43" s="13" t="n">
         <f aca="false">G12-G28</f>
         <v>2132</v>
       </c>
-      <c r="H43" s="12" t="n">
+      <c r="H43" s="13" t="n">
         <f aca="false">H12-H28</f>
-        <v>4229</v>
-      </c>
-      <c r="I43" s="12" t="n">
+        <v>-3</v>
+      </c>
+      <c r="I43" s="13" t="n">
         <f aca="false">I12-I28</f>
         <v>4229</v>
       </c>
-      <c r="J43" s="12" t="n">
+      <c r="J43" s="13" t="n">
         <f aca="false">J12-J28</f>
         <v>3722</v>
       </c>
-      <c r="K43" s="12" t="n">
+      <c r="K43" s="13" t="n">
         <f aca="false">K12-K28</f>
         <v>3722</v>
       </c>
-      <c r="L43" s="12" t="n">
+      <c r="L43" s="13" t="n">
         <f aca="false">L12-L28</f>
         <v>3722</v>
       </c>
-      <c r="M43" s="12" t="n">
+      <c r="M43" s="13" t="n">
         <f aca="false">M12-M28</f>
         <v>3722</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B44" s="12" t="n">
+      <c r="B44" s="13" t="n">
         <f aca="false">B39</f>
         <v>222</v>
       </c>
-      <c r="C44" s="12" t="n">
+      <c r="C44" s="13" t="n">
         <f aca="false">C39</f>
         <v>1612</v>
       </c>
-      <c r="D44" s="12" t="n">
+      <c r="D44" s="13" t="n">
         <f aca="false">D39</f>
         <v>1318</v>
       </c>
-      <c r="E44" s="12" t="n">
+      <c r="E44" s="13" t="n">
         <f aca="false">E39</f>
         <v>-3333</v>
       </c>
-      <c r="F44" s="12" t="n">
+      <c r="F44" s="13" t="n">
         <f aca="false">F39</f>
         <v>683</v>
       </c>
-      <c r="G44" s="12" t="n">
+      <c r="G44" s="13" t="n">
         <f aca="false">G39</f>
         <v>-2689</v>
       </c>
-      <c r="H44" s="12" t="n">
+      <c r="H44" s="13" t="n">
         <f aca="false">H39</f>
-        <v>977</v>
-      </c>
-      <c r="I44" s="12" t="n">
+        <v>-4785</v>
+      </c>
+      <c r="I44" s="13" t="n">
         <f aca="false">I39</f>
         <v>277</v>
       </c>
-      <c r="J44" s="12" t="n">
+      <c r="J44" s="13" t="n">
         <f aca="false">J39</f>
         <v>1270</v>
       </c>
-      <c r="K44" s="12" t="n">
+      <c r="K44" s="13" t="n">
         <f aca="false">K39</f>
         <v>1270</v>
       </c>
-      <c r="L44" s="12" t="n">
+      <c r="L44" s="13" t="n">
         <f aca="false">L39</f>
         <v>1270</v>
       </c>
-      <c r="M44" s="12" t="n">
+      <c r="M44" s="13" t="n">
         <f aca="false">M39</f>
         <v>1270</v>
       </c>

</xml_diff>

<commit_message>
Ajout ligne Revenus Revolut joint + recalcul entrées Jan-Juil 2026
</commit_message>
<xml_diff>
--- a/Tresorerie_2026_Bely_v2.xlsx
+++ b/Tresorerie_2026_Bely_v2.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t xml:space="preserve">TRÉSORERIE 2026 — FAMILLE BELY</t>
   </si>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t xml:space="preserve"> Revenus Audrey (archi, salaire, remb. pro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Revenus Revolut joint (Julien &amp; Audrey)</t>
   </si>
   <si>
     <t xml:space="preserve">Abely SASU (virement mensuel)</t>
@@ -722,7 +725,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P44"/>
+  <dimension ref="A1:P45"/>
   <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="59.85"/>
@@ -878,7 +881,7 @@
         <v>2200</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>0</v>
+        <v>1230</v>
       </c>
       <c r="I6" s="8" t="n">
         <v>2700</v>
@@ -897,11 +900,11 @@
       </c>
       <c r="N6" s="8" t="n">
         <f aca="false">SUM(B6:M6)</f>
-        <v>27740</v>
+        <v>28970</v>
       </c>
       <c r="O6" s="8" t="n">
         <f aca="false">IFERROR(N6/12,0)</f>
-        <v>2311.66666666667</v>
+        <v>2414.16666666667</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -927,7 +930,7 @@
         <v>920</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>0</v>
+        <v>850</v>
       </c>
       <c r="I7" s="8" t="n">
         <v>920</v>
@@ -946,11 +949,11 @@
       </c>
       <c r="N7" s="8" t="n">
         <f aca="false">SUM(B7:M7)</f>
-        <v>10120</v>
+        <v>10970</v>
       </c>
       <c r="O7" s="8" t="n">
         <f aca="false">IFERROR(N7/12,0)</f>
-        <v>843.333333333333</v>
+        <v>914.166666666667</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -958,359 +961,343 @@
         <v>21</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>600</v>
+        <v>1307</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>600</v>
+        <v>3935</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>600</v>
+        <v>3841</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>600</v>
+        <v>3447</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>600</v>
+        <v>2660</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>600</v>
+        <v>7490</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>600</v>
-      </c>
-      <c r="I8" s="8" t="n">
-        <v>600</v>
-      </c>
-      <c r="J8" s="8" t="n">
-        <v>600</v>
-      </c>
-      <c r="K8" s="8" t="n">
-        <v>600</v>
-      </c>
-      <c r="L8" s="8" t="n">
-        <v>600</v>
-      </c>
-      <c r="M8" s="8" t="n">
-        <v>600</v>
-      </c>
-      <c r="N8" s="8" t="n">
-        <f aca="false">SUM(B8:M8)</f>
-        <v>7200</v>
-      </c>
-      <c r="O8" s="8" t="n">
-        <f aca="false">IFERROR(N8/12,0)</f>
-        <v>600</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
         <v>22</v>
       </c>
       <c r="B9" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>152</v>
+        <v>600</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>152</v>
+        <v>600</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>152</v>
+        <v>600</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="M9" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="N9" s="8" t="n">
         <f aca="false">SUM(B9:M9)</f>
-        <v>1815</v>
+        <v>7200</v>
       </c>
       <c r="O9" s="8" t="n">
         <f aca="false">IFERROR(N9/12,0)</f>
-        <v>151.25</v>
+        <v>600</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="8"/>
+      <c r="B10" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>152</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>152</v>
+      </c>
       <c r="H10" s="8" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>600</v>
+        <v>151</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>600</v>
+        <v>151</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>600</v>
+        <v>151</v>
       </c>
       <c r="L10" s="8" t="n">
-        <v>600</v>
+        <v>151</v>
       </c>
       <c r="M10" s="8" t="n">
-        <v>600</v>
+        <v>151</v>
       </c>
       <c r="N10" s="8" t="n">
         <f aca="false">SUM(B10:M10)</f>
-        <v>3000</v>
+        <v>1815</v>
       </c>
       <c r="O10" s="8" t="n">
         <f aca="false">IFERROR(N10/12,0)</f>
-        <v>250</v>
+        <v>151.25</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="8" t="n">
-        <v>725</v>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>1743</v>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>1443</v>
-      </c>
-      <c r="E11" s="8" t="n">
-        <v>812</v>
-      </c>
-      <c r="F11" s="9" t="n">
-        <v>309</v>
-      </c>
-      <c r="G11" s="8" t="n">
-        <v>1595</v>
-      </c>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="8"/>
       <c r="H11" s="8" t="n">
-        <v>555</v>
+        <v>0</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="M11" s="8" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="N11" s="8" t="n">
         <f aca="false">SUM(B11:M11)</f>
-        <v>9182</v>
+        <v>3000</v>
       </c>
       <c r="O11" s="8" t="n">
         <f aca="false">IFERROR(N11/12,0)</f>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>1743</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>1443</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>812</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>309</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>1595</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>555</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <f aca="false">SUM(B12:M12)</f>
+        <v>9182</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <f aca="false">IFERROR(N12/12,0)</f>
         <v>765.166666666667</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="10" t="n">
-        <f aca="false">SUM(B6:B11)</f>
-        <v>4596</v>
-      </c>
-      <c r="C12" s="10" t="n">
-        <f aca="false">SUM(C6:C11)</f>
-        <v>5614</v>
-      </c>
-      <c r="D12" s="10" t="n">
-        <f aca="false">SUM(D6:D11)</f>
-        <v>5314</v>
-      </c>
-      <c r="E12" s="10" t="n">
-        <f aca="false">SUM(E6:E11)</f>
-        <v>4683</v>
-      </c>
-      <c r="F12" s="11" t="n">
-        <f aca="false">SUM(F6:F11)</f>
-        <v>5221</v>
-      </c>
-      <c r="G12" s="10" t="n">
-        <f aca="false">SUM(G6:G11)</f>
-        <v>5467</v>
-      </c>
-      <c r="H12" s="10" t="n">
-        <f aca="false">SUM(H6:H11)</f>
-        <v>1307</v>
-      </c>
-      <c r="I12" s="10" t="n">
-        <f aca="false">SUM(I6:I11)</f>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="10" t="n">
+        <f aca="false">SUM(B6:B12)</f>
+        <v>5903</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <f aca="false">SUM(C6:C12)</f>
+        <v>9549</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <f aca="false">SUM(D6:D12)</f>
+        <v>9155</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <f aca="false">SUM(E6:E12)</f>
+        <v>8130</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <f aca="false">SUM(F6:F12)</f>
+        <v>7881</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <f aca="false">SUM(G6:G12)</f>
+        <v>12957</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <f aca="false">SUM(H6:H12)</f>
+        <v>3387</v>
+      </c>
+      <c r="I13" s="10" t="n">
+        <f aca="false">SUM(I6:I12)</f>
         <v>5371</v>
       </c>
-      <c r="J12" s="10" t="n">
-        <f aca="false">SUM(J6:J11)</f>
+      <c r="J13" s="10" t="n">
+        <f aca="false">SUM(J6:J12)</f>
         <v>5371</v>
       </c>
-      <c r="K12" s="10" t="n">
-        <f aca="false">SUM(K6:K11)</f>
+      <c r="K13" s="10" t="n">
+        <f aca="false">SUM(K6:K12)</f>
         <v>5371</v>
       </c>
-      <c r="L12" s="10" t="n">
-        <f aca="false">SUM(L6:L11)</f>
+      <c r="L13" s="10" t="n">
+        <f aca="false">SUM(L6:L12)</f>
         <v>5371</v>
       </c>
-      <c r="M12" s="10" t="n">
-        <f aca="false">SUM(M6:M11)</f>
+      <c r="M13" s="10" t="n">
+        <f aca="false">SUM(M6:M12)</f>
         <v>5371</v>
       </c>
-      <c r="N12" s="10" t="n">
-        <f aca="false">SUM(N6:N11)</f>
-        <v>59057</v>
-      </c>
-      <c r="O12" s="10" t="n">
-        <f aca="false">IFERROR(N12/12,0)</f>
-        <v>4921.41666666667</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-    </row>
-    <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="N13" s="10" t="n">
+        <f aca="false">SUM(N6:N12)</f>
+        <v>61137</v>
+      </c>
+      <c r="O13" s="10" t="n">
+        <f aca="false">IFERROR(N13/12,0)</f>
+        <v>5094.75</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="8" t="n">
-        <v>154</v>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>141</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>141</v>
-      </c>
-      <c r="E14" s="8" t="n">
-        <v>142</v>
-      </c>
-      <c r="F14" s="9" t="n">
-        <v>142</v>
-      </c>
-      <c r="G14" s="8" t="n">
-        <v>162</v>
-      </c>
-      <c r="H14" s="8" t="n">
-        <v>142</v>
-      </c>
-      <c r="I14" s="8" t="n">
-        <v>134</v>
-      </c>
-      <c r="J14" s="8" t="n">
-        <v>134</v>
-      </c>
-      <c r="K14" s="8" t="n">
-        <v>134</v>
-      </c>
-      <c r="L14" s="8" t="n">
-        <v>134</v>
-      </c>
-      <c r="M14" s="8" t="n">
-        <v>134</v>
-      </c>
-      <c r="N14" s="8" t="n">
-        <f aca="false">SUM(B14:M14)</f>
-        <v>1694</v>
-      </c>
-      <c r="O14" s="8" t="n">
-        <f aca="false">IFERROR(N14/12,0)</f>
-        <v>141.166666666667</v>
-      </c>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
         <v>28</v>
       </c>
       <c r="B15" s="8" t="n">
-        <v>35</v>
+        <v>154</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>35</v>
+        <v>141</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>35</v>
+        <v>141</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>35</v>
+        <v>142</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>35</v>
+        <v>142</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>35</v>
+        <v>162</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>38</v>
+        <v>142</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>35</v>
+        <v>134</v>
       </c>
       <c r="J15" s="8" t="n">
-        <v>35</v>
+        <v>134</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>35</v>
+        <v>134</v>
       </c>
       <c r="L15" s="8" t="n">
-        <v>35</v>
+        <v>134</v>
       </c>
       <c r="M15" s="8" t="n">
-        <v>35</v>
+        <v>134</v>
       </c>
       <c r="N15" s="8" t="n">
         <f aca="false">SUM(B15:M15)</f>
-        <v>423</v>
+        <v>1694</v>
       </c>
       <c r="O15" s="8" t="n">
         <f aca="false">IFERROR(N15/12,0)</f>
-        <v>35.25</v>
+        <v>141.166666666667</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1318,46 +1305,48 @@
         <v>29</v>
       </c>
       <c r="B16" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>81</v>
-      </c>
-      <c r="E16" s="8"/>
+        <v>35</v>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>35</v>
+      </c>
       <c r="F16" s="9" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>81</v>
+        <v>38</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="J16" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="K16" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="L16" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="M16" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="N16" s="8" t="n">
         <f aca="false">SUM(B16:M16)</f>
-        <v>891</v>
+        <v>423</v>
       </c>
       <c r="O16" s="8" t="n">
         <f aca="false">IFERROR(N16/12,0)</f>
-        <v>74.25</v>
+        <v>35.25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1365,48 +1354,46 @@
         <v>30</v>
       </c>
       <c r="B17" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>60</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="E17" s="8"/>
       <c r="F17" s="9" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="J17" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="L17" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="M17" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="N17" s="8" t="n">
         <f aca="false">SUM(B17:M17)</f>
-        <v>725</v>
+        <v>891</v>
       </c>
       <c r="O17" s="8" t="n">
         <f aca="false">IFERROR(N17/12,0)</f>
-        <v>60.4166666666667</v>
+        <v>74.25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1414,142 +1401,142 @@
         <v>31</v>
       </c>
       <c r="B18" s="8" t="n">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="I18" s="8" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="L18" s="8" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="M18" s="8" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="N18" s="8" t="n">
         <f aca="false">SUM(B18:M18)</f>
-        <v>872</v>
+        <v>725</v>
       </c>
       <c r="O18" s="8" t="n">
         <f aca="false">IFERROR(N18/12,0)</f>
-        <v>72.6666666666667</v>
+        <v>60.4166666666667</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="8"/>
+      <c r="B19" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="C19" s="8" t="n">
-        <v>561</v>
-      </c>
-      <c r="D19" s="8"/>
+        <v>64</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>64</v>
+      </c>
       <c r="E19" s="8" t="n">
-        <v>377</v>
+        <v>70</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>173</v>
+        <v>92</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>159</v>
+        <v>86</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>206</v>
+        <v>92</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="J19" s="8" t="n">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="K19" s="8" t="n">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="L19" s="8" t="n">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="M19" s="8" t="n">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="N19" s="8" t="n">
         <f aca="false">SUM(B19:M19)</f>
-        <v>2651</v>
+        <v>872</v>
       </c>
       <c r="O19" s="8" t="n">
         <f aca="false">IFERROR(N19/12,0)</f>
-        <v>220.916666666667</v>
+        <v>72.6666666666667</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="8" t="n">
-        <v>254</v>
-      </c>
+      <c r="B20" s="8"/>
       <c r="C20" s="8" t="n">
-        <v>254</v>
-      </c>
-      <c r="D20" s="8" t="n">
-        <v>254</v>
-      </c>
+        <v>561</v>
+      </c>
+      <c r="D20" s="8"/>
       <c r="E20" s="8" t="n">
-        <v>254</v>
+        <v>377</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>254</v>
+        <v>173</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>254</v>
+        <v>159</v>
       </c>
       <c r="H20" s="8" t="n">
-        <v>254</v>
+        <v>206</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="M20" s="8" t="n">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="N20" s="8" t="n">
         <f aca="false">SUM(B20:M20)</f>
-        <v>3048</v>
+        <v>2651</v>
       </c>
       <c r="O20" s="8" t="n">
         <f aca="false">IFERROR(N20/12,0)</f>
-        <v>254</v>
+        <v>220.916666666667</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1557,48 +1544,48 @@
         <v>34</v>
       </c>
       <c r="B21" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="C21" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="J21" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="K21" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="L21" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="M21" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="N21" s="8" t="n">
         <f aca="false">SUM(B21:M21)</f>
-        <v>1764</v>
+        <v>3048</v>
       </c>
       <c r="O21" s="8" t="n">
         <f aca="false">IFERROR(N21/12,0)</f>
-        <v>147</v>
+        <v>254</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1606,46 +1593,48 @@
         <v>35</v>
       </c>
       <c r="B22" s="8" t="n">
-        <v>164</v>
+        <v>147</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>283</v>
+        <v>147</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="I22" s="8"/>
+        <v>147</v>
+      </c>
+      <c r="I22" s="8" t="n">
+        <v>147</v>
+      </c>
       <c r="J22" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="N22" s="8" t="n">
         <f aca="false">SUM(B22:M22)</f>
-        <v>2806</v>
+        <v>1764</v>
       </c>
       <c r="O22" s="8" t="n">
         <f aca="false">IFERROR(N22/12,0)</f>
-        <v>233.833333333333</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1653,46 +1642,46 @@
         <v>36</v>
       </c>
       <c r="B23" s="8" t="n">
-        <v>60</v>
+        <v>164</v>
       </c>
       <c r="C23" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>60</v>
+        <v>283</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="I23" s="8"/>
       <c r="J23" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="N23" s="8" t="n">
         <f aca="false">SUM(B23:M23)</f>
-        <v>660</v>
+        <v>2806</v>
       </c>
       <c r="O23" s="8" t="n">
         <f aca="false">IFERROR(N23/12,0)</f>
-        <v>55</v>
+        <v>233.833333333333</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1700,48 +1689,46 @@
         <v>37</v>
       </c>
       <c r="B24" s="8" t="n">
-        <v>219</v>
+        <v>60</v>
       </c>
       <c r="C24" s="8" t="n">
-        <v>157</v>
+        <v>60</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>131</v>
+        <v>60</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>190</v>
+        <v>60</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>123</v>
-      </c>
-      <c r="I24" s="8" t="n">
-        <v>130</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="I24" s="8"/>
       <c r="J24" s="8" t="n">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="L24" s="8" t="n">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="M24" s="8" t="n">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="N24" s="8" t="n">
         <f aca="false">SUM(B24:M24)</f>
-        <v>1527</v>
+        <v>660</v>
       </c>
       <c r="O24" s="8" t="n">
         <f aca="false">IFERROR(N24/12,0)</f>
-        <v>127.25</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1749,69 +1736,81 @@
         <v>38</v>
       </c>
       <c r="B25" s="8" t="n">
-        <v>700</v>
-      </c>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
+        <v>219</v>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>157</v>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>131</v>
+      </c>
       <c r="E25" s="8" t="n">
-        <v>1400</v>
-      </c>
-      <c r="F25" s="9"/>
+        <v>14</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>190</v>
+      </c>
       <c r="G25" s="8" t="n">
-        <v>1000</v>
+        <v>43</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
-      <c r="L25" s="8"/>
-      <c r="M25" s="8"/>
+        <v>123</v>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="J25" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="K25" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="L25" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="M25" s="8" t="n">
+        <v>130</v>
+      </c>
       <c r="N25" s="8" t="n">
         <f aca="false">SUM(B25:M25)</f>
-        <v>3104</v>
+        <v>1527</v>
       </c>
       <c r="O25" s="8" t="n">
         <f aca="false">IFERROR(N25/12,0)</f>
-        <v>258.666666666667</v>
+        <v>127.25</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="8"/>
+      <c r="B26" s="8" t="n">
+        <v>700</v>
+      </c>
       <c r="C26" s="8"/>
       <c r="D26" s="8"/>
       <c r="E26" s="8" t="n">
-        <v>494</v>
+        <v>1400</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="8" t="n">
-        <v>466</v>
-      </c>
-      <c r="H26" s="8"/>
+        <v>1000</v>
+      </c>
+      <c r="H26" s="8" t="n">
+        <v>4</v>
+      </c>
       <c r="I26" s="8"/>
-      <c r="J26" s="8" t="n">
-        <v>165</v>
-      </c>
-      <c r="K26" s="8" t="n">
-        <v>165</v>
-      </c>
-      <c r="L26" s="8" t="n">
-        <v>165</v>
-      </c>
-      <c r="M26" s="8" t="n">
-        <v>165</v>
-      </c>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+      <c r="M26" s="8"/>
       <c r="N26" s="8" t="n">
         <f aca="false">SUM(B26:M26)</f>
-        <v>1620</v>
+        <v>3104</v>
       </c>
       <c r="O26" s="8" t="n">
         <f aca="false">IFERROR(N26/12,0)</f>
-        <v>135</v>
+        <v>258.666666666667</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1822,203 +1821,191 @@
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
       <c r="E27" s="8" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F27" s="9" t="n">
-        <v>200</v>
-      </c>
+        <v>494</v>
+      </c>
+      <c r="F27" s="9"/>
       <c r="G27" s="8" t="n">
-        <v>500</v>
+        <v>466</v>
       </c>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
-      <c r="J27" s="8"/>
-      <c r="K27" s="8"/>
-      <c r="L27" s="8"/>
-      <c r="M27" s="8"/>
+      <c r="J27" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="K27" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="L27" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="M27" s="8" t="n">
+        <v>165</v>
+      </c>
       <c r="N27" s="8" t="n">
         <f aca="false">SUM(B27:M27)</f>
-        <v>2200</v>
+        <v>1620</v>
       </c>
       <c r="O27" s="8" t="n">
         <f aca="false">IFERROR(N27/12,0)</f>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8" t="n">
+        <f aca="false">SUM(B28:M28)</f>
+        <v>2200</v>
+      </c>
+      <c r="O28" s="8" t="n">
+        <f aca="false">IFERROR(N28/12,0)</f>
         <v>183.333333333333</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="B28" s="10" t="n">
-        <f aca="false">SUM(B14:B27)</f>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="10" t="n">
+        <f aca="false">SUM(B15:B28)</f>
         <v>1948</v>
       </c>
-      <c r="C28" s="10" t="n">
-        <f aca="false">SUM(C14:C27)</f>
+      <c r="C29" s="10" t="n">
+        <f aca="false">SUM(C15:C28)</f>
         <v>1847</v>
       </c>
-      <c r="D28" s="10" t="n">
-        <f aca="false">SUM(D14:D27)</f>
+      <c r="D29" s="10" t="n">
+        <f aca="false">SUM(D15:D28)</f>
         <v>1255</v>
       </c>
-      <c r="E28" s="10" t="n">
-        <f aca="false">SUM(E14:E27)</f>
+      <c r="E29" s="10" t="n">
+        <f aca="false">SUM(E15:E28)</f>
         <v>4835</v>
       </c>
-      <c r="F28" s="11" t="n">
-        <f aca="false">SUM(F14:F27)</f>
+      <c r="F29" s="11" t="n">
+        <f aca="false">SUM(F15:F28)</f>
         <v>1717</v>
       </c>
-      <c r="G28" s="10" t="n">
-        <f aca="false">SUM(G14:G27)</f>
+      <c r="G29" s="10" t="n">
+        <f aca="false">SUM(G15:G28)</f>
         <v>3335</v>
       </c>
-      <c r="H28" s="10" t="n">
-        <f aca="false">SUM(H14:H27)</f>
+      <c r="H29" s="10" t="n">
+        <f aca="false">SUM(H15:H28)</f>
         <v>1310</v>
       </c>
-      <c r="I28" s="10" t="n">
-        <f aca="false">SUM(I14:I27)</f>
+      <c r="I29" s="10" t="n">
+        <f aca="false">SUM(I15:I28)</f>
         <v>1142</v>
       </c>
-      <c r="J28" s="10" t="n">
-        <f aca="false">SUM(J14:J27)</f>
+      <c r="J29" s="10" t="n">
+        <f aca="false">SUM(J15:J28)</f>
         <v>1649</v>
       </c>
-      <c r="K28" s="10" t="n">
-        <f aca="false">SUM(K14:K27)</f>
+      <c r="K29" s="10" t="n">
+        <f aca="false">SUM(K15:K28)</f>
         <v>1649</v>
       </c>
-      <c r="L28" s="10" t="n">
-        <f aca="false">SUM(L14:L27)</f>
+      <c r="L29" s="10" t="n">
+        <f aca="false">SUM(L15:L28)</f>
         <v>1649</v>
       </c>
-      <c r="M28" s="10" t="n">
-        <f aca="false">SUM(M14:M27)</f>
+      <c r="M29" s="10" t="n">
+        <f aca="false">SUM(M15:M28)</f>
         <v>1649</v>
       </c>
-      <c r="N28" s="10" t="n">
-        <f aca="false">SUM(N14:N27)</f>
+      <c r="N29" s="10" t="n">
+        <f aca="false">SUM(N15:N28)</f>
         <v>23985</v>
       </c>
-      <c r="O28" s="10" t="n">
-        <f aca="false">IFERROR(N28/12,0)</f>
+      <c r="O29" s="10" t="n">
+        <f aca="false">IFERROR(N29/12,0)</f>
         <v>1998.75</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B29" s="6"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="6"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
-      <c r="I29" s="6"/>
-      <c r="J29" s="6"/>
-      <c r="K29" s="6"/>
-      <c r="L29" s="6"/>
-      <c r="M29" s="6"/>
-    </row>
-    <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
+    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B30" s="8" t="n">
-        <v>250</v>
-      </c>
-      <c r="C30" s="8" t="n">
-        <v>230</v>
-      </c>
-      <c r="D30" s="8" t="n">
-        <v>260</v>
-      </c>
-      <c r="E30" s="8" t="n">
-        <v>200</v>
-      </c>
-      <c r="F30" s="9" t="n">
-        <v>834</v>
-      </c>
-      <c r="G30" s="8" t="n">
-        <v>569</v>
-      </c>
-      <c r="H30" s="8" t="n">
-        <v>801</v>
-      </c>
-      <c r="I30" s="8" t="n">
-        <v>235</v>
-      </c>
-      <c r="J30" s="8" t="n">
-        <v>235</v>
-      </c>
-      <c r="K30" s="8" t="n">
-        <v>235</v>
-      </c>
-      <c r="L30" s="8" t="n">
-        <v>235</v>
-      </c>
-      <c r="M30" s="8" t="n">
-        <v>235</v>
-      </c>
-      <c r="N30" s="8" t="n">
-        <f aca="false">SUM(B30:M30)</f>
-        <v>4319</v>
-      </c>
-      <c r="O30" s="8" t="n">
-        <f aca="false">IFERROR(N30/12,0)</f>
-        <v>359.916666666667</v>
-      </c>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="6"/>
+      <c r="J30" s="6"/>
+      <c r="K30" s="6"/>
+      <c r="L30" s="6"/>
+      <c r="M30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
         <v>44</v>
       </c>
       <c r="B31" s="8" t="n">
-        <v>450</v>
+        <v>250</v>
       </c>
       <c r="C31" s="8" t="n">
-        <v>380</v>
+        <v>230</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>480</v>
+        <v>260</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>312</v>
+        <v>834</v>
       </c>
       <c r="G31" s="8" t="n">
-        <v>347</v>
+        <v>569</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>579</v>
+        <v>801</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>453</v>
+        <v>235</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>453</v>
+        <v>235</v>
       </c>
       <c r="K31" s="8" t="n">
-        <v>453</v>
+        <v>235</v>
       </c>
       <c r="L31" s="8" t="n">
-        <v>453</v>
+        <v>235</v>
       </c>
       <c r="M31" s="8" t="n">
-        <v>453</v>
+        <v>235</v>
       </c>
       <c r="N31" s="8" t="n">
         <f aca="false">SUM(B31:M31)</f>
-        <v>5313</v>
+        <v>4319</v>
       </c>
       <c r="O31" s="8" t="n">
         <f aca="false">IFERROR(N31/12,0)</f>
-        <v>442.75</v>
+        <v>359.916666666667</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2026,48 +2013,48 @@
         <v>45</v>
       </c>
       <c r="B32" s="8" t="n">
-        <v>850</v>
+        <v>450</v>
       </c>
       <c r="C32" s="8" t="n">
-        <v>520</v>
+        <v>380</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>380</v>
+        <v>480</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>620</v>
+        <v>500</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>632</v>
+        <v>312</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>546</v>
+        <v>347</v>
       </c>
       <c r="H32" s="8" t="n">
-        <v>876</v>
+        <v>579</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>593</v>
+        <v>453</v>
       </c>
       <c r="J32" s="8" t="n">
-        <v>593</v>
+        <v>453</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>593</v>
+        <v>453</v>
       </c>
       <c r="L32" s="8" t="n">
-        <v>593</v>
+        <v>453</v>
       </c>
       <c r="M32" s="8" t="n">
-        <v>593</v>
+        <v>453</v>
       </c>
       <c r="N32" s="8" t="n">
         <f aca="false">SUM(B32:M32)</f>
-        <v>7389</v>
+        <v>5313</v>
       </c>
       <c r="O32" s="8" t="n">
         <f aca="false">IFERROR(N32/12,0)</f>
-        <v>615.75</v>
+        <v>442.75</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2075,48 +2062,48 @@
         <v>46</v>
       </c>
       <c r="B33" s="8" t="n">
-        <v>200</v>
+        <v>850</v>
       </c>
       <c r="C33" s="8" t="n">
-        <v>80</v>
+        <v>520</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>45</v>
+        <v>380</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>120</v>
+        <v>620</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>190</v>
+        <v>632</v>
       </c>
       <c r="G33" s="8" t="n">
-        <v>66</v>
+        <v>546</v>
       </c>
       <c r="H33" s="8" t="n">
-        <v>44</v>
+        <v>876</v>
       </c>
       <c r="I33" s="8" t="n">
-        <v>111</v>
+        <v>593</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>111</v>
+        <v>593</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>111</v>
+        <v>593</v>
       </c>
       <c r="L33" s="8" t="n">
-        <v>111</v>
+        <v>593</v>
       </c>
       <c r="M33" s="8" t="n">
-        <v>111</v>
+        <v>593</v>
       </c>
       <c r="N33" s="8" t="n">
         <f aca="false">SUM(B33:M33)</f>
-        <v>1300</v>
+        <v>7389</v>
       </c>
       <c r="O33" s="8" t="n">
         <f aca="false">IFERROR(N33/12,0)</f>
-        <v>108.333333333333</v>
+        <v>615.75</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2127,45 +2114,45 @@
         <v>200</v>
       </c>
       <c r="C34" s="8" t="n">
-        <v>280</v>
+        <v>80</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>480</v>
+        <v>45</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>380</v>
+        <v>120</v>
       </c>
       <c r="F34" s="9" t="n">
-        <v>432</v>
+        <v>190</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>251</v>
+        <v>66</v>
       </c>
       <c r="H34" s="8" t="n">
-        <v>559</v>
+        <v>44</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>335</v>
+        <v>111</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>335</v>
+        <v>111</v>
       </c>
       <c r="K34" s="8" t="n">
-        <v>335</v>
+        <v>111</v>
       </c>
       <c r="L34" s="8" t="n">
-        <v>335</v>
+        <v>111</v>
       </c>
       <c r="M34" s="8" t="n">
-        <v>335</v>
+        <v>111</v>
       </c>
       <c r="N34" s="8" t="n">
         <f aca="false">SUM(B34:M34)</f>
-        <v>4257</v>
+        <v>1300</v>
       </c>
       <c r="O34" s="8" t="n">
         <f aca="false">IFERROR(N34/12,0)</f>
-        <v>354.75</v>
+        <v>108.333333333333</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2173,40 +2160,48 @@
         <v>48</v>
       </c>
       <c r="B35" s="8" t="n">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="C35" s="8" t="n">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>245</v>
+        <v>480</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>85</v>
+        <v>380</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>20</v>
+        <v>432</v>
       </c>
       <c r="G35" s="8" t="n">
-        <v>1500</v>
+        <v>251</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>395</v>
+        <v>559</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J35" s="8"/>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="8"/>
+        <v>335</v>
+      </c>
+      <c r="J35" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="K35" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="L35" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="M35" s="8" t="n">
+        <v>335</v>
+      </c>
       <c r="N35" s="8" t="n">
         <f aca="false">SUM(B35:M35)</f>
-        <v>4115</v>
+        <v>4257</v>
       </c>
       <c r="O35" s="8" t="n">
         <f aca="false">IFERROR(N35/12,0)</f>
-        <v>342.916666666667</v>
+        <v>354.75</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2214,231 +2209,211 @@
         <v>49</v>
       </c>
       <c r="B36" s="8" t="n">
-        <v>396</v>
+        <v>80</v>
       </c>
       <c r="C36" s="8" t="n">
-        <v>375</v>
+        <v>290</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>851</v>
+        <v>245</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>1276</v>
+        <v>85</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>401</v>
+        <v>20</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>1542</v>
+        <v>1500</v>
       </c>
       <c r="H36" s="8" t="n">
-        <v>1528</v>
+        <v>395</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>725</v>
-      </c>
-      <c r="J36" s="8" t="n">
-        <v>725</v>
-      </c>
-      <c r="K36" s="8" t="n">
-        <v>725</v>
-      </c>
-      <c r="L36" s="8" t="n">
-        <v>725</v>
-      </c>
-      <c r="M36" s="8" t="n">
-        <v>725</v>
-      </c>
+        <v>1500</v>
+      </c>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
+      <c r="M36" s="8"/>
       <c r="N36" s="8" t="n">
         <f aca="false">SUM(B36:M36)</f>
-        <v>9994</v>
+        <v>4115</v>
       </c>
       <c r="O36" s="8" t="n">
         <f aca="false">IFERROR(N36/12,0)</f>
+        <v>342.916666666667</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" s="8" t="n">
+        <v>396</v>
+      </c>
+      <c r="C37" s="8" t="n">
+        <v>375</v>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>851</v>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>1276</v>
+      </c>
+      <c r="F37" s="9" t="n">
+        <v>401</v>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>1542</v>
+      </c>
+      <c r="H37" s="8" t="n">
+        <v>1528</v>
+      </c>
+      <c r="I37" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="J37" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="K37" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="L37" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="M37" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="N37" s="8" t="n">
+        <f aca="false">SUM(B37:M37)</f>
+        <v>9994</v>
+      </c>
+      <c r="O37" s="8" t="n">
+        <f aca="false">IFERROR(N37/12,0)</f>
         <v>832.833333333333</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="B37" s="10" t="n">
-        <f aca="false">SUM(B30:B36)</f>
+    <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="10" t="n">
+        <f aca="false">SUM(B31:B37)</f>
         <v>2426</v>
       </c>
-      <c r="C37" s="10" t="n">
-        <f aca="false">SUM(C30:C36)</f>
+      <c r="C38" s="10" t="n">
+        <f aca="false">SUM(C31:C37)</f>
         <v>2155</v>
       </c>
-      <c r="D37" s="10" t="n">
-        <f aca="false">SUM(D30:D36)</f>
+      <c r="D38" s="10" t="n">
+        <f aca="false">SUM(D31:D37)</f>
         <v>2741</v>
       </c>
-      <c r="E37" s="10" t="n">
-        <f aca="false">SUM(E30:E36)</f>
+      <c r="E38" s="10" t="n">
+        <f aca="false">SUM(E31:E37)</f>
         <v>3181</v>
       </c>
-      <c r="F37" s="11" t="n">
-        <f aca="false">SUM(F30:F36)</f>
+      <c r="F38" s="11" t="n">
+        <f aca="false">SUM(F31:F37)</f>
         <v>2821</v>
       </c>
-      <c r="G37" s="10" t="n">
-        <f aca="false">SUM(G30:G36)</f>
+      <c r="G38" s="10" t="n">
+        <f aca="false">SUM(G31:G37)</f>
         <v>4821</v>
       </c>
-      <c r="H37" s="10" t="n">
-        <f aca="false">SUM(H30:H36)</f>
+      <c r="H38" s="10" t="n">
+        <f aca="false">SUM(H31:H37)</f>
         <v>4782</v>
       </c>
-      <c r="I37" s="10" t="n">
-        <f aca="false">SUM(I30:I36)</f>
+      <c r="I38" s="10" t="n">
+        <f aca="false">SUM(I31:I37)</f>
         <v>3952</v>
       </c>
-      <c r="J37" s="10" t="n">
-        <f aca="false">SUM(J30:J36)</f>
+      <c r="J38" s="10" t="n">
+        <f aca="false">SUM(J31:J37)</f>
         <v>2452</v>
       </c>
-      <c r="K37" s="10" t="n">
-        <f aca="false">SUM(K30:K36)</f>
+      <c r="K38" s="10" t="n">
+        <f aca="false">SUM(K31:K37)</f>
         <v>2452</v>
       </c>
-      <c r="L37" s="10" t="n">
-        <f aca="false">SUM(L30:L36)</f>
+      <c r="L38" s="10" t="n">
+        <f aca="false">SUM(L31:L37)</f>
         <v>2452</v>
       </c>
-      <c r="M37" s="10" t="n">
-        <f aca="false">SUM(M30:M36)</f>
+      <c r="M38" s="10" t="n">
+        <f aca="false">SUM(M31:M37)</f>
         <v>2452</v>
       </c>
-      <c r="N37" s="10" t="n">
-        <f aca="false">SUM(N30:N36)</f>
+      <c r="N38" s="10" t="n">
+        <f aca="false">SUM(N31:N37)</f>
         <v>36687</v>
       </c>
-      <c r="O37" s="10" t="n">
-        <f aca="false">IFERROR(N37/12,0)</f>
+      <c r="O38" s="10" t="n">
+        <f aca="false">IFERROR(N38/12,0)</f>
         <v>3057.25</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="B38" s="12" t="n">
-        <f aca="false">B28+B37</f>
+    <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" s="12" t="n">
+        <f aca="false">B29+B38</f>
         <v>4374</v>
       </c>
-      <c r="C38" s="12" t="n">
-        <f aca="false">C28+C37</f>
+      <c r="C39" s="12" t="n">
+        <f aca="false">C29+C38</f>
         <v>4002</v>
       </c>
-      <c r="D38" s="12" t="n">
-        <f aca="false">D28+D37</f>
+      <c r="D39" s="12" t="n">
+        <f aca="false">D29+D38</f>
         <v>3996</v>
       </c>
-      <c r="E38" s="12" t="n">
-        <f aca="false">E28+E37</f>
+      <c r="E39" s="12" t="n">
+        <f aca="false">E29+E38</f>
         <v>8016</v>
       </c>
-      <c r="F38" s="12" t="n">
-        <f aca="false">F28+F37</f>
+      <c r="F39" s="12" t="n">
+        <f aca="false">F29+F38</f>
         <v>4538</v>
       </c>
-      <c r="G38" s="12" t="n">
-        <f aca="false">G28+G37</f>
+      <c r="G39" s="12" t="n">
+        <f aca="false">G29+G38</f>
         <v>8156</v>
       </c>
-      <c r="H38" s="12" t="n">
-        <f aca="false">H28+H37</f>
+      <c r="H39" s="12" t="n">
+        <f aca="false">H29+H38</f>
         <v>6092</v>
       </c>
-      <c r="I38" s="12" t="n">
-        <f aca="false">I28+I37</f>
+      <c r="I39" s="12" t="n">
+        <f aca="false">I29+I38</f>
         <v>5094</v>
       </c>
-      <c r="J38" s="12" t="n">
-        <f aca="false">J28+J37</f>
+      <c r="J39" s="12" t="n">
+        <f aca="false">J29+J38</f>
         <v>4101</v>
       </c>
-      <c r="K38" s="12" t="n">
-        <f aca="false">K28+K37</f>
+      <c r="K39" s="12" t="n">
+        <f aca="false">K29+K38</f>
         <v>4101</v>
       </c>
-      <c r="L38" s="12" t="n">
-        <f aca="false">L28+L37</f>
+      <c r="L39" s="12" t="n">
+        <f aca="false">L29+L38</f>
         <v>4101</v>
       </c>
-      <c r="M38" s="12" t="n">
-        <f aca="false">M28+M37</f>
+      <c r="M39" s="12" t="n">
+        <f aca="false">M29+M38</f>
         <v>4101</v>
       </c>
-      <c r="N38" s="12" t="n">
-        <f aca="false">N28+N37</f>
+      <c r="N39" s="12" t="n">
+        <f aca="false">N29+N38</f>
         <v>60672</v>
       </c>
-      <c r="O38" s="12" t="n">
-        <f aca="false">IFERROR(N38/12,0)</f>
+      <c r="O39" s="12" t="n">
+        <f aca="false">IFERROR(N39/12,0)</f>
         <v>5056</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="B39" s="13" t="n">
-        <f aca="false">B12-B28-B37</f>
-        <v>222</v>
-      </c>
-      <c r="C39" s="13" t="n">
-        <f aca="false">C12-C28-C37</f>
-        <v>1612</v>
-      </c>
-      <c r="D39" s="13" t="n">
-        <f aca="false">D12-D28-D37</f>
-        <v>1318</v>
-      </c>
-      <c r="E39" s="13" t="n">
-        <f aca="false">E12-E28-E37</f>
-        <v>-3333</v>
-      </c>
-      <c r="F39" s="13" t="n">
-        <f aca="false">F12-F28-F37</f>
-        <v>683</v>
-      </c>
-      <c r="G39" s="13" t="n">
-        <f aca="false">G12-G28-G37</f>
-        <v>-2689</v>
-      </c>
-      <c r="H39" s="13" t="n">
-        <f aca="false">H12-H28-H37</f>
-        <v>-4785</v>
-      </c>
-      <c r="I39" s="13" t="n">
-        <f aca="false">I12-I28-I37</f>
-        <v>277</v>
-      </c>
-      <c r="J39" s="13" t="n">
-        <f aca="false">J12-J28-J37</f>
-        <v>1270</v>
-      </c>
-      <c r="K39" s="13" t="n">
-        <f aca="false">K12-K28-K37</f>
-        <v>1270</v>
-      </c>
-      <c r="L39" s="13" t="n">
-        <f aca="false">L12-L28-L37</f>
-        <v>1270</v>
-      </c>
-      <c r="M39" s="13" t="n">
-        <f aca="false">M12-M28-M37</f>
-        <v>1270</v>
-      </c>
-      <c r="N39" s="13" t="n">
-        <f aca="false">N12-N28-N37</f>
-        <v>-1615</v>
-      </c>
-      <c r="O39" s="13" t="n">
-        <f aca="false">IFERROR(N39/12,0)</f>
-        <v>-134.583333333333</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2446,162 +2421,224 @@
         <v>53</v>
       </c>
       <c r="B40" s="13" t="n">
+        <f aca="false">B13-B29-B38</f>
+        <v>1529</v>
+      </c>
+      <c r="C40" s="13" t="n">
+        <f aca="false">C13-C29-C38</f>
+        <v>5547</v>
+      </c>
+      <c r="D40" s="13" t="n">
+        <f aca="false">D13-D29-D38</f>
+        <v>5159</v>
+      </c>
+      <c r="E40" s="13" t="n">
+        <f aca="false">E13-E29-E38</f>
+        <v>114</v>
+      </c>
+      <c r="F40" s="13" t="n">
+        <f aca="false">F13-F29-F38</f>
+        <v>3343</v>
+      </c>
+      <c r="G40" s="13" t="n">
+        <f aca="false">G13-G29-G38</f>
+        <v>4801</v>
+      </c>
+      <c r="H40" s="13" t="n">
+        <f aca="false">H13-H29-H38</f>
+        <v>-2705</v>
+      </c>
+      <c r="I40" s="13" t="n">
+        <f aca="false">I13-I29-I38</f>
+        <v>277</v>
+      </c>
+      <c r="J40" s="13" t="n">
+        <f aca="false">J13-J29-J38</f>
+        <v>1270</v>
+      </c>
+      <c r="K40" s="13" t="n">
+        <f aca="false">K13-K29-K38</f>
+        <v>1270</v>
+      </c>
+      <c r="L40" s="13" t="n">
+        <f aca="false">L13-L29-L38</f>
+        <v>1270</v>
+      </c>
+      <c r="M40" s="13" t="n">
+        <f aca="false">M13-M29-M38</f>
+        <v>1270</v>
+      </c>
+      <c r="N40" s="13" t="n">
+        <f aca="false">N13-N29-N38</f>
+        <v>465</v>
+      </c>
+      <c r="O40" s="13" t="n">
+        <f aca="false">IFERROR(N40/12,0)</f>
+        <v>38.75</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="13" t="n">
         <v>-29</v>
       </c>
-      <c r="C40" s="13" t="n">
+      <c r="C41" s="13" t="n">
         <v>1540</v>
       </c>
-      <c r="D40" s="13" t="n">
+      <c r="D41" s="13" t="n">
         <v>2525</v>
       </c>
-      <c r="E40" s="13" t="n">
+      <c r="E41" s="13" t="n">
         <v>729</v>
       </c>
-      <c r="F40" s="13" t="n">
+      <c r="F41" s="13" t="n">
         <v>934</v>
       </c>
-      <c r="G40" s="13" t="n">
+      <c r="G41" s="13" t="n">
         <v>4978</v>
       </c>
-      <c r="H40" s="13" t="n">
+      <c r="H41" s="13" t="n">
         <v>2355</v>
       </c>
-      <c r="I40" s="13" t="n">
+      <c r="I41" s="13" t="n">
         <v>2632</v>
       </c>
-      <c r="J40" s="13" t="n">
+      <c r="J41" s="13" t="n">
         <v>3902</v>
       </c>
-      <c r="K40" s="13" t="n">
+      <c r="K41" s="13" t="n">
         <v>5172</v>
       </c>
-      <c r="L40" s="13" t="n">
+      <c r="L41" s="13" t="n">
         <v>6442</v>
       </c>
-      <c r="M40" s="13" t="n">
+      <c r="M41" s="13" t="n">
         <v>7712</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="14"/>
-      <c r="J42" s="14"/>
-      <c r="K42" s="14"/>
-      <c r="L42" s="14"/>
-      <c r="M42" s="14"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="13" t="s">
+    <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="B43" s="13" t="n">
-        <f aca="false">B12-B28</f>
-        <v>2648</v>
-      </c>
-      <c r="C43" s="13" t="n">
-        <f aca="false">C12-C28</f>
-        <v>3767</v>
-      </c>
-      <c r="D43" s="13" t="n">
-        <f aca="false">D12-D28</f>
-        <v>4059</v>
-      </c>
-      <c r="E43" s="13" t="n">
-        <f aca="false">E12-E28</f>
-        <v>-152</v>
-      </c>
-      <c r="F43" s="13" t="n">
-        <f aca="false">F12-F28</f>
-        <v>3504</v>
-      </c>
-      <c r="G43" s="13" t="n">
-        <f aca="false">G12-G28</f>
-        <v>2132</v>
-      </c>
-      <c r="H43" s="13" t="n">
-        <f aca="false">H12-H28</f>
-        <v>-3</v>
-      </c>
-      <c r="I43" s="13" t="n">
-        <f aca="false">I12-I28</f>
-        <v>4229</v>
-      </c>
-      <c r="J43" s="13" t="n">
-        <f aca="false">J12-J28</f>
-        <v>3722</v>
-      </c>
-      <c r="K43" s="13" t="n">
-        <f aca="false">K12-K28</f>
-        <v>3722</v>
-      </c>
-      <c r="L43" s="13" t="n">
-        <f aca="false">L12-L28</f>
-        <v>3722</v>
-      </c>
-      <c r="M43" s="13" t="n">
-        <f aca="false">M12-M28</f>
-        <v>3722</v>
-      </c>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="14"/>
+      <c r="H43" s="14"/>
+      <c r="I43" s="14"/>
+      <c r="J43" s="14"/>
+      <c r="K43" s="14"/>
+      <c r="L43" s="14"/>
+      <c r="M43" s="14"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="13" t="s">
         <v>56</v>
       </c>
       <c r="B44" s="13" t="n">
-        <f aca="false">B39</f>
-        <v>222</v>
+        <f aca="false">B13-B29</f>
+        <v>3955</v>
       </c>
       <c r="C44" s="13" t="n">
-        <f aca="false">C39</f>
-        <v>1612</v>
+        <f aca="false">C13-C29</f>
+        <v>7702</v>
       </c>
       <c r="D44" s="13" t="n">
-        <f aca="false">D39</f>
-        <v>1318</v>
+        <f aca="false">D13-D29</f>
+        <v>7900</v>
       </c>
       <c r="E44" s="13" t="n">
-        <f aca="false">E39</f>
-        <v>-3333</v>
+        <f aca="false">E13-E29</f>
+        <v>3295</v>
       </c>
       <c r="F44" s="13" t="n">
-        <f aca="false">F39</f>
-        <v>683</v>
+        <f aca="false">F13-F29</f>
+        <v>6164</v>
       </c>
       <c r="G44" s="13" t="n">
-        <f aca="false">G39</f>
-        <v>-2689</v>
+        <f aca="false">G13-G29</f>
+        <v>9622</v>
       </c>
       <c r="H44" s="13" t="n">
-        <f aca="false">H39</f>
-        <v>-4785</v>
+        <f aca="false">H13-H29</f>
+        <v>2077</v>
       </c>
       <c r="I44" s="13" t="n">
-        <f aca="false">I39</f>
+        <f aca="false">I13-I29</f>
+        <v>4229</v>
+      </c>
+      <c r="J44" s="13" t="n">
+        <f aca="false">J13-J29</f>
+        <v>3722</v>
+      </c>
+      <c r="K44" s="13" t="n">
+        <f aca="false">K13-K29</f>
+        <v>3722</v>
+      </c>
+      <c r="L44" s="13" t="n">
+        <f aca="false">L13-L29</f>
+        <v>3722</v>
+      </c>
+      <c r="M44" s="13" t="n">
+        <f aca="false">M13-M29</f>
+        <v>3722</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45" s="13" t="n">
+        <f aca="false">B40</f>
+        <v>1529</v>
+      </c>
+      <c r="C45" s="13" t="n">
+        <f aca="false">C40</f>
+        <v>5547</v>
+      </c>
+      <c r="D45" s="13" t="n">
+        <f aca="false">D40</f>
+        <v>5159</v>
+      </c>
+      <c r="E45" s="13" t="n">
+        <f aca="false">E40</f>
+        <v>114</v>
+      </c>
+      <c r="F45" s="13" t="n">
+        <f aca="false">F40</f>
+        <v>3343</v>
+      </c>
+      <c r="G45" s="13" t="n">
+        <f aca="false">G40</f>
+        <v>4801</v>
+      </c>
+      <c r="H45" s="13" t="n">
+        <f aca="false">H40</f>
+        <v>-2705</v>
+      </c>
+      <c r="I45" s="13" t="n">
+        <f aca="false">I40</f>
         <v>277</v>
       </c>
-      <c r="J44" s="13" t="n">
-        <f aca="false">J39</f>
+      <c r="J45" s="13" t="n">
+        <f aca="false">J40</f>
         <v>1270</v>
       </c>
-      <c r="K44" s="13" t="n">
-        <f aca="false">K39</f>
+      <c r="K45" s="13" t="n">
+        <f aca="false">K40</f>
         <v>1270</v>
       </c>
-      <c r="L44" s="13" t="n">
-        <f aca="false">L39</f>
+      <c r="L45" s="13" t="n">
+        <f aca="false">L40</f>
         <v>1270</v>
       </c>
-      <c r="M44" s="13" t="n">
-        <f aca="false">M39</f>
+      <c r="M45" s="13" t="n">
+        <f aca="false">M40</f>
         <v>1270</v>
       </c>
     </row>
@@ -2611,9 +2648,9 @@
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A13:M13"/>
-    <mergeCell ref="A29:M29"/>
-    <mergeCell ref="A42:M42"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A30:M30"/>
+    <mergeCell ref="A43:M43"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Ajout ligne Entrainements Ju, correction Kaki+Autres, zero Julien/Audrey Jan-Juin (donnees reelles releves)
</commit_message>
<xml_diff>
--- a/Tresorerie_2026_Bely_v2.xlsx
+++ b/Tresorerie_2026_Bely_v2.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t xml:space="preserve">TRÉSORERIE 2026 — FAMILLE BELY</t>
   </si>
@@ -88,13 +88,16 @@
     <t xml:space="preserve"> Revenus Revolut joint (Julien &amp; Audrey)</t>
   </si>
   <si>
+    <t xml:space="preserve"> Entraînements Ju (défraiements entraîneur, chèques)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Abely SASU (virement mensuel)</t>
   </si>
   <si>
     <t xml:space="preserve">CAF</t>
   </si>
   <si>
-    <t xml:space="preserve">Kaki (locataire — SCI)</t>
+    <t xml:space="preserve"> Kaki (grand-mère — cadeaux, ex-Lydie Bessière)</t>
   </si>
   <si>
     <t xml:space="preserve"> Autres (remboursements, arbitrage, divers)</t>
@@ -725,7 +728,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="59.85"/>
@@ -863,22 +866,22 @@
         <v>19</v>
       </c>
       <c r="B6" s="8" t="n">
-        <v>2200</v>
+        <v>0</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>2200</v>
+        <v>0</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>2200</v>
+        <v>0</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>2200</v>
+        <v>0</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>3240</v>
+        <v>0</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>2200</v>
+        <v>0</v>
       </c>
       <c r="H6" s="8" t="n">
         <v>1230</v>
@@ -900,11 +903,11 @@
       </c>
       <c r="N6" s="8" t="n">
         <f aca="false">SUM(B6:M6)</f>
-        <v>28970</v>
+        <v>14730</v>
       </c>
       <c r="O6" s="8" t="n">
         <f aca="false">IFERROR(N6/12,0)</f>
-        <v>2414.16666666667</v>
+        <v>1227.5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -912,22 +915,22 @@
         <v>20</v>
       </c>
       <c r="B7" s="8" t="n">
-        <v>920</v>
+        <v>0</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>920</v>
+        <v>0</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>920</v>
+        <v>0</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>920</v>
+        <v>0</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>920</v>
+        <v>0</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>920</v>
+        <v>0</v>
       </c>
       <c r="H7" s="8" t="n">
         <v>850</v>
@@ -949,11 +952,11 @@
       </c>
       <c r="N7" s="8" t="n">
         <f aca="false">SUM(B7:M7)</f>
-        <v>10970</v>
+        <v>5450</v>
       </c>
       <c r="O7" s="8" t="n">
         <f aca="false">IFERROR(N7/12,0)</f>
-        <v>914.166666666667</v>
+        <v>454.166666666667</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -994,48 +997,38 @@
         <v>22</v>
       </c>
       <c r="B9" s="8" t="n">
-        <v>600</v>
+        <v>344</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>600</v>
+        <v>263</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>600</v>
+        <v>1315</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>600</v>
+        <v>1028</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>600</v>
-      </c>
-      <c r="I9" s="8" t="n">
-        <v>600</v>
-      </c>
-      <c r="J9" s="8" t="n">
-        <v>600</v>
-      </c>
-      <c r="K9" s="8" t="n">
-        <v>600</v>
-      </c>
-      <c r="L9" s="8" t="n">
-        <v>600</v>
-      </c>
-      <c r="M9" s="8" t="n">
-        <v>600</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
       <c r="N9" s="8" t="n">
         <f aca="false">SUM(B9:M9)</f>
-        <v>7200</v>
+        <v>2950</v>
       </c>
       <c r="O9" s="8" t="n">
         <f aca="false">IFERROR(N9/12,0)</f>
-        <v>600</v>
+        <v>245.833333333333</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1043,85 +1036,97 @@
         <v>23</v>
       </c>
       <c r="B10" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>152</v>
+        <v>600</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>152</v>
+        <v>600</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>152</v>
+        <v>600</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="L10" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="M10" s="8" t="n">
-        <v>151</v>
+        <v>600</v>
       </c>
       <c r="N10" s="8" t="n">
         <f aca="false">SUM(B10:M10)</f>
-        <v>1815</v>
+        <v>7200</v>
       </c>
       <c r="O10" s="8" t="n">
         <f aca="false">IFERROR(N10/12,0)</f>
-        <v>151.25</v>
+        <v>600</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="8"/>
+      <c r="B11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>152</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>152</v>
+      </c>
       <c r="H11" s="8" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>600</v>
+        <v>151</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>600</v>
+        <v>151</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>600</v>
+        <v>151</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>600</v>
+        <v>151</v>
       </c>
       <c r="M11" s="8" t="n">
-        <v>600</v>
+        <v>151</v>
       </c>
       <c r="N11" s="8" t="n">
         <f aca="false">SUM(B11:M11)</f>
-        <v>3000</v>
+        <v>1815</v>
       </c>
       <c r="O11" s="8" t="n">
         <f aca="false">IFERROR(N11/12,0)</f>
-        <v>250</v>
+        <v>151.25</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1129,224 +1134,224 @@
         <v>25</v>
       </c>
       <c r="B12" s="8" t="n">
-        <v>725</v>
+        <v>0</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>1743</v>
+        <v>350</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>1443</v>
+        <v>200</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>812</v>
+        <v>0</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>309</v>
+        <v>0</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>1595</v>
+        <v>200</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>555</v>
+        <v>0</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="N12" s="8" t="n">
         <f aca="false">SUM(B12:M12)</f>
-        <v>9182</v>
+        <v>3750</v>
       </c>
       <c r="O12" s="8" t="n">
         <f aca="false">IFERROR(N12/12,0)</f>
-        <v>765.166666666667</v>
+        <v>312.5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="10" t="n">
-        <f aca="false">SUM(B6:B12)</f>
-        <v>5903</v>
-      </c>
-      <c r="C13" s="10" t="n">
-        <f aca="false">SUM(C6:C12)</f>
-        <v>9549</v>
-      </c>
-      <c r="D13" s="10" t="n">
-        <f aca="false">SUM(D6:D12)</f>
-        <v>9155</v>
-      </c>
-      <c r="E13" s="10" t="n">
-        <f aca="false">SUM(E6:E12)</f>
-        <v>8130</v>
-      </c>
-      <c r="F13" s="11" t="n">
-        <f aca="false">SUM(F6:F12)</f>
-        <v>7881</v>
-      </c>
-      <c r="G13" s="10" t="n">
-        <f aca="false">SUM(G6:G12)</f>
-        <v>12957</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <f aca="false">SUM(H6:H12)</f>
+      <c r="B13" s="8" t="n">
+        <v>929.82</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>492.29</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>414.48</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>229.63</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>177.89</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>555</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="J13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="K13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="L13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="M13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <f aca="false">SUM(B13:M13)</f>
+        <v>4840.11</v>
+      </c>
+      <c r="O13" s="8" t="n">
+        <f aca="false">IFERROR(N13/12,0)</f>
+        <v>403.3425</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <f aca="false">SUM(B6:B13)</f>
+        <v>3331.82</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <f aca="false">SUM(C6:C13)</f>
+        <v>5340</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <f aca="false">SUM(D6:D13)</f>
+        <v>5284.29</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <f aca="false">SUM(E6:E13)</f>
+        <v>5927.48</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <f aca="false">SUM(F6:F13)</f>
+        <v>3641.63</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <f aca="false">SUM(G6:G13)</f>
+        <v>9647.89</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <f aca="false">SUM(H6:H13)</f>
         <v>3387</v>
       </c>
-      <c r="I13" s="10" t="n">
-        <f aca="false">SUM(I6:I12)</f>
+      <c r="I14" s="10" t="n">
+        <f aca="false">SUM(I6:I13)</f>
         <v>5371</v>
       </c>
-      <c r="J13" s="10" t="n">
-        <f aca="false">SUM(J6:J12)</f>
+      <c r="J14" s="10" t="n">
+        <f aca="false">SUM(J6:J13)</f>
         <v>5371</v>
       </c>
-      <c r="K13" s="10" t="n">
-        <f aca="false">SUM(K6:K12)</f>
+      <c r="K14" s="10" t="n">
+        <f aca="false">SUM(K6:K13)</f>
         <v>5371</v>
       </c>
-      <c r="L13" s="10" t="n">
-        <f aca="false">SUM(L6:L12)</f>
+      <c r="L14" s="10" t="n">
+        <f aca="false">SUM(L6:L13)</f>
         <v>5371</v>
       </c>
-      <c r="M13" s="10" t="n">
-        <f aca="false">SUM(M6:M12)</f>
+      <c r="M14" s="10" t="n">
+        <f aca="false">SUM(M6:M13)</f>
         <v>5371</v>
       </c>
-      <c r="N13" s="10" t="n">
-        <f aca="false">SUM(N6:N12)</f>
-        <v>61137</v>
-      </c>
-      <c r="O13" s="10" t="n">
-        <f aca="false">IFERROR(N13/12,0)</f>
-        <v>5094.75</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
+      <c r="N14" s="10" t="n">
+        <f aca="false">SUM(N6:N13)</f>
+        <v>40735.11</v>
+      </c>
+      <c r="O14" s="10" t="n">
+        <f aca="false">IFERROR(N14/12,0)</f>
+        <v>3394.5925</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="8" t="n">
-        <v>154</v>
-      </c>
-      <c r="C15" s="8" t="n">
-        <v>141</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>141</v>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>142</v>
-      </c>
-      <c r="F15" s="9" t="n">
-        <v>142</v>
-      </c>
-      <c r="G15" s="8" t="n">
-        <v>162</v>
-      </c>
-      <c r="H15" s="8" t="n">
-        <v>142</v>
-      </c>
-      <c r="I15" s="8" t="n">
-        <v>134</v>
-      </c>
-      <c r="J15" s="8" t="n">
-        <v>134</v>
-      </c>
-      <c r="K15" s="8" t="n">
-        <v>134</v>
-      </c>
-      <c r="L15" s="8" t="n">
-        <v>134</v>
-      </c>
-      <c r="M15" s="8" t="n">
-        <v>134</v>
-      </c>
-      <c r="N15" s="8" t="n">
-        <f aca="false">SUM(B15:M15)</f>
-        <v>1694</v>
-      </c>
-      <c r="O15" s="8" t="n">
-        <f aca="false">IFERROR(N15/12,0)</f>
-        <v>141.166666666667</v>
-      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
         <v>29</v>
       </c>
       <c r="B16" s="8" t="n">
-        <v>35</v>
+        <v>154</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>35</v>
+        <v>141</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>35</v>
+        <v>141</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>35</v>
+        <v>142</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>35</v>
+        <v>142</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>35</v>
+        <v>162</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>38</v>
+        <v>142</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>35</v>
+        <v>134</v>
       </c>
       <c r="J16" s="8" t="n">
-        <v>35</v>
+        <v>134</v>
       </c>
       <c r="K16" s="8" t="n">
-        <v>35</v>
+        <v>134</v>
       </c>
       <c r="L16" s="8" t="n">
-        <v>35</v>
+        <v>134</v>
       </c>
       <c r="M16" s="8" t="n">
-        <v>35</v>
+        <v>134</v>
       </c>
       <c r="N16" s="8" t="n">
         <f aca="false">SUM(B16:M16)</f>
-        <v>423</v>
+        <v>1694</v>
       </c>
       <c r="O16" s="8" t="n">
         <f aca="false">IFERROR(N16/12,0)</f>
-        <v>35.25</v>
+        <v>141.166666666667</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1354,46 +1359,48 @@
         <v>30</v>
       </c>
       <c r="B17" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>81</v>
-      </c>
-      <c r="E17" s="8"/>
+        <v>35</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>35</v>
+      </c>
       <c r="F17" s="9" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>81</v>
+        <v>38</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="J17" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="L17" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="M17" s="8" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="N17" s="8" t="n">
         <f aca="false">SUM(B17:M17)</f>
-        <v>891</v>
+        <v>423</v>
       </c>
       <c r="O17" s="8" t="n">
         <f aca="false">IFERROR(N17/12,0)</f>
-        <v>74.25</v>
+        <v>35.25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1401,48 +1408,46 @@
         <v>31</v>
       </c>
       <c r="B18" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="E18" s="8" t="n">
-        <v>60</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="E18" s="8"/>
       <c r="F18" s="9" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="I18" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="L18" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="M18" s="8" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="N18" s="8" t="n">
         <f aca="false">SUM(B18:M18)</f>
-        <v>725</v>
+        <v>891</v>
       </c>
       <c r="O18" s="8" t="n">
         <f aca="false">IFERROR(N18/12,0)</f>
-        <v>60.4166666666667</v>
+        <v>74.25</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1450,142 +1455,142 @@
         <v>32</v>
       </c>
       <c r="B19" s="8" t="n">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="J19" s="8" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="K19" s="8" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="L19" s="8" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="M19" s="8" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="N19" s="8" t="n">
         <f aca="false">SUM(B19:M19)</f>
-        <v>872</v>
+        <v>725</v>
       </c>
       <c r="O19" s="8" t="n">
         <f aca="false">IFERROR(N19/12,0)</f>
-        <v>72.6666666666667</v>
+        <v>60.4166666666667</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="8"/>
+      <c r="B20" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="C20" s="8" t="n">
-        <v>561</v>
-      </c>
-      <c r="D20" s="8"/>
+        <v>64</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>64</v>
+      </c>
       <c r="E20" s="8" t="n">
-        <v>377</v>
+        <v>70</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>173</v>
+        <v>92</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>159</v>
+        <v>86</v>
       </c>
       <c r="H20" s="8" t="n">
-        <v>206</v>
+        <v>92</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="M20" s="8" t="n">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="N20" s="8" t="n">
         <f aca="false">SUM(B20:M20)</f>
-        <v>2651</v>
+        <v>872</v>
       </c>
       <c r="O20" s="8" t="n">
         <f aca="false">IFERROR(N20/12,0)</f>
-        <v>220.916666666667</v>
+        <v>72.6666666666667</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="8" t="n">
-        <v>254</v>
-      </c>
+      <c r="B21" s="8"/>
       <c r="C21" s="8" t="n">
-        <v>254</v>
-      </c>
-      <c r="D21" s="8" t="n">
-        <v>254</v>
-      </c>
+        <v>561</v>
+      </c>
+      <c r="D21" s="8"/>
       <c r="E21" s="8" t="n">
-        <v>254</v>
+        <v>377</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>254</v>
+        <v>173</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>254</v>
+        <v>159</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>254</v>
+        <v>206</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="J21" s="8" t="n">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="K21" s="8" t="n">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="L21" s="8" t="n">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="M21" s="8" t="n">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="N21" s="8" t="n">
         <f aca="false">SUM(B21:M21)</f>
-        <v>3048</v>
+        <v>2651</v>
       </c>
       <c r="O21" s="8" t="n">
         <f aca="false">IFERROR(N21/12,0)</f>
-        <v>254</v>
+        <v>220.916666666667</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1593,48 +1598,48 @@
         <v>35</v>
       </c>
       <c r="B22" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>147</v>
+        <v>254</v>
       </c>
       <c r="N22" s="8" t="n">
         <f aca="false">SUM(B22:M22)</f>
-        <v>1764</v>
+        <v>3048</v>
       </c>
       <c r="O22" s="8" t="n">
         <f aca="false">IFERROR(N22/12,0)</f>
-        <v>147</v>
+        <v>254</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1642,46 +1647,48 @@
         <v>36</v>
       </c>
       <c r="B23" s="8" t="n">
-        <v>164</v>
+        <v>147</v>
       </c>
       <c r="C23" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>283</v>
+        <v>147</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="I23" s="8"/>
+        <v>147</v>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>147</v>
+      </c>
       <c r="J23" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>282</v>
+        <v>147</v>
       </c>
       <c r="N23" s="8" t="n">
         <f aca="false">SUM(B23:M23)</f>
-        <v>2806</v>
+        <v>1764</v>
       </c>
       <c r="O23" s="8" t="n">
         <f aca="false">IFERROR(N23/12,0)</f>
-        <v>233.833333333333</v>
+        <v>147</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1689,46 +1696,46 @@
         <v>37</v>
       </c>
       <c r="B24" s="8" t="n">
-        <v>60</v>
+        <v>164</v>
       </c>
       <c r="C24" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>60</v>
+        <v>283</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="I24" s="8"/>
       <c r="J24" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="L24" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="M24" s="8" t="n">
-        <v>60</v>
+        <v>282</v>
       </c>
       <c r="N24" s="8" t="n">
         <f aca="false">SUM(B24:M24)</f>
-        <v>660</v>
+        <v>2806</v>
       </c>
       <c r="O24" s="8" t="n">
         <f aca="false">IFERROR(N24/12,0)</f>
-        <v>55</v>
+        <v>233.833333333333</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1736,48 +1743,46 @@
         <v>38</v>
       </c>
       <c r="B25" s="8" t="n">
-        <v>219</v>
+        <v>60</v>
       </c>
       <c r="C25" s="8" t="n">
-        <v>157</v>
+        <v>60</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>131</v>
+        <v>60</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>190</v>
+        <v>60</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>123</v>
-      </c>
-      <c r="I25" s="8" t="n">
-        <v>130</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="I25" s="8"/>
       <c r="J25" s="8" t="n">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="K25" s="8" t="n">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="L25" s="8" t="n">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="M25" s="8" t="n">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="N25" s="8" t="n">
         <f aca="false">SUM(B25:M25)</f>
-        <v>1527</v>
+        <v>660</v>
       </c>
       <c r="O25" s="8" t="n">
         <f aca="false">IFERROR(N25/12,0)</f>
-        <v>127.25</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1785,69 +1790,81 @@
         <v>39</v>
       </c>
       <c r="B26" s="8" t="n">
-        <v>700</v>
-      </c>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
+        <v>219</v>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>157</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>131</v>
+      </c>
       <c r="E26" s="8" t="n">
-        <v>1400</v>
-      </c>
-      <c r="F26" s="9"/>
+        <v>14</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>190</v>
+      </c>
       <c r="G26" s="8" t="n">
-        <v>1000</v>
+        <v>43</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="I26" s="8"/>
-      <c r="J26" s="8"/>
-      <c r="K26" s="8"/>
-      <c r="L26" s="8"/>
-      <c r="M26" s="8"/>
+        <v>123</v>
+      </c>
+      <c r="I26" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="J26" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="K26" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="L26" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="M26" s="8" t="n">
+        <v>130</v>
+      </c>
       <c r="N26" s="8" t="n">
         <f aca="false">SUM(B26:M26)</f>
-        <v>3104</v>
+        <v>1527</v>
       </c>
       <c r="O26" s="8" t="n">
         <f aca="false">IFERROR(N26/12,0)</f>
-        <v>258.666666666667</v>
+        <v>127.25</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="8"/>
+      <c r="B27" s="8" t="n">
+        <v>700</v>
+      </c>
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
       <c r="E27" s="8" t="n">
-        <v>494</v>
+        <v>1400</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="8" t="n">
-        <v>466</v>
-      </c>
-      <c r="H27" s="8"/>
+        <v>1000</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>4</v>
+      </c>
       <c r="I27" s="8"/>
-      <c r="J27" s="8" t="n">
-        <v>165</v>
-      </c>
-      <c r="K27" s="8" t="n">
-        <v>165</v>
-      </c>
-      <c r="L27" s="8" t="n">
-        <v>165</v>
-      </c>
-      <c r="M27" s="8" t="n">
-        <v>165</v>
-      </c>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8"/>
       <c r="N27" s="8" t="n">
         <f aca="false">SUM(B27:M27)</f>
-        <v>1620</v>
+        <v>3104</v>
       </c>
       <c r="O27" s="8" t="n">
         <f aca="false">IFERROR(N27/12,0)</f>
-        <v>135</v>
+        <v>258.666666666667</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1858,203 +1875,191 @@
       <c r="C28" s="8"/>
       <c r="D28" s="8"/>
       <c r="E28" s="8" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F28" s="9" t="n">
-        <v>200</v>
-      </c>
+        <v>494</v>
+      </c>
+      <c r="F28" s="9"/>
       <c r="G28" s="8" t="n">
-        <v>500</v>
+        <v>466</v>
       </c>
       <c r="H28" s="8"/>
       <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
-      <c r="K28" s="8"/>
-      <c r="L28" s="8"/>
-      <c r="M28" s="8"/>
+      <c r="J28" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="K28" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="L28" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="M28" s="8" t="n">
+        <v>165</v>
+      </c>
       <c r="N28" s="8" t="n">
         <f aca="false">SUM(B28:M28)</f>
-        <v>2200</v>
+        <v>1620</v>
       </c>
       <c r="O28" s="8" t="n">
         <f aca="false">IFERROR(N28/12,0)</f>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="8" t="n">
+        <f aca="false">SUM(B29:M29)</f>
+        <v>2200</v>
+      </c>
+      <c r="O29" s="8" t="n">
+        <f aca="false">IFERROR(N29/12,0)</f>
         <v>183.333333333333</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="B29" s="10" t="n">
-        <f aca="false">SUM(B15:B28)</f>
+    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="10" t="n">
+        <f aca="false">SUM(B16:B29)</f>
         <v>1948</v>
       </c>
-      <c r="C29" s="10" t="n">
-        <f aca="false">SUM(C15:C28)</f>
+      <c r="C30" s="10" t="n">
+        <f aca="false">SUM(C16:C29)</f>
         <v>1847</v>
       </c>
-      <c r="D29" s="10" t="n">
-        <f aca="false">SUM(D15:D28)</f>
+      <c r="D30" s="10" t="n">
+        <f aca="false">SUM(D16:D29)</f>
         <v>1255</v>
       </c>
-      <c r="E29" s="10" t="n">
-        <f aca="false">SUM(E15:E28)</f>
+      <c r="E30" s="10" t="n">
+        <f aca="false">SUM(E16:E29)</f>
         <v>4835</v>
       </c>
-      <c r="F29" s="11" t="n">
-        <f aca="false">SUM(F15:F28)</f>
+      <c r="F30" s="11" t="n">
+        <f aca="false">SUM(F16:F29)</f>
         <v>1717</v>
       </c>
-      <c r="G29" s="10" t="n">
-        <f aca="false">SUM(G15:G28)</f>
+      <c r="G30" s="10" t="n">
+        <f aca="false">SUM(G16:G29)</f>
         <v>3335</v>
       </c>
-      <c r="H29" s="10" t="n">
-        <f aca="false">SUM(H15:H28)</f>
+      <c r="H30" s="10" t="n">
+        <f aca="false">SUM(H16:H29)</f>
         <v>1310</v>
       </c>
-      <c r="I29" s="10" t="n">
-        <f aca="false">SUM(I15:I28)</f>
+      <c r="I30" s="10" t="n">
+        <f aca="false">SUM(I16:I29)</f>
         <v>1142</v>
       </c>
-      <c r="J29" s="10" t="n">
-        <f aca="false">SUM(J15:J28)</f>
+      <c r="J30" s="10" t="n">
+        <f aca="false">SUM(J16:J29)</f>
         <v>1649</v>
       </c>
-      <c r="K29" s="10" t="n">
-        <f aca="false">SUM(K15:K28)</f>
+      <c r="K30" s="10" t="n">
+        <f aca="false">SUM(K16:K29)</f>
         <v>1649</v>
       </c>
-      <c r="L29" s="10" t="n">
-        <f aca="false">SUM(L15:L28)</f>
+      <c r="L30" s="10" t="n">
+        <f aca="false">SUM(L16:L29)</f>
         <v>1649</v>
       </c>
-      <c r="M29" s="10" t="n">
-        <f aca="false">SUM(M15:M28)</f>
+      <c r="M30" s="10" t="n">
+        <f aca="false">SUM(M16:M29)</f>
         <v>1649</v>
       </c>
-      <c r="N29" s="10" t="n">
-        <f aca="false">SUM(N15:N28)</f>
+      <c r="N30" s="10" t="n">
+        <f aca="false">SUM(N16:N29)</f>
         <v>23985</v>
       </c>
-      <c r="O29" s="10" t="n">
-        <f aca="false">IFERROR(N29/12,0)</f>
+      <c r="O30" s="10" t="n">
+        <f aca="false">IFERROR(N30/12,0)</f>
         <v>1998.75</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
-      <c r="K30" s="6"/>
-      <c r="L30" s="6"/>
-      <c r="M30" s="6"/>
-    </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B31" s="8" t="n">
-        <v>250</v>
-      </c>
-      <c r="C31" s="8" t="n">
-        <v>230</v>
-      </c>
-      <c r="D31" s="8" t="n">
-        <v>260</v>
-      </c>
-      <c r="E31" s="8" t="n">
-        <v>200</v>
-      </c>
-      <c r="F31" s="9" t="n">
-        <v>834</v>
-      </c>
-      <c r="G31" s="8" t="n">
-        <v>569</v>
-      </c>
-      <c r="H31" s="8" t="n">
-        <v>801</v>
-      </c>
-      <c r="I31" s="8" t="n">
-        <v>235</v>
-      </c>
-      <c r="J31" s="8" t="n">
-        <v>235</v>
-      </c>
-      <c r="K31" s="8" t="n">
-        <v>235</v>
-      </c>
-      <c r="L31" s="8" t="n">
-        <v>235</v>
-      </c>
-      <c r="M31" s="8" t="n">
-        <v>235</v>
-      </c>
-      <c r="N31" s="8" t="n">
-        <f aca="false">SUM(B31:M31)</f>
-        <v>4319</v>
-      </c>
-      <c r="O31" s="8" t="n">
-        <f aca="false">IFERROR(N31/12,0)</f>
-        <v>359.916666666667</v>
-      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
         <v>45</v>
       </c>
       <c r="B32" s="8" t="n">
-        <v>450</v>
+        <v>250</v>
       </c>
       <c r="C32" s="8" t="n">
-        <v>380</v>
+        <v>230</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>480</v>
+        <v>260</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>312</v>
+        <v>834</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>347</v>
+        <v>569</v>
       </c>
       <c r="H32" s="8" t="n">
-        <v>579</v>
+        <v>801</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>453</v>
+        <v>235</v>
       </c>
       <c r="J32" s="8" t="n">
-        <v>453</v>
+        <v>235</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>453</v>
+        <v>235</v>
       </c>
       <c r="L32" s="8" t="n">
-        <v>453</v>
+        <v>235</v>
       </c>
       <c r="M32" s="8" t="n">
-        <v>453</v>
+        <v>235</v>
       </c>
       <c r="N32" s="8" t="n">
         <f aca="false">SUM(B32:M32)</f>
-        <v>5313</v>
+        <v>4319</v>
       </c>
       <c r="O32" s="8" t="n">
         <f aca="false">IFERROR(N32/12,0)</f>
-        <v>442.75</v>
+        <v>359.916666666667</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2062,48 +2067,48 @@
         <v>46</v>
       </c>
       <c r="B33" s="8" t="n">
-        <v>850</v>
+        <v>450</v>
       </c>
       <c r="C33" s="8" t="n">
-        <v>520</v>
+        <v>380</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>380</v>
+        <v>480</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>620</v>
+        <v>500</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>632</v>
+        <v>312</v>
       </c>
       <c r="G33" s="8" t="n">
-        <v>546</v>
+        <v>347</v>
       </c>
       <c r="H33" s="8" t="n">
-        <v>876</v>
+        <v>579</v>
       </c>
       <c r="I33" s="8" t="n">
-        <v>593</v>
+        <v>453</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>593</v>
+        <v>453</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>593</v>
+        <v>453</v>
       </c>
       <c r="L33" s="8" t="n">
-        <v>593</v>
+        <v>453</v>
       </c>
       <c r="M33" s="8" t="n">
-        <v>593</v>
+        <v>453</v>
       </c>
       <c r="N33" s="8" t="n">
         <f aca="false">SUM(B33:M33)</f>
-        <v>7389</v>
+        <v>5313</v>
       </c>
       <c r="O33" s="8" t="n">
         <f aca="false">IFERROR(N33/12,0)</f>
-        <v>615.75</v>
+        <v>442.75</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2111,48 +2116,48 @@
         <v>47</v>
       </c>
       <c r="B34" s="8" t="n">
-        <v>200</v>
+        <v>850</v>
       </c>
       <c r="C34" s="8" t="n">
-        <v>80</v>
+        <v>520</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>45</v>
+        <v>380</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>120</v>
+        <v>620</v>
       </c>
       <c r="F34" s="9" t="n">
-        <v>190</v>
+        <v>632</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>66</v>
+        <v>546</v>
       </c>
       <c r="H34" s="8" t="n">
-        <v>44</v>
+        <v>876</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>111</v>
+        <v>593</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>111</v>
+        <v>593</v>
       </c>
       <c r="K34" s="8" t="n">
-        <v>111</v>
+        <v>593</v>
       </c>
       <c r="L34" s="8" t="n">
-        <v>111</v>
+        <v>593</v>
       </c>
       <c r="M34" s="8" t="n">
-        <v>111</v>
+        <v>593</v>
       </c>
       <c r="N34" s="8" t="n">
         <f aca="false">SUM(B34:M34)</f>
-        <v>1300</v>
+        <v>7389</v>
       </c>
       <c r="O34" s="8" t="n">
         <f aca="false">IFERROR(N34/12,0)</f>
-        <v>108.333333333333</v>
+        <v>615.75</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2163,45 +2168,45 @@
         <v>200</v>
       </c>
       <c r="C35" s="8" t="n">
-        <v>280</v>
+        <v>80</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>480</v>
+        <v>45</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>380</v>
+        <v>120</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>432</v>
+        <v>190</v>
       </c>
       <c r="G35" s="8" t="n">
-        <v>251</v>
+        <v>66</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>559</v>
+        <v>44</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>335</v>
+        <v>111</v>
       </c>
       <c r="J35" s="8" t="n">
-        <v>335</v>
+        <v>111</v>
       </c>
       <c r="K35" s="8" t="n">
-        <v>335</v>
+        <v>111</v>
       </c>
       <c r="L35" s="8" t="n">
-        <v>335</v>
+        <v>111</v>
       </c>
       <c r="M35" s="8" t="n">
-        <v>335</v>
+        <v>111</v>
       </c>
       <c r="N35" s="8" t="n">
         <f aca="false">SUM(B35:M35)</f>
-        <v>4257</v>
+        <v>1300</v>
       </c>
       <c r="O35" s="8" t="n">
         <f aca="false">IFERROR(N35/12,0)</f>
-        <v>354.75</v>
+        <v>108.333333333333</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2209,40 +2214,48 @@
         <v>49</v>
       </c>
       <c r="B36" s="8" t="n">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="C36" s="8" t="n">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>245</v>
+        <v>480</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>85</v>
+        <v>380</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>20</v>
+        <v>432</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>1500</v>
+        <v>251</v>
       </c>
       <c r="H36" s="8" t="n">
-        <v>395</v>
+        <v>559</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J36" s="8"/>
-      <c r="K36" s="8"/>
-      <c r="L36" s="8"/>
-      <c r="M36" s="8"/>
+        <v>335</v>
+      </c>
+      <c r="J36" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="K36" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="L36" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="M36" s="8" t="n">
+        <v>335</v>
+      </c>
       <c r="N36" s="8" t="n">
         <f aca="false">SUM(B36:M36)</f>
-        <v>4115</v>
+        <v>4257</v>
       </c>
       <c r="O36" s="8" t="n">
         <f aca="false">IFERROR(N36/12,0)</f>
-        <v>342.916666666667</v>
+        <v>354.75</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2250,231 +2263,211 @@
         <v>50</v>
       </c>
       <c r="B37" s="8" t="n">
-        <v>396</v>
+        <v>80</v>
       </c>
       <c r="C37" s="8" t="n">
-        <v>375</v>
+        <v>290</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>851</v>
+        <v>245</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>1276</v>
+        <v>85</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>401</v>
+        <v>20</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>1542</v>
+        <v>1500</v>
       </c>
       <c r="H37" s="8" t="n">
-        <v>1528</v>
+        <v>395</v>
       </c>
       <c r="I37" s="8" t="n">
-        <v>725</v>
-      </c>
-      <c r="J37" s="8" t="n">
-        <v>725</v>
-      </c>
-      <c r="K37" s="8" t="n">
-        <v>725</v>
-      </c>
-      <c r="L37" s="8" t="n">
-        <v>725</v>
-      </c>
-      <c r="M37" s="8" t="n">
-        <v>725</v>
-      </c>
+        <v>1500</v>
+      </c>
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
+      <c r="M37" s="8"/>
       <c r="N37" s="8" t="n">
         <f aca="false">SUM(B37:M37)</f>
-        <v>9994</v>
+        <v>4115</v>
       </c>
       <c r="O37" s="8" t="n">
         <f aca="false">IFERROR(N37/12,0)</f>
+        <v>342.916666666667</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="8" t="n">
+        <v>396</v>
+      </c>
+      <c r="C38" s="8" t="n">
+        <v>375</v>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>851</v>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>1276</v>
+      </c>
+      <c r="F38" s="9" t="n">
+        <v>401</v>
+      </c>
+      <c r="G38" s="8" t="n">
+        <v>1542</v>
+      </c>
+      <c r="H38" s="8" t="n">
+        <v>1528</v>
+      </c>
+      <c r="I38" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="J38" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="K38" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="L38" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="M38" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="N38" s="8" t="n">
+        <f aca="false">SUM(B38:M38)</f>
+        <v>9994</v>
+      </c>
+      <c r="O38" s="8" t="n">
+        <f aca="false">IFERROR(N38/12,0)</f>
         <v>832.833333333333</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="B38" s="10" t="n">
-        <f aca="false">SUM(B31:B37)</f>
+    <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" s="10" t="n">
+        <f aca="false">SUM(B32:B38)</f>
         <v>2426</v>
       </c>
-      <c r="C38" s="10" t="n">
-        <f aca="false">SUM(C31:C37)</f>
+      <c r="C39" s="10" t="n">
+        <f aca="false">SUM(C32:C38)</f>
         <v>2155</v>
       </c>
-      <c r="D38" s="10" t="n">
-        <f aca="false">SUM(D31:D37)</f>
+      <c r="D39" s="10" t="n">
+        <f aca="false">SUM(D32:D38)</f>
         <v>2741</v>
       </c>
-      <c r="E38" s="10" t="n">
-        <f aca="false">SUM(E31:E37)</f>
+      <c r="E39" s="10" t="n">
+        <f aca="false">SUM(E32:E38)</f>
         <v>3181</v>
       </c>
-      <c r="F38" s="11" t="n">
-        <f aca="false">SUM(F31:F37)</f>
+      <c r="F39" s="11" t="n">
+        <f aca="false">SUM(F32:F38)</f>
         <v>2821</v>
       </c>
-      <c r="G38" s="10" t="n">
-        <f aca="false">SUM(G31:G37)</f>
+      <c r="G39" s="10" t="n">
+        <f aca="false">SUM(G32:G38)</f>
         <v>4821</v>
       </c>
-      <c r="H38" s="10" t="n">
-        <f aca="false">SUM(H31:H37)</f>
+      <c r="H39" s="10" t="n">
+        <f aca="false">SUM(H32:H38)</f>
         <v>4782</v>
       </c>
-      <c r="I38" s="10" t="n">
-        <f aca="false">SUM(I31:I37)</f>
+      <c r="I39" s="10" t="n">
+        <f aca="false">SUM(I32:I38)</f>
         <v>3952</v>
       </c>
-      <c r="J38" s="10" t="n">
-        <f aca="false">SUM(J31:J37)</f>
+      <c r="J39" s="10" t="n">
+        <f aca="false">SUM(J32:J38)</f>
         <v>2452</v>
       </c>
-      <c r="K38" s="10" t="n">
-        <f aca="false">SUM(K31:K37)</f>
+      <c r="K39" s="10" t="n">
+        <f aca="false">SUM(K32:K38)</f>
         <v>2452</v>
       </c>
-      <c r="L38" s="10" t="n">
-        <f aca="false">SUM(L31:L37)</f>
+      <c r="L39" s="10" t="n">
+        <f aca="false">SUM(L32:L38)</f>
         <v>2452</v>
       </c>
-      <c r="M38" s="10" t="n">
-        <f aca="false">SUM(M31:M37)</f>
+      <c r="M39" s="10" t="n">
+        <f aca="false">SUM(M32:M38)</f>
         <v>2452</v>
       </c>
-      <c r="N38" s="10" t="n">
-        <f aca="false">SUM(N31:N37)</f>
+      <c r="N39" s="10" t="n">
+        <f aca="false">SUM(N32:N38)</f>
         <v>36687</v>
       </c>
-      <c r="O38" s="10" t="n">
-        <f aca="false">IFERROR(N38/12,0)</f>
+      <c r="O39" s="10" t="n">
+        <f aca="false">IFERROR(N39/12,0)</f>
         <v>3057.25</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="B39" s="12" t="n">
-        <f aca="false">B29+B38</f>
+    <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="B40" s="12" t="n">
+        <f aca="false">B30+B39</f>
         <v>4374</v>
       </c>
-      <c r="C39" s="12" t="n">
-        <f aca="false">C29+C38</f>
+      <c r="C40" s="12" t="n">
+        <f aca="false">C30+C39</f>
         <v>4002</v>
       </c>
-      <c r="D39" s="12" t="n">
-        <f aca="false">D29+D38</f>
+      <c r="D40" s="12" t="n">
+        <f aca="false">D30+D39</f>
         <v>3996</v>
       </c>
-      <c r="E39" s="12" t="n">
-        <f aca="false">E29+E38</f>
+      <c r="E40" s="12" t="n">
+        <f aca="false">E30+E39</f>
         <v>8016</v>
       </c>
-      <c r="F39" s="12" t="n">
-        <f aca="false">F29+F38</f>
+      <c r="F40" s="12" t="n">
+        <f aca="false">F30+F39</f>
         <v>4538</v>
       </c>
-      <c r="G39" s="12" t="n">
-        <f aca="false">G29+G38</f>
+      <c r="G40" s="12" t="n">
+        <f aca="false">G30+G39</f>
         <v>8156</v>
       </c>
-      <c r="H39" s="12" t="n">
-        <f aca="false">H29+H38</f>
+      <c r="H40" s="12" t="n">
+        <f aca="false">H30+H39</f>
         <v>6092</v>
       </c>
-      <c r="I39" s="12" t="n">
-        <f aca="false">I29+I38</f>
+      <c r="I40" s="12" t="n">
+        <f aca="false">I30+I39</f>
         <v>5094</v>
       </c>
-      <c r="J39" s="12" t="n">
-        <f aca="false">J29+J38</f>
+      <c r="J40" s="12" t="n">
+        <f aca="false">J30+J39</f>
         <v>4101</v>
       </c>
-      <c r="K39" s="12" t="n">
-        <f aca="false">K29+K38</f>
+      <c r="K40" s="12" t="n">
+        <f aca="false">K30+K39</f>
         <v>4101</v>
       </c>
-      <c r="L39" s="12" t="n">
-        <f aca="false">L29+L38</f>
+      <c r="L40" s="12" t="n">
+        <f aca="false">L30+L39</f>
         <v>4101</v>
       </c>
-      <c r="M39" s="12" t="n">
-        <f aca="false">M29+M38</f>
+      <c r="M40" s="12" t="n">
+        <f aca="false">M30+M39</f>
         <v>4101</v>
       </c>
-      <c r="N39" s="12" t="n">
-        <f aca="false">N29+N38</f>
+      <c r="N40" s="12" t="n">
+        <f aca="false">N30+N39</f>
         <v>60672</v>
       </c>
-      <c r="O39" s="12" t="n">
-        <f aca="false">IFERROR(N39/12,0)</f>
+      <c r="O40" s="12" t="n">
+        <f aca="false">IFERROR(N40/12,0)</f>
         <v>5056</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="B40" s="13" t="n">
-        <f aca="false">B13-B29-B38</f>
-        <v>1529</v>
-      </c>
-      <c r="C40" s="13" t="n">
-        <f aca="false">C13-C29-C38</f>
-        <v>5547</v>
-      </c>
-      <c r="D40" s="13" t="n">
-        <f aca="false">D13-D29-D38</f>
-        <v>5159</v>
-      </c>
-      <c r="E40" s="13" t="n">
-        <f aca="false">E13-E29-E38</f>
-        <v>114</v>
-      </c>
-      <c r="F40" s="13" t="n">
-        <f aca="false">F13-F29-F38</f>
-        <v>3343</v>
-      </c>
-      <c r="G40" s="13" t="n">
-        <f aca="false">G13-G29-G38</f>
-        <v>4801</v>
-      </c>
-      <c r="H40" s="13" t="n">
-        <f aca="false">H13-H29-H38</f>
-        <v>-2705</v>
-      </c>
-      <c r="I40" s="13" t="n">
-        <f aca="false">I13-I29-I38</f>
-        <v>277</v>
-      </c>
-      <c r="J40" s="13" t="n">
-        <f aca="false">J13-J29-J38</f>
-        <v>1270</v>
-      </c>
-      <c r="K40" s="13" t="n">
-        <f aca="false">K13-K29-K38</f>
-        <v>1270</v>
-      </c>
-      <c r="L40" s="13" t="n">
-        <f aca="false">L13-L29-L38</f>
-        <v>1270</v>
-      </c>
-      <c r="M40" s="13" t="n">
-        <f aca="false">M13-M29-M38</f>
-        <v>1270</v>
-      </c>
-      <c r="N40" s="13" t="n">
-        <f aca="false">N13-N29-N38</f>
-        <v>465</v>
-      </c>
-      <c r="O40" s="13" t="n">
-        <f aca="false">IFERROR(N40/12,0)</f>
-        <v>38.75</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2482,163 +2475,224 @@
         <v>54</v>
       </c>
       <c r="B41" s="13" t="n">
+        <f aca="false">B14-B30-B39</f>
+        <v>-1042.18</v>
+      </c>
+      <c r="C41" s="13" t="n">
+        <f aca="false">C14-C30-C39</f>
+        <v>1338</v>
+      </c>
+      <c r="D41" s="13" t="n">
+        <f aca="false">D14-D30-D39</f>
+        <v>1288.29</v>
+      </c>
+      <c r="E41" s="13" t="n">
+        <f aca="false">E14-E30-E39</f>
+        <v>-2088.52</v>
+      </c>
+      <c r="F41" s="13" t="n">
+        <f aca="false">F14-F30-F39</f>
+        <v>-896.37</v>
+      </c>
+      <c r="G41" s="13" t="n">
+        <f aca="false">G14-G30-G39</f>
+        <v>1491.89</v>
+      </c>
+      <c r="H41" s="13" t="n">
+        <f aca="false">H14-H30-H39</f>
+        <v>-2705</v>
+      </c>
+      <c r="I41" s="13" t="n">
+        <f aca="false">I14-I30-I39</f>
+        <v>277</v>
+      </c>
+      <c r="J41" s="13" t="n">
+        <f aca="false">J14-J30-J39</f>
+        <v>1270</v>
+      </c>
+      <c r="K41" s="13" t="n">
+        <f aca="false">K14-K30-K39</f>
+        <v>1270</v>
+      </c>
+      <c r="L41" s="13" t="n">
+        <f aca="false">L14-L30-L39</f>
+        <v>1270</v>
+      </c>
+      <c r="M41" s="13" t="n">
+        <f aca="false">M14-M30-M39</f>
+        <v>1270</v>
+      </c>
+      <c r="N41" s="13" t="n">
+        <f aca="false">N14-N30-N39</f>
+        <v>-19936.89</v>
+      </c>
+      <c r="O41" s="13" t="n">
+        <f aca="false">IFERROR(N41/12,0)</f>
+        <v>-1661.4075</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="13" t="n">
         <v>-29</v>
       </c>
-      <c r="C41" s="13" t="n">
+      <c r="C42" s="13" t="n">
         <v>1540</v>
       </c>
-      <c r="D41" s="13" t="n">
+      <c r="D42" s="13" t="n">
         <v>2525</v>
       </c>
-      <c r="E41" s="13" t="n">
+      <c r="E42" s="13" t="n">
         <v>729</v>
       </c>
-      <c r="F41" s="13" t="n">
+      <c r="F42" s="13" t="n">
         <v>934</v>
       </c>
-      <c r="G41" s="13" t="n">
+      <c r="G42" s="13" t="n">
         <v>4978</v>
       </c>
-      <c r="H41" s="13" t="n">
+      <c r="H42" s="13" t="n">
         <v>2355</v>
       </c>
-      <c r="I41" s="13" t="n">
+      <c r="I42" s="13" t="n">
         <v>2632</v>
       </c>
-      <c r="J41" s="13" t="n">
+      <c r="J42" s="13" t="n">
         <v>3902</v>
       </c>
-      <c r="K41" s="13" t="n">
+      <c r="K42" s="13" t="n">
         <v>5172</v>
       </c>
-      <c r="L41" s="13" t="n">
+      <c r="L42" s="13" t="n">
         <v>6442</v>
       </c>
-      <c r="M41" s="13" t="n">
+      <c r="M42" s="13" t="n">
         <v>7712</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="14"/>
-      <c r="J43" s="14"/>
-      <c r="K43" s="14"/>
-      <c r="L43" s="14"/>
-      <c r="M43" s="14"/>
-    </row>
+    <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="13" t="s">
+      <c r="A44" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="B44" s="13" t="n">
-        <f aca="false">B13-B29</f>
-        <v>3955</v>
-      </c>
-      <c r="C44" s="13" t="n">
-        <f aca="false">C13-C29</f>
-        <v>7702</v>
-      </c>
-      <c r="D44" s="13" t="n">
-        <f aca="false">D13-D29</f>
-        <v>7900</v>
-      </c>
-      <c r="E44" s="13" t="n">
-        <f aca="false">E13-E29</f>
-        <v>3295</v>
-      </c>
-      <c r="F44" s="13" t="n">
-        <f aca="false">F13-F29</f>
-        <v>6164</v>
-      </c>
-      <c r="G44" s="13" t="n">
-        <f aca="false">G13-G29</f>
-        <v>9622</v>
-      </c>
-      <c r="H44" s="13" t="n">
-        <f aca="false">H13-H29</f>
-        <v>2077</v>
-      </c>
-      <c r="I44" s="13" t="n">
-        <f aca="false">I13-I29</f>
-        <v>4229</v>
-      </c>
-      <c r="J44" s="13" t="n">
-        <f aca="false">J13-J29</f>
-        <v>3722</v>
-      </c>
-      <c r="K44" s="13" t="n">
-        <f aca="false">K13-K29</f>
-        <v>3722</v>
-      </c>
-      <c r="L44" s="13" t="n">
-        <f aca="false">L13-L29</f>
-        <v>3722</v>
-      </c>
-      <c r="M44" s="13" t="n">
-        <f aca="false">M13-M29</f>
-        <v>3722</v>
-      </c>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="14"/>
+      <c r="H44" s="14"/>
+      <c r="I44" s="14"/>
+      <c r="J44" s="14"/>
+      <c r="K44" s="14"/>
+      <c r="L44" s="14"/>
+      <c r="M44" s="14"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
         <v>57</v>
       </c>
       <c r="B45" s="13" t="n">
-        <f aca="false">B40</f>
-        <v>1529</v>
+        <f aca="false">B14-B30</f>
+        <v>1383.82</v>
       </c>
       <c r="C45" s="13" t="n">
-        <f aca="false">C40</f>
-        <v>5547</v>
+        <f aca="false">C14-C30</f>
+        <v>3493</v>
       </c>
       <c r="D45" s="13" t="n">
-        <f aca="false">D40</f>
-        <v>5159</v>
+        <f aca="false">D14-D30</f>
+        <v>4029.29</v>
       </c>
       <c r="E45" s="13" t="n">
-        <f aca="false">E40</f>
-        <v>114</v>
+        <f aca="false">E14-E30</f>
+        <v>1092.48</v>
       </c>
       <c r="F45" s="13" t="n">
-        <f aca="false">F40</f>
-        <v>3343</v>
+        <f aca="false">F14-F30</f>
+        <v>1924.63</v>
       </c>
       <c r="G45" s="13" t="n">
-        <f aca="false">G40</f>
-        <v>4801</v>
+        <f aca="false">G14-G30</f>
+        <v>6312.89</v>
       </c>
       <c r="H45" s="13" t="n">
-        <f aca="false">H40</f>
+        <f aca="false">H14-H30</f>
+        <v>2077</v>
+      </c>
+      <c r="I45" s="13" t="n">
+        <f aca="false">I14-I30</f>
+        <v>4229</v>
+      </c>
+      <c r="J45" s="13" t="n">
+        <f aca="false">J14-J30</f>
+        <v>3722</v>
+      </c>
+      <c r="K45" s="13" t="n">
+        <f aca="false">K14-K30</f>
+        <v>3722</v>
+      </c>
+      <c r="L45" s="13" t="n">
+        <f aca="false">L14-L30</f>
+        <v>3722</v>
+      </c>
+      <c r="M45" s="13" t="n">
+        <f aca="false">M14-M30</f>
+        <v>3722</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B46" s="13" t="n">
+        <f aca="false">B41</f>
+        <v>-1042.18</v>
+      </c>
+      <c r="C46" s="13" t="n">
+        <f aca="false">C41</f>
+        <v>1338</v>
+      </c>
+      <c r="D46" s="13" t="n">
+        <f aca="false">D41</f>
+        <v>1288.29</v>
+      </c>
+      <c r="E46" s="13" t="n">
+        <f aca="false">E41</f>
+        <v>-2088.52</v>
+      </c>
+      <c r="F46" s="13" t="n">
+        <f aca="false">F41</f>
+        <v>-896.37</v>
+      </c>
+      <c r="G46" s="13" t="n">
+        <f aca="false">G41</f>
+        <v>1491.89</v>
+      </c>
+      <c r="H46" s="13" t="n">
+        <f aca="false">H41</f>
         <v>-2705</v>
       </c>
-      <c r="I45" s="13" t="n">
-        <f aca="false">I40</f>
+      <c r="I46" s="13" t="n">
+        <f aca="false">I41</f>
         <v>277</v>
       </c>
-      <c r="J45" s="13" t="n">
-        <f aca="false">J40</f>
+      <c r="J46" s="13" t="n">
+        <f aca="false">J41</f>
         <v>1270</v>
       </c>
-      <c r="K45" s="13" t="n">
-        <f aca="false">K40</f>
+      <c r="K46" s="13" t="n">
+        <f aca="false">K41</f>
         <v>1270</v>
       </c>
-      <c r="L45" s="13" t="n">
-        <f aca="false">L40</f>
+      <c r="L46" s="13" t="n">
+        <f aca="false">L41</f>
         <v>1270</v>
       </c>
-      <c r="M45" s="13" t="n">
-        <f aca="false">M40</f>
+      <c r="M46" s="13" t="n">
+        <f aca="false">M41</f>
         <v>1270</v>
       </c>
     </row>
@@ -2648,9 +2702,9 @@
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A30:M30"/>
-    <mergeCell ref="A43:M43"/>
+    <mergeCell ref="A15:M15"/>
+    <mergeCell ref="A31:M31"/>
+    <mergeCell ref="A44:M44"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Charges variables recalculees depuis les releves reels Jan-Juin, correction Abely Qonto et Sevigne juin
</commit_message>
<xml_diff>
--- a/Tresorerie_2026_Bely_v2.xlsx
+++ b/Tresorerie_2026_Bely_v2.xlsx
@@ -724,4 +724,2032 @@
     </a:fmtScheme>
   </a:themeElements>
 </a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:P47"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="59.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>1230</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>2700</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>2700</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>2700</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>2700</v>
+      </c>
+      <c r="M6" s="8" t="n">
+        <v>2700</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <f aca="false">SUM(B6:M6)</f>
+        <v>14730</v>
+      </c>
+      <c r="O6" s="8" t="n">
+        <f aca="false">IFERROR(N6/12,0)</f>
+        <v>1227.5</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>850</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>920</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>920</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>920</v>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>920</v>
+      </c>
+      <c r="M7" s="8" t="n">
+        <v>920</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <f aca="false">SUM(B7:M7)</f>
+        <v>5450</v>
+      </c>
+      <c r="O7" s="8" t="n">
+        <f aca="false">IFERROR(N7/12,0)</f>
+        <v>454.166666666667</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>1307</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>3855.29</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>3841</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>3447</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>2041.25</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>7490</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>344</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>263</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>1315</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>1028</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8" t="n">
+        <f aca="false">SUM(B9:M9)</f>
+        <v>2950</v>
+      </c>
+      <c r="O9" s="8" t="n">
+        <f aca="false">IFERROR(N9/12,0)</f>
+        <v>245.833333333333</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>600</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="J10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="L10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="M10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <f aca="false">SUM(B10:M10)</f>
+        <v>7200</v>
+      </c>
+      <c r="O10" s="8" t="n">
+        <f aca="false">IFERROR(N10/12,0)</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>152</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>152</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>152</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="M11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <f aca="false">SUM(B11:M11)</f>
+        <v>1815</v>
+      </c>
+      <c r="O11" s="8" t="n">
+        <f aca="false">IFERROR(N11/12,0)</f>
+        <v>151.25</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>350</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <f aca="false">SUM(B12:M12)</f>
+        <v>3750</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <f aca="false">IFERROR(N12/12,0)</f>
+        <v>312.5</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>929.82</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>24.95</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>414.48</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>308.67</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>293.04</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>555</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="J13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="K13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="L13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="M13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <f aca="false">SUM(B13:M13)</f>
+        <v>4566.96</v>
+      </c>
+      <c r="O13" s="8" t="n">
+        <f aca="false">IFERROR(N13/12,0)</f>
+        <v>380.58</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>482.29</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10" t="n">
+        <f aca="false">SUM(B14:M14)</f>
+        <v>482.29</v>
+      </c>
+      <c r="O14" s="10" t="n">
+        <f aca="false">IFERROR(N14/12,0)</f>
+        <v>40.1908333333333</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="10" t="n">
+        <f aca="false">SUM(B6:B14)</f>
+        <v>3331.82</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <f aca="false">SUM(C6:C14)</f>
+        <v>5260.29</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <f aca="false">SUM(D6:D14)</f>
+        <v>5299.24</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <f aca="false">SUM(E6:E14)</f>
+        <v>5927.48</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <f aca="false">SUM(F6:F14)</f>
+        <v>3101.92</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <f aca="false">SUM(G6:G14)</f>
+        <v>9763.04</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <f aca="false">SUM(H6:H14)</f>
+        <v>3387</v>
+      </c>
+      <c r="I15" s="10" t="n">
+        <f aca="false">SUM(I6:I14)</f>
+        <v>5371</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <f aca="false">SUM(J6:J14)</f>
+        <v>5371</v>
+      </c>
+      <c r="K15" s="10" t="n">
+        <f aca="false">SUM(K6:K14)</f>
+        <v>5371</v>
+      </c>
+      <c r="L15" s="10" t="n">
+        <f aca="false">SUM(L6:L14)</f>
+        <v>5371</v>
+      </c>
+      <c r="M15" s="10" t="n">
+        <f aca="false">SUM(M6:M14)</f>
+        <v>5371</v>
+      </c>
+      <c r="N15" s="10" t="n">
+        <f aca="false">SUM(N6:N14)</f>
+        <v>40944.25</v>
+      </c>
+      <c r="O15" s="10" t="n">
+        <f aca="false">IFERROR(N15/12,0)</f>
+        <v>3412.02083333333</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6"/>
+    </row>
+    <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>154</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>141</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>141</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>142</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>142</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>162</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>142</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>134</v>
+      </c>
+      <c r="J17" s="8" t="n">
+        <v>134</v>
+      </c>
+      <c r="K17" s="8" t="n">
+        <v>134</v>
+      </c>
+      <c r="L17" s="8" t="n">
+        <v>134</v>
+      </c>
+      <c r="M17" s="8" t="n">
+        <v>134</v>
+      </c>
+      <c r="N17" s="8" t="n">
+        <f aca="false">SUM(B17:M17)</f>
+        <v>1694</v>
+      </c>
+      <c r="O17" s="8" t="n">
+        <f aca="false">IFERROR(N17/12,0)</f>
+        <v>141.166666666667</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="I18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="J18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="K18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="L18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="M18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="N18" s="8" t="n">
+        <f aca="false">SUM(B18:M18)</f>
+        <v>423</v>
+      </c>
+      <c r="O18" s="8" t="n">
+        <f aca="false">IFERROR(N18/12,0)</f>
+        <v>35.25</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E19" s="8"/>
+      <c r="F19" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="J19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="K19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="L19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="M19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="N19" s="8" t="n">
+        <f aca="false">SUM(B19:M19)</f>
+        <v>891</v>
+      </c>
+      <c r="O19" s="8" t="n">
+        <f aca="false">IFERROR(N19/12,0)</f>
+        <v>74.25</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="I20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="J20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="K20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="L20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="M20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="N20" s="8" t="n">
+        <f aca="false">SUM(B20:M20)</f>
+        <v>725</v>
+      </c>
+      <c r="O20" s="8" t="n">
+        <f aca="false">IFERROR(N20/12,0)</f>
+        <v>60.4166666666667</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>92</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="J21" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="K21" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="L21" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="M21" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="N21" s="8" t="n">
+        <f aca="false">SUM(B21:M21)</f>
+        <v>872</v>
+      </c>
+      <c r="O21" s="8" t="n">
+        <f aca="false">IFERROR(N21/12,0)</f>
+        <v>72.6666666666667</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8" t="n">
+        <v>561</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8" t="n">
+        <v>377</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>173</v>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>159</v>
+      </c>
+      <c r="H22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="I22" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="J22" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="K22" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="L22" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <f aca="false">SUM(B22:M22)</f>
+        <v>2651</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <f aca="false">IFERROR(N22/12,0)</f>
+        <v>220.916666666667</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>254</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <f aca="false">SUM(B23:M23)</f>
+        <v>3048</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <f aca="false">IFERROR(N23/12,0)</f>
+        <v>254</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="H24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="I24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="J24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="K24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="L24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="M24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="N24" s="8" t="n">
+        <f aca="false">SUM(B24:M24)</f>
+        <v>1764</v>
+      </c>
+      <c r="O24" s="8" t="n">
+        <f aca="false">IFERROR(N24/12,0)</f>
+        <v>147</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="8" t="n">
+        <v>164</v>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>283</v>
+      </c>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="K25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="L25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="M25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="N25" s="8" t="n">
+        <f aca="false">SUM(B25:M25)</f>
+        <v>2524</v>
+      </c>
+      <c r="O25" s="8" t="n">
+        <f aca="false">IFERROR(N25/12,0)</f>
+        <v>210.333333333333</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="K26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="L26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="M26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="N26" s="8" t="n">
+        <f aca="false">SUM(B26:M26)</f>
+        <v>660</v>
+      </c>
+      <c r="O26" s="8" t="n">
+        <f aca="false">IFERROR(N26/12,0)</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="8" t="n">
+        <v>219</v>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>157</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>123</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="J27" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="K27" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="L27" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="M27" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="N27" s="8" t="n">
+        <f aca="false">SUM(B27:M27)</f>
+        <v>1527</v>
+      </c>
+      <c r="O27" s="8" t="n">
+        <f aca="false">IFERROR(N27/12,0)</f>
+        <v>127.25</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F28" s="9"/>
+      <c r="G28" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H28" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8" t="n">
+        <f aca="false">SUM(B28:M28)</f>
+        <v>3104</v>
+      </c>
+      <c r="O28" s="8" t="n">
+        <f aca="false">IFERROR(N28/12,0)</f>
+        <v>258.666666666667</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8" t="n">
+        <v>494</v>
+      </c>
+      <c r="F29" s="9"/>
+      <c r="G29" s="8" t="n">
+        <v>466</v>
+      </c>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="K29" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="L29" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="M29" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="N29" s="8" t="n">
+        <f aca="false">SUM(B29:M29)</f>
+        <v>1620</v>
+      </c>
+      <c r="O29" s="8" t="n">
+        <f aca="false">IFERROR(N29/12,0)</f>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="G30" s="8"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="8"/>
+      <c r="M30" s="8"/>
+      <c r="N30" s="8" t="n">
+        <f aca="false">SUM(B30:M30)</f>
+        <v>1700</v>
+      </c>
+      <c r="O30" s="8" t="n">
+        <f aca="false">IFERROR(N30/12,0)</f>
+        <v>141.666666666667</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" s="10" t="n">
+        <f aca="false">SUM(B17:B30)</f>
+        <v>1948</v>
+      </c>
+      <c r="C31" s="10" t="n">
+        <f aca="false">SUM(C17:C30)</f>
+        <v>1847</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <f aca="false">SUM(D17:D30)</f>
+        <v>1255</v>
+      </c>
+      <c r="E31" s="10" t="n">
+        <f aca="false">SUM(E17:E30)</f>
+        <v>4835</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <f aca="false">SUM(F17:F30)</f>
+        <v>1717</v>
+      </c>
+      <c r="G31" s="10" t="n">
+        <f aca="false">SUM(G17:G30)</f>
+        <v>2553</v>
+      </c>
+      <c r="H31" s="10" t="n">
+        <f aca="false">SUM(H17:H30)</f>
+        <v>1310</v>
+      </c>
+      <c r="I31" s="10" t="n">
+        <f aca="false">SUM(I17:I30)</f>
+        <v>1142</v>
+      </c>
+      <c r="J31" s="10" t="n">
+        <f aca="false">SUM(J17:J30)</f>
+        <v>1649</v>
+      </c>
+      <c r="K31" s="10" t="n">
+        <f aca="false">SUM(K17:K30)</f>
+        <v>1649</v>
+      </c>
+      <c r="L31" s="10" t="n">
+        <f aca="false">SUM(L17:L30)</f>
+        <v>1649</v>
+      </c>
+      <c r="M31" s="10" t="n">
+        <f aca="false">SUM(M17:M30)</f>
+        <v>1649</v>
+      </c>
+      <c r="N31" s="10" t="n">
+        <f aca="false">SUM(N17:N30)</f>
+        <v>23203</v>
+      </c>
+      <c r="O31" s="10" t="n">
+        <f aca="false">IFERROR(N31/12,0)</f>
+        <v>1933.58333333333</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="6"/>
+      <c r="K32" s="6"/>
+      <c r="L32" s="6"/>
+      <c r="M32" s="6"/>
+    </row>
+    <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>227.99</v>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>124.82</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>292.02</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>545.19</v>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>294.9</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>253.4</v>
+      </c>
+      <c r="H33" s="8" t="n">
+        <v>801</v>
+      </c>
+      <c r="I33" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="J33" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="K33" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="L33" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="M33" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="N33" s="8" t="n">
+        <f aca="false">SUM(B33:M33)</f>
+        <v>3714.32</v>
+      </c>
+      <c r="O33" s="8" t="n">
+        <f aca="false">IFERROR(N33/12,0)</f>
+        <v>309.526666666667</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" s="8" t="n">
+        <v>221.2</v>
+      </c>
+      <c r="C34" s="8" t="n">
+        <v>171.55</v>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>383.95</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>229.3</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>306.85</v>
+      </c>
+      <c r="G34" s="8" t="n">
+        <v>336.47</v>
+      </c>
+      <c r="H34" s="8" t="n">
+        <v>579</v>
+      </c>
+      <c r="I34" s="8" t="n">
+        <v>453</v>
+      </c>
+      <c r="J34" s="8" t="n">
+        <v>453</v>
+      </c>
+      <c r="K34" s="8" t="n">
+        <v>453</v>
+      </c>
+      <c r="L34" s="8" t="n">
+        <v>453</v>
+      </c>
+      <c r="M34" s="8" t="n">
+        <v>453</v>
+      </c>
+      <c r="N34" s="8" t="n">
+        <f aca="false">SUM(B34:M34)</f>
+        <v>4493.32</v>
+      </c>
+      <c r="O34" s="8" t="n">
+        <f aca="false">IFERROR(N34/12,0)</f>
+        <v>374.443333333333</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" s="8" t="n">
+        <v>874.02</v>
+      </c>
+      <c r="C35" s="8" t="n">
+        <v>283.98</v>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>224.88</v>
+      </c>
+      <c r="E35" s="8" t="n">
+        <v>235.2</v>
+      </c>
+      <c r="F35" s="9" t="n">
+        <v>543.78</v>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>744.23</v>
+      </c>
+      <c r="H35" s="8" t="n">
+        <v>876</v>
+      </c>
+      <c r="I35" s="8" t="n">
+        <v>593</v>
+      </c>
+      <c r="J35" s="8" t="n">
+        <v>593</v>
+      </c>
+      <c r="K35" s="8" t="n">
+        <v>593</v>
+      </c>
+      <c r="L35" s="8" t="n">
+        <v>593</v>
+      </c>
+      <c r="M35" s="8" t="n">
+        <v>593</v>
+      </c>
+      <c r="N35" s="8" t="n">
+        <f aca="false">SUM(B35:M35)</f>
+        <v>6747.09</v>
+      </c>
+      <c r="O35" s="8" t="n">
+        <f aca="false">IFERROR(N35/12,0)</f>
+        <v>562.2575</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" s="8" t="n">
+        <v>188.29</v>
+      </c>
+      <c r="C36" s="8" t="n">
+        <v>13.92</v>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>160</v>
+      </c>
+      <c r="F36" s="9" t="n">
+        <v>190.08</v>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="H36" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="I36" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="J36" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="K36" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="L36" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="M36" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="N36" s="8" t="n">
+        <f aca="false">SUM(B36:M36)</f>
+        <v>1189.19</v>
+      </c>
+      <c r="O36" s="8" t="n">
+        <f aca="false">IFERROR(N36/12,0)</f>
+        <v>99.0991666666667</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" s="8" t="n">
+        <v>90.99</v>
+      </c>
+      <c r="C37" s="8" t="n">
+        <v>268.78</v>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>444.59</v>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>203.99</v>
+      </c>
+      <c r="F37" s="9" t="n">
+        <v>375.39</v>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>86.29</v>
+      </c>
+      <c r="H37" s="8" t="n">
+        <v>559</v>
+      </c>
+      <c r="I37" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="J37" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="K37" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="L37" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="M37" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="N37" s="8" t="n">
+        <f aca="false">SUM(B37:M37)</f>
+        <v>3704.03</v>
+      </c>
+      <c r="O37" s="8" t="n">
+        <f aca="false">IFERROR(N37/12,0)</f>
+        <v>308.669166666667</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="8" t="n">
+        <v>166.99</v>
+      </c>
+      <c r="C38" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>334.34</v>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>165.09</v>
+      </c>
+      <c r="F38" s="9" t="n">
+        <v>164.6</v>
+      </c>
+      <c r="G38" s="8" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="H38" s="8" t="n">
+        <v>395</v>
+      </c>
+      <c r="I38" s="8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8"/>
+      <c r="N38" s="8" t="n">
+        <f aca="false">SUM(B38:M38)</f>
+        <v>2868.82</v>
+      </c>
+      <c r="O38" s="8" t="n">
+        <f aca="false">IFERROR(N38/12,0)</f>
+        <v>239.068333333333</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" s="8" t="n">
+        <v>552.8</v>
+      </c>
+      <c r="C39" s="8" t="n">
+        <v>1131.64</v>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>1387.05</v>
+      </c>
+      <c r="E39" s="8" t="n">
+        <v>1517.17</v>
+      </c>
+      <c r="F39" s="9" t="n">
+        <v>907.82</v>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>1830.11</v>
+      </c>
+      <c r="H39" s="8" t="n">
+        <v>1528</v>
+      </c>
+      <c r="I39" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="J39" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="K39" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="L39" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="M39" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="N39" s="8" t="n">
+        <f aca="false">SUM(B39:M39)</f>
+        <v>12479.59</v>
+      </c>
+      <c r="O39" s="8" t="n">
+        <f aca="false">IFERROR(N39/12,0)</f>
+        <v>1039.96583333333</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B40" s="10" t="n">
+        <f aca="false">SUM(B33:B39)</f>
+        <v>2322.28</v>
+      </c>
+      <c r="C40" s="10" t="n">
+        <f aca="false">SUM(C33:C39)</f>
+        <v>2124.69</v>
+      </c>
+      <c r="D40" s="10" t="n">
+        <f aca="false">SUM(D33:D39)</f>
+        <v>3066.83</v>
+      </c>
+      <c r="E40" s="10" t="n">
+        <f aca="false">SUM(E33:E39)</f>
+        <v>3055.94</v>
+      </c>
+      <c r="F40" s="11" t="n">
+        <f aca="false">SUM(F33:F39)</f>
+        <v>2783.42</v>
+      </c>
+      <c r="G40" s="10" t="n">
+        <f aca="false">SUM(G33:G39)</f>
+        <v>3301.2</v>
+      </c>
+      <c r="H40" s="10" t="n">
+        <f aca="false">SUM(H33:H39)</f>
+        <v>4782</v>
+      </c>
+      <c r="I40" s="10" t="n">
+        <f aca="false">SUM(I33:I39)</f>
+        <v>3952</v>
+      </c>
+      <c r="J40" s="10" t="n">
+        <f aca="false">SUM(J33:J39)</f>
+        <v>2452</v>
+      </c>
+      <c r="K40" s="10" t="n">
+        <f aca="false">SUM(K33:K39)</f>
+        <v>2452</v>
+      </c>
+      <c r="L40" s="10" t="n">
+        <f aca="false">SUM(L33:L39)</f>
+        <v>2452</v>
+      </c>
+      <c r="M40" s="10" t="n">
+        <f aca="false">SUM(M33:M39)</f>
+        <v>2452</v>
+      </c>
+      <c r="N40" s="10" t="n">
+        <f aca="false">SUM(N33:N39)</f>
+        <v>35196.36</v>
+      </c>
+      <c r="O40" s="10" t="n">
+        <f aca="false">IFERROR(N40/12,0)</f>
+        <v>2933.03</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="12" t="n">
+        <f aca="false">B31+B40</f>
+        <v>4270.28</v>
+      </c>
+      <c r="C41" s="12" t="n">
+        <f aca="false">C31+C40</f>
+        <v>3971.69</v>
+      </c>
+      <c r="D41" s="12" t="n">
+        <f aca="false">D31+D40</f>
+        <v>4321.83</v>
+      </c>
+      <c r="E41" s="12" t="n">
+        <f aca="false">E31+E40</f>
+        <v>7890.94</v>
+      </c>
+      <c r="F41" s="12" t="n">
+        <f aca="false">F31+F40</f>
+        <v>4500.42</v>
+      </c>
+      <c r="G41" s="12" t="n">
+        <f aca="false">G31+G40</f>
+        <v>5854.2</v>
+      </c>
+      <c r="H41" s="12" t="n">
+        <f aca="false">H31+H40</f>
+        <v>6092</v>
+      </c>
+      <c r="I41" s="12" t="n">
+        <f aca="false">I31+I40</f>
+        <v>5094</v>
+      </c>
+      <c r="J41" s="12" t="n">
+        <f aca="false">J31+J40</f>
+        <v>4101</v>
+      </c>
+      <c r="K41" s="12" t="n">
+        <f aca="false">K31+K40</f>
+        <v>4101</v>
+      </c>
+      <c r="L41" s="12" t="n">
+        <f aca="false">L31+L40</f>
+        <v>4101</v>
+      </c>
+      <c r="M41" s="12" t="n">
+        <f aca="false">M31+M40</f>
+        <v>4101</v>
+      </c>
+      <c r="N41" s="12" t="n">
+        <f aca="false">N31+N40</f>
+        <v>58399.36</v>
+      </c>
+      <c r="O41" s="12" t="n">
+        <f aca="false">IFERROR(N41/12,0)</f>
+        <v>4866.61333333333</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="13" t="n">
+        <f aca="false">B15-B31-B40</f>
+        <v>-938.46</v>
+      </c>
+      <c r="C42" s="13" t="n">
+        <f aca="false">C15-C31-C40</f>
+        <v>1288.6</v>
+      </c>
+      <c r="D42" s="13" t="n">
+        <f aca="false">D15-D31-D40</f>
+        <v>977.41</v>
+      </c>
+      <c r="E42" s="13" t="n">
+        <f aca="false">E15-E31-E40</f>
+        <v>-1963.46</v>
+      </c>
+      <c r="F42" s="13" t="n">
+        <f aca="false">F15-F31-F40</f>
+        <v>-1398.5</v>
+      </c>
+      <c r="G42" s="13" t="n">
+        <f aca="false">G15-G31-G40</f>
+        <v>3908.84</v>
+      </c>
+      <c r="H42" s="13" t="n">
+        <f aca="false">H15-H31-H40</f>
+        <v>-2705</v>
+      </c>
+      <c r="I42" s="13" t="n">
+        <f aca="false">I15-I31-I40</f>
+        <v>277</v>
+      </c>
+      <c r="J42" s="13" t="n">
+        <f aca="false">J15-J31-J40</f>
+        <v>1270</v>
+      </c>
+      <c r="K42" s="13" t="n">
+        <f aca="false">K15-K31-K40</f>
+        <v>1270</v>
+      </c>
+      <c r="L42" s="13" t="n">
+        <f aca="false">L15-L31-L40</f>
+        <v>1270</v>
+      </c>
+      <c r="M42" s="13" t="n">
+        <f aca="false">M15-M31-M40</f>
+        <v>1270</v>
+      </c>
+      <c r="N42" s="13" t="n">
+        <f aca="false">N15-N31-N40</f>
+        <v>-17455.11</v>
+      </c>
+      <c r="O42" s="13" t="n">
+        <f aca="false">IFERROR(N42/12,0)</f>
+        <v>-1454.5925</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B43" s="13" t="n">
+        <v>-29</v>
+      </c>
+      <c r="C43" s="13" t="n">
+        <v>1540</v>
+      </c>
+      <c r="D43" s="13" t="n">
+        <v>2525</v>
+      </c>
+      <c r="E43" s="13" t="n">
+        <v>729</v>
+      </c>
+      <c r="F43" s="13" t="n">
+        <v>934</v>
+      </c>
+      <c r="G43" s="13" t="n">
+        <v>4978</v>
+      </c>
+      <c r="H43" s="13" t="n">
+        <v>2355</v>
+      </c>
+      <c r="I43" s="13" t="n">
+        <v>2632</v>
+      </c>
+      <c r="J43" s="13" t="n">
+        <v>3902</v>
+      </c>
+      <c r="K43" s="13" t="n">
+        <v>5172</v>
+      </c>
+      <c r="L43" s="13" t="n">
+        <v>6442</v>
+      </c>
+      <c r="M43" s="13" t="n">
+        <v>7712</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="14"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="14"/>
+      <c r="J45" s="14"/>
+      <c r="K45" s="14"/>
+      <c r="L45" s="14"/>
+      <c r="M45" s="14"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B46" s="13" t="n">
+        <f aca="false">B15-B31</f>
+        <v>1383.82</v>
+      </c>
+      <c r="C46" s="13" t="n">
+        <f aca="false">C15-C31</f>
+        <v>3413.29</v>
+      </c>
+      <c r="D46" s="13" t="n">
+        <f aca="false">D15-D31</f>
+        <v>4044.24</v>
+      </c>
+      <c r="E46" s="13" t="n">
+        <f aca="false">E15-E31</f>
+        <v>1092.48</v>
+      </c>
+      <c r="F46" s="13" t="n">
+        <f aca="false">F15-F31</f>
+        <v>1384.92</v>
+      </c>
+      <c r="G46" s="13" t="n">
+        <f aca="false">G15-G31</f>
+        <v>7210.04</v>
+      </c>
+      <c r="H46" s="13" t="n">
+        <f aca="false">H15-H31</f>
+        <v>2077</v>
+      </c>
+      <c r="I46" s="13" t="n">
+        <f aca="false">I15-I31</f>
+        <v>4229</v>
+      </c>
+      <c r="J46" s="13" t="n">
+        <f aca="false">J15-J31</f>
+        <v>3722</v>
+      </c>
+      <c r="K46" s="13" t="n">
+        <f aca="false">K15-K31</f>
+        <v>3722</v>
+      </c>
+      <c r="L46" s="13" t="n">
+        <f aca="false">L15-L31</f>
+        <v>3722</v>
+      </c>
+      <c r="M46" s="13" t="n">
+        <f aca="false">M15-M31</f>
+        <v>3722</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B47" s="13" t="n">
+        <f aca="false">B42</f>
+        <v>-938.46</v>
+      </c>
+      <c r="C47" s="13" t="n">
+        <f aca="false">C42</f>
+        <v>1288.6</v>
+      </c>
+      <c r="D47" s="13" t="n">
+        <f aca="false">D42</f>
+        <v>977.41</v>
+      </c>
+      <c r="E47" s="13" t="n">
+        <f aca="false">E42</f>
+        <v>-1963.46</v>
+      </c>
+      <c r="F47" s="13" t="n">
+        <f aca="false">F42</f>
+        <v>-1398.5</v>
+      </c>
+      <c r="G47" s="13" t="n">
+        <f aca="false">G42</f>
+        <v>3908.84</v>
+      </c>
+      <c r="H47" s="13" t="n">
+        <f aca="false">H42</f>
+        <v>-2705</v>
+      </c>
+      <c r="I47" s="13" t="n">
+        <f aca="false">I42</f>
+        <v>277</v>
+      </c>
+      <c r="J47" s="13" t="n">
+        <f aca="false">J42</f>
+        <v>1270</v>
+      </c>
+      <c r="K47" s="13" t="n">
+        <f aca="false">K42</f>
+        <v>1270</v>
+      </c>
+      <c r="L47" s="13" t="n">
+        <f aca="false">L42</f>
+        <v>1270</v>
+      </c>
+      <c r="M47" s="13" t="n">
+        <f aca="false">M42</f>
+        <v>1270</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A16:M16"/>
+    <mergeCell ref="A32:M32"/>
+    <mergeCell ref="A45:M45"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Reclassement voyages (Desirs2reves, Breitenstein, Dojcilovic, Anais C)
</commit_message>
<xml_diff>
--- a/Tresorerie_2026_Bely_v2.xlsx
+++ b/Tresorerie_2026_Bely_v2.xlsx
@@ -2154,7 +2154,7 @@
         <v>48</v>
       </c>
       <c r="B35" s="8" t="n">
-        <v>874.02</v>
+        <v>294.02</v>
       </c>
       <c r="C35" s="8" t="n">
         <v>283.98</v>
@@ -2191,11 +2191,11 @@
       </c>
       <c r="N35" s="8" t="n">
         <f aca="false">SUM(B35:M35)</f>
-        <v>6747.09</v>
+        <v>6167.09</v>
       </c>
       <c r="O35" s="8" t="n">
         <f aca="false">IFERROR(N35/12,0)</f>
-        <v>562.2575</v>
+        <v>513.924166666667</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2301,22 +2301,22 @@
         <v>51</v>
       </c>
       <c r="B38" s="8" t="n">
-        <v>166.99</v>
+        <v>746.99</v>
       </c>
       <c r="C38" s="8" t="n">
         <v>130</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>334.34</v>
+        <v>780.34</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>165.09</v>
+        <v>841.59</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>164.6</v>
+        <v>275.93</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>12.8</v>
+        <v>529.05</v>
       </c>
       <c r="H38" s="8" t="n">
         <v>395</v>
@@ -2330,11 +2330,11 @@
       <c r="M38" s="8"/>
       <c r="N38" s="8" t="n">
         <f aca="false">SUM(B38:M38)</f>
-        <v>2868.82</v>
+        <v>5198.9</v>
       </c>
       <c r="O38" s="8" t="n">
         <f aca="false">IFERROR(N38/12,0)</f>
-        <v>239.068333333333</v>
+        <v>433.241666666667</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2348,16 +2348,16 @@
         <v>1131.64</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>1387.05</v>
+        <v>941.05</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>1517.17</v>
+        <v>840.67</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>907.82</v>
+        <v>796.49</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>1830.11</v>
+        <v>1313.86</v>
       </c>
       <c r="H39" s="8" t="n">
         <v>1528</v>
@@ -2379,11 +2379,11 @@
       </c>
       <c r="N39" s="8" t="n">
         <f aca="false">SUM(B39:M39)</f>
-        <v>12479.59</v>
+        <v>10729.51</v>
       </c>
       <c r="O39" s="8" t="n">
         <f aca="false">IFERROR(N39/12,0)</f>
-        <v>1039.96583333333</v>
+        <v>894.125833333333</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
AXA scinde habitation/auto, SCI Gambetta->Logement, Voyages en ligne dediee
</commit_message>
<xml_diff>
--- a/Tresorerie_2026_Bely_v2.xlsx
+++ b/Tresorerie_2026_Bely_v2.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="97">
   <si>
     <t xml:space="preserve">TRÉSORERIE 2026 — FAMILLE BELY</t>
   </si>
@@ -254,6 +254,9 @@
     <t xml:space="preserve">Loisirs et Sorties</t>
   </si>
   <si>
+    <t xml:space="preserve">   ↳ Voyages (ss-cat. de Loisirs et Sorties)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Alimentation et Restos</t>
   </si>
   <si>
@@ -296,10 +299,19 @@
     <t xml:space="preserve">TOTAL TOUTES CATÉGORIES</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes / points à confirmer avec Julien :</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- AXA (assurances mutuelle + auto) est mis intégralement en "Auto et transports" faute de ventilation détaillée par contrat — à corriger si tu peux séparer mutuelle santé / assurance auto.</t>
+    <t xml:space="preserve">Notes / points tranchés avec Julien (19/08/2026) :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- AXA scindé selon les montants donnés par Julien : 86,70€/mois assurance habitation (-&gt; Logement), 59,80€/mois assurance auto (-&gt; Auto et transports), répartis au prorata sur le montant réel prélevé chaque mois.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Virements SCI Gambetta reclassés de "Dépenses pro" vers "Logement" (c'est un bien immobilier).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Abely QONTO reste en "Dépenses pro" (confirmé).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Voyages sorti de "Loisirs et Sorties" en ligne dédiée, comme sous-catégorie dans Bankin' (le total des deux lignes = ce qui était avant dans Loisirs et Sorties).</t>
   </si>
 </sst>
 </file>
@@ -311,7 +323,7 @@
     <numFmt numFmtId="165" formatCode="#,##0&quot; €&quot;;[RED]\(#,##0&quot; €)&quot;;\-"/>
     <numFmt numFmtId="166" formatCode="#,##0.00&quot; €&quot;"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -433,6 +445,31 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <name val="Cambria"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color rgb="FF595959"/>
+      <name val="Cambria"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color rgb="FF595959"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <i val="true"/>
+      <sz val="11"/>
+      <color rgb="FF595959"/>
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
@@ -581,7 +618,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -646,11 +683,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -658,27 +695,51 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -739,7 +800,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF595959"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF1F4E79"/>
       <rgbColor rgb="FF339966"/>
@@ -929,17 +990,2045 @@
 </a:theme>
 </file>
 
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:P47"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="59.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>1230</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>2700</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>2700</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>2700</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>2700</v>
+      </c>
+      <c r="M6" s="8" t="n">
+        <v>2700</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <f aca="false">SUM(B6:M6)</f>
+        <v>14730</v>
+      </c>
+      <c r="O6" s="8" t="n">
+        <f aca="false">IFERROR(N6/12,0)</f>
+        <v>1227.5</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>850</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>920</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>920</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>920</v>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>920</v>
+      </c>
+      <c r="M7" s="8" t="n">
+        <v>920</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <f aca="false">SUM(B7:M7)</f>
+        <v>5450</v>
+      </c>
+      <c r="O7" s="8" t="n">
+        <f aca="false">IFERROR(N7/12,0)</f>
+        <v>454.166666666667</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>1307</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>3855.29</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>3841</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>3447</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>2041.25</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>7490</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>344</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>263</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>1315</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>1028</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8" t="n">
+        <f aca="false">SUM(B9:M9)</f>
+        <v>2950</v>
+      </c>
+      <c r="O9" s="8" t="n">
+        <f aca="false">IFERROR(N9/12,0)</f>
+        <v>245.833333333333</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>600</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="J10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="L10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="M10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <f aca="false">SUM(B10:M10)</f>
+        <v>7200</v>
+      </c>
+      <c r="O10" s="8" t="n">
+        <f aca="false">IFERROR(N10/12,0)</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>152</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>152</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>152</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="M11" s="8" t="n">
+        <v>151</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <f aca="false">SUM(B11:M11)</f>
+        <v>1815</v>
+      </c>
+      <c r="O11" s="8" t="n">
+        <f aca="false">IFERROR(N11/12,0)</f>
+        <v>151.25</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>350</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <f aca="false">SUM(B12:M12)</f>
+        <v>3750</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <f aca="false">IFERROR(N12/12,0)</f>
+        <v>312.5</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>929.82</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>24.95</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>414.48</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>308.67</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>293.04</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>555</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="J13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="K13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="L13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="M13" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <f aca="false">SUM(B13:M13)</f>
+        <v>4566.96</v>
+      </c>
+      <c r="O13" s="8" t="n">
+        <f aca="false">IFERROR(N13/12,0)</f>
+        <v>380.58</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>482.29</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10" t="n">
+        <f aca="false">SUM(B14:M14)</f>
+        <v>482.29</v>
+      </c>
+      <c r="O14" s="10" t="n">
+        <f aca="false">IFERROR(N14/12,0)</f>
+        <v>40.1908333333333</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="10" t="n">
+        <f aca="false">SUM(B6:B14)</f>
+        <v>3331.82</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <f aca="false">SUM(C6:C14)</f>
+        <v>5260.29</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <f aca="false">SUM(D6:D14)</f>
+        <v>5299.24</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <f aca="false">SUM(E6:E14)</f>
+        <v>5927.48</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <f aca="false">SUM(F6:F14)</f>
+        <v>3101.92</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <f aca="false">SUM(G6:G14)</f>
+        <v>9763.04</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <f aca="false">SUM(H6:H14)</f>
+        <v>3387</v>
+      </c>
+      <c r="I15" s="10" t="n">
+        <f aca="false">SUM(I6:I14)</f>
+        <v>5371</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <f aca="false">SUM(J6:J14)</f>
+        <v>5371</v>
+      </c>
+      <c r="K15" s="10" t="n">
+        <f aca="false">SUM(K6:K14)</f>
+        <v>5371</v>
+      </c>
+      <c r="L15" s="10" t="n">
+        <f aca="false">SUM(L6:L14)</f>
+        <v>5371</v>
+      </c>
+      <c r="M15" s="10" t="n">
+        <f aca="false">SUM(M6:M14)</f>
+        <v>5371</v>
+      </c>
+      <c r="N15" s="10" t="n">
+        <f aca="false">SUM(N6:N14)</f>
+        <v>40944.25</v>
+      </c>
+      <c r="O15" s="10" t="n">
+        <f aca="false">IFERROR(N15/12,0)</f>
+        <v>3412.02083333333</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6"/>
+    </row>
+    <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>154</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>141</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>141</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>142</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>142</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>162</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>142</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>134</v>
+      </c>
+      <c r="J17" s="8" t="n">
+        <v>134</v>
+      </c>
+      <c r="K17" s="8" t="n">
+        <v>134</v>
+      </c>
+      <c r="L17" s="8" t="n">
+        <v>134</v>
+      </c>
+      <c r="M17" s="8" t="n">
+        <v>134</v>
+      </c>
+      <c r="N17" s="8" t="n">
+        <f aca="false">SUM(B17:M17)</f>
+        <v>1694</v>
+      </c>
+      <c r="O17" s="8" t="n">
+        <f aca="false">IFERROR(N17/12,0)</f>
+        <v>141.166666666667</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="I18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="J18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="K18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="L18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="M18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="N18" s="8" t="n">
+        <f aca="false">SUM(B18:M18)</f>
+        <v>423</v>
+      </c>
+      <c r="O18" s="8" t="n">
+        <f aca="false">IFERROR(N18/12,0)</f>
+        <v>35.25</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E19" s="8"/>
+      <c r="F19" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="J19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="K19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="L19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="M19" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="N19" s="8" t="n">
+        <f aca="false">SUM(B19:M19)</f>
+        <v>891</v>
+      </c>
+      <c r="O19" s="8" t="n">
+        <f aca="false">IFERROR(N19/12,0)</f>
+        <v>74.25</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="I20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="J20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="K20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="L20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="M20" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="N20" s="8" t="n">
+        <f aca="false">SUM(B20:M20)</f>
+        <v>725</v>
+      </c>
+      <c r="O20" s="8" t="n">
+        <f aca="false">IFERROR(N20/12,0)</f>
+        <v>60.4166666666667</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>92</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="J21" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="K21" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="L21" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="M21" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="N21" s="8" t="n">
+        <f aca="false">SUM(B21:M21)</f>
+        <v>872</v>
+      </c>
+      <c r="O21" s="8" t="n">
+        <f aca="false">IFERROR(N21/12,0)</f>
+        <v>72.6666666666667</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8" t="n">
+        <v>561</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8" t="n">
+        <v>377</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>173</v>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>159</v>
+      </c>
+      <c r="H22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="I22" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="J22" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="K22" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="L22" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <f aca="false">SUM(B22:M22)</f>
+        <v>2651</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <f aca="false">IFERROR(N22/12,0)</f>
+        <v>220.916666666667</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>254</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>254</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <f aca="false">SUM(B23:M23)</f>
+        <v>3048</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <f aca="false">IFERROR(N23/12,0)</f>
+        <v>254</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="H24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="I24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="J24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="K24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="L24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="M24" s="8" t="n">
+        <v>147</v>
+      </c>
+      <c r="N24" s="8" t="n">
+        <f aca="false">SUM(B24:M24)</f>
+        <v>1764</v>
+      </c>
+      <c r="O24" s="8" t="n">
+        <f aca="false">IFERROR(N24/12,0)</f>
+        <v>147</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="8" t="n">
+        <v>164</v>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>283</v>
+      </c>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="K25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="L25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="M25" s="8" t="n">
+        <v>282</v>
+      </c>
+      <c r="N25" s="8" t="n">
+        <f aca="false">SUM(B25:M25)</f>
+        <v>2524</v>
+      </c>
+      <c r="O25" s="8" t="n">
+        <f aca="false">IFERROR(N25/12,0)</f>
+        <v>210.333333333333</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="K26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="L26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="M26" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="N26" s="8" t="n">
+        <f aca="false">SUM(B26:M26)</f>
+        <v>660</v>
+      </c>
+      <c r="O26" s="8" t="n">
+        <f aca="false">IFERROR(N26/12,0)</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="8" t="n">
+        <v>219</v>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>157</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>123</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="J27" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="K27" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="L27" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="M27" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="N27" s="8" t="n">
+        <f aca="false">SUM(B27:M27)</f>
+        <v>1527</v>
+      </c>
+      <c r="O27" s="8" t="n">
+        <f aca="false">IFERROR(N27/12,0)</f>
+        <v>127.25</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F28" s="9"/>
+      <c r="G28" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H28" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8" t="n">
+        <f aca="false">SUM(B28:M28)</f>
+        <v>3104</v>
+      </c>
+      <c r="O28" s="8" t="n">
+        <f aca="false">IFERROR(N28/12,0)</f>
+        <v>258.666666666667</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8" t="n">
+        <v>494</v>
+      </c>
+      <c r="F29" s="9"/>
+      <c r="G29" s="8" t="n">
+        <v>466</v>
+      </c>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="K29" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="L29" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="M29" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="N29" s="8" t="n">
+        <f aca="false">SUM(B29:M29)</f>
+        <v>1620</v>
+      </c>
+      <c r="O29" s="8" t="n">
+        <f aca="false">IFERROR(N29/12,0)</f>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="G30" s="8"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="8"/>
+      <c r="M30" s="8"/>
+      <c r="N30" s="8" t="n">
+        <f aca="false">SUM(B30:M30)</f>
+        <v>1700</v>
+      </c>
+      <c r="O30" s="8" t="n">
+        <f aca="false">IFERROR(N30/12,0)</f>
+        <v>141.666666666667</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" s="10" t="n">
+        <f aca="false">SUM(B17:B30)</f>
+        <v>1948</v>
+      </c>
+      <c r="C31" s="10" t="n">
+        <f aca="false">SUM(C17:C30)</f>
+        <v>1847</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <f aca="false">SUM(D17:D30)</f>
+        <v>1255</v>
+      </c>
+      <c r="E31" s="10" t="n">
+        <f aca="false">SUM(E17:E30)</f>
+        <v>4835</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <f aca="false">SUM(F17:F30)</f>
+        <v>1717</v>
+      </c>
+      <c r="G31" s="10" t="n">
+        <f aca="false">SUM(G17:G30)</f>
+        <v>2553</v>
+      </c>
+      <c r="H31" s="10" t="n">
+        <f aca="false">SUM(H17:H30)</f>
+        <v>1310</v>
+      </c>
+      <c r="I31" s="10" t="n">
+        <f aca="false">SUM(I17:I30)</f>
+        <v>1142</v>
+      </c>
+      <c r="J31" s="10" t="n">
+        <f aca="false">SUM(J17:J30)</f>
+        <v>1649</v>
+      </c>
+      <c r="K31" s="10" t="n">
+        <f aca="false">SUM(K17:K30)</f>
+        <v>1649</v>
+      </c>
+      <c r="L31" s="10" t="n">
+        <f aca="false">SUM(L17:L30)</f>
+        <v>1649</v>
+      </c>
+      <c r="M31" s="10" t="n">
+        <f aca="false">SUM(M17:M30)</f>
+        <v>1649</v>
+      </c>
+      <c r="N31" s="10" t="n">
+        <f aca="false">SUM(N17:N30)</f>
+        <v>23203</v>
+      </c>
+      <c r="O31" s="10" t="n">
+        <f aca="false">IFERROR(N31/12,0)</f>
+        <v>1933.58333333333</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="6"/>
+      <c r="K32" s="6"/>
+      <c r="L32" s="6"/>
+      <c r="M32" s="6"/>
+    </row>
+    <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>227.99</v>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>124.82</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>292.02</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>545.19</v>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>294.9</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>253.4</v>
+      </c>
+      <c r="H33" s="8" t="n">
+        <v>801</v>
+      </c>
+      <c r="I33" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="J33" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="K33" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="L33" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="M33" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="N33" s="8" t="n">
+        <f aca="false">SUM(B33:M33)</f>
+        <v>3714.32</v>
+      </c>
+      <c r="O33" s="8" t="n">
+        <f aca="false">IFERROR(N33/12,0)</f>
+        <v>309.526666666667</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" s="8" t="n">
+        <v>221.2</v>
+      </c>
+      <c r="C34" s="8" t="n">
+        <v>171.55</v>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>383.95</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>229.3</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>306.85</v>
+      </c>
+      <c r="G34" s="8" t="n">
+        <v>336.47</v>
+      </c>
+      <c r="H34" s="8" t="n">
+        <v>579</v>
+      </c>
+      <c r="I34" s="8" t="n">
+        <v>453</v>
+      </c>
+      <c r="J34" s="8" t="n">
+        <v>453</v>
+      </c>
+      <c r="K34" s="8" t="n">
+        <v>453</v>
+      </c>
+      <c r="L34" s="8" t="n">
+        <v>453</v>
+      </c>
+      <c r="M34" s="8" t="n">
+        <v>453</v>
+      </c>
+      <c r="N34" s="8" t="n">
+        <f aca="false">SUM(B34:M34)</f>
+        <v>4493.32</v>
+      </c>
+      <c r="O34" s="8" t="n">
+        <f aca="false">IFERROR(N34/12,0)</f>
+        <v>374.443333333333</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" s="8" t="n">
+        <v>294.02</v>
+      </c>
+      <c r="C35" s="8" t="n">
+        <v>283.98</v>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>224.88</v>
+      </c>
+      <c r="E35" s="8" t="n">
+        <v>235.2</v>
+      </c>
+      <c r="F35" s="9" t="n">
+        <v>543.78</v>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>744.23</v>
+      </c>
+      <c r="H35" s="8" t="n">
+        <v>876</v>
+      </c>
+      <c r="I35" s="8" t="n">
+        <v>593</v>
+      </c>
+      <c r="J35" s="8" t="n">
+        <v>593</v>
+      </c>
+      <c r="K35" s="8" t="n">
+        <v>593</v>
+      </c>
+      <c r="L35" s="8" t="n">
+        <v>593</v>
+      </c>
+      <c r="M35" s="8" t="n">
+        <v>593</v>
+      </c>
+      <c r="N35" s="8" t="n">
+        <f aca="false">SUM(B35:M35)</f>
+        <v>6167.09</v>
+      </c>
+      <c r="O35" s="8" t="n">
+        <f aca="false">IFERROR(N35/12,0)</f>
+        <v>513.924166666667</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" s="8" t="n">
+        <v>188.29</v>
+      </c>
+      <c r="C36" s="8" t="n">
+        <v>13.92</v>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>160</v>
+      </c>
+      <c r="F36" s="9" t="n">
+        <v>190.08</v>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="H36" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="I36" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="J36" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="K36" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="L36" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="M36" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="N36" s="8" t="n">
+        <f aca="false">SUM(B36:M36)</f>
+        <v>1189.19</v>
+      </c>
+      <c r="O36" s="8" t="n">
+        <f aca="false">IFERROR(N36/12,0)</f>
+        <v>99.0991666666667</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" s="8" t="n">
+        <v>90.99</v>
+      </c>
+      <c r="C37" s="8" t="n">
+        <v>268.78</v>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>444.59</v>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>203.99</v>
+      </c>
+      <c r="F37" s="9" t="n">
+        <v>375.39</v>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>86.29</v>
+      </c>
+      <c r="H37" s="8" t="n">
+        <v>559</v>
+      </c>
+      <c r="I37" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="J37" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="K37" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="L37" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="M37" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="N37" s="8" t="n">
+        <f aca="false">SUM(B37:M37)</f>
+        <v>3704.03</v>
+      </c>
+      <c r="O37" s="8" t="n">
+        <f aca="false">IFERROR(N37/12,0)</f>
+        <v>308.669166666667</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="8" t="n">
+        <v>746.99</v>
+      </c>
+      <c r="C38" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>780.34</v>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>841.59</v>
+      </c>
+      <c r="F38" s="9" t="n">
+        <v>275.93</v>
+      </c>
+      <c r="G38" s="8" t="n">
+        <v>529.05</v>
+      </c>
+      <c r="H38" s="8" t="n">
+        <v>395</v>
+      </c>
+      <c r="I38" s="8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8"/>
+      <c r="N38" s="8" t="n">
+        <f aca="false">SUM(B38:M38)</f>
+        <v>5198.9</v>
+      </c>
+      <c r="O38" s="8" t="n">
+        <f aca="false">IFERROR(N38/12,0)</f>
+        <v>433.241666666667</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" s="8" t="n">
+        <v>552.8</v>
+      </c>
+      <c r="C39" s="8" t="n">
+        <v>1131.64</v>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>941.05</v>
+      </c>
+      <c r="E39" s="8" t="n">
+        <v>840.67</v>
+      </c>
+      <c r="F39" s="9" t="n">
+        <v>796.49</v>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>1313.86</v>
+      </c>
+      <c r="H39" s="8" t="n">
+        <v>1528</v>
+      </c>
+      <c r="I39" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="J39" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="K39" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="L39" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="M39" s="8" t="n">
+        <v>725</v>
+      </c>
+      <c r="N39" s="8" t="n">
+        <f aca="false">SUM(B39:M39)</f>
+        <v>10729.51</v>
+      </c>
+      <c r="O39" s="8" t="n">
+        <f aca="false">IFERROR(N39/12,0)</f>
+        <v>894.125833333333</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B40" s="10" t="n">
+        <f aca="false">SUM(B33:B39)</f>
+        <v>2322.28</v>
+      </c>
+      <c r="C40" s="10" t="n">
+        <f aca="false">SUM(C33:C39)</f>
+        <v>2124.69</v>
+      </c>
+      <c r="D40" s="10" t="n">
+        <f aca="false">SUM(D33:D39)</f>
+        <v>3066.83</v>
+      </c>
+      <c r="E40" s="10" t="n">
+        <f aca="false">SUM(E33:E39)</f>
+        <v>3055.94</v>
+      </c>
+      <c r="F40" s="11" t="n">
+        <f aca="false">SUM(F33:F39)</f>
+        <v>2783.42</v>
+      </c>
+      <c r="G40" s="10" t="n">
+        <f aca="false">SUM(G33:G39)</f>
+        <v>3301.2</v>
+      </c>
+      <c r="H40" s="10" t="n">
+        <f aca="false">SUM(H33:H39)</f>
+        <v>4782</v>
+      </c>
+      <c r="I40" s="10" t="n">
+        <f aca="false">SUM(I33:I39)</f>
+        <v>3952</v>
+      </c>
+      <c r="J40" s="10" t="n">
+        <f aca="false">SUM(J33:J39)</f>
+        <v>2452</v>
+      </c>
+      <c r="K40" s="10" t="n">
+        <f aca="false">SUM(K33:K39)</f>
+        <v>2452</v>
+      </c>
+      <c r="L40" s="10" t="n">
+        <f aca="false">SUM(L33:L39)</f>
+        <v>2452</v>
+      </c>
+      <c r="M40" s="10" t="n">
+        <f aca="false">SUM(M33:M39)</f>
+        <v>2452</v>
+      </c>
+      <c r="N40" s="10" t="n">
+        <f aca="false">SUM(N33:N39)</f>
+        <v>35196.36</v>
+      </c>
+      <c r="O40" s="10" t="n">
+        <f aca="false">IFERROR(N40/12,0)</f>
+        <v>2933.03</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="12" t="n">
+        <f aca="false">B31+B40</f>
+        <v>4270.28</v>
+      </c>
+      <c r="C41" s="12" t="n">
+        <f aca="false">C31+C40</f>
+        <v>3971.69</v>
+      </c>
+      <c r="D41" s="12" t="n">
+        <f aca="false">D31+D40</f>
+        <v>4321.83</v>
+      </c>
+      <c r="E41" s="12" t="n">
+        <f aca="false">E31+E40</f>
+        <v>7890.94</v>
+      </c>
+      <c r="F41" s="12" t="n">
+        <f aca="false">F31+F40</f>
+        <v>4500.42</v>
+      </c>
+      <c r="G41" s="12" t="n">
+        <f aca="false">G31+G40</f>
+        <v>5854.2</v>
+      </c>
+      <c r="H41" s="12" t="n">
+        <f aca="false">H31+H40</f>
+        <v>6092</v>
+      </c>
+      <c r="I41" s="12" t="n">
+        <f aca="false">I31+I40</f>
+        <v>5094</v>
+      </c>
+      <c r="J41" s="12" t="n">
+        <f aca="false">J31+J40</f>
+        <v>4101</v>
+      </c>
+      <c r="K41" s="12" t="n">
+        <f aca="false">K31+K40</f>
+        <v>4101</v>
+      </c>
+      <c r="L41" s="12" t="n">
+        <f aca="false">L31+L40</f>
+        <v>4101</v>
+      </c>
+      <c r="M41" s="12" t="n">
+        <f aca="false">M31+M40</f>
+        <v>4101</v>
+      </c>
+      <c r="N41" s="12" t="n">
+        <f aca="false">N31+N40</f>
+        <v>58399.36</v>
+      </c>
+      <c r="O41" s="12" t="n">
+        <f aca="false">IFERROR(N41/12,0)</f>
+        <v>4866.61333333333</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="13" t="n">
+        <f aca="false">B15-B31-B40</f>
+        <v>-938.46</v>
+      </c>
+      <c r="C42" s="13" t="n">
+        <f aca="false">C15-C31-C40</f>
+        <v>1288.6</v>
+      </c>
+      <c r="D42" s="13" t="n">
+        <f aca="false">D15-D31-D40</f>
+        <v>977.41</v>
+      </c>
+      <c r="E42" s="13" t="n">
+        <f aca="false">E15-E31-E40</f>
+        <v>-1963.46</v>
+      </c>
+      <c r="F42" s="13" t="n">
+        <f aca="false">F15-F31-F40</f>
+        <v>-1398.5</v>
+      </c>
+      <c r="G42" s="13" t="n">
+        <f aca="false">G15-G31-G40</f>
+        <v>3908.84</v>
+      </c>
+      <c r="H42" s="13" t="n">
+        <f aca="false">H15-H31-H40</f>
+        <v>-2705</v>
+      </c>
+      <c r="I42" s="13" t="n">
+        <f aca="false">I15-I31-I40</f>
+        <v>277</v>
+      </c>
+      <c r="J42" s="13" t="n">
+        <f aca="false">J15-J31-J40</f>
+        <v>1270</v>
+      </c>
+      <c r="K42" s="13" t="n">
+        <f aca="false">K15-K31-K40</f>
+        <v>1270</v>
+      </c>
+      <c r="L42" s="13" t="n">
+        <f aca="false">L15-L31-L40</f>
+        <v>1270</v>
+      </c>
+      <c r="M42" s="13" t="n">
+        <f aca="false">M15-M31-M40</f>
+        <v>1270</v>
+      </c>
+      <c r="N42" s="13" t="n">
+        <f aca="false">N15-N31-N40</f>
+        <v>-17455.11</v>
+      </c>
+      <c r="O42" s="13" t="n">
+        <f aca="false">IFERROR(N42/12,0)</f>
+        <v>-1454.5925</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B43" s="13" t="n">
+        <v>-29</v>
+      </c>
+      <c r="C43" s="13" t="n">
+        <v>1540</v>
+      </c>
+      <c r="D43" s="13" t="n">
+        <v>2525</v>
+      </c>
+      <c r="E43" s="13" t="n">
+        <v>729</v>
+      </c>
+      <c r="F43" s="13" t="n">
+        <v>934</v>
+      </c>
+      <c r="G43" s="13" t="n">
+        <v>4978</v>
+      </c>
+      <c r="H43" s="13" t="n">
+        <v>2355</v>
+      </c>
+      <c r="I43" s="13" t="n">
+        <v>2632</v>
+      </c>
+      <c r="J43" s="13" t="n">
+        <v>3902</v>
+      </c>
+      <c r="K43" s="13" t="n">
+        <v>5172</v>
+      </c>
+      <c r="L43" s="13" t="n">
+        <v>6442</v>
+      </c>
+      <c r="M43" s="13" t="n">
+        <v>7712</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="14"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="14"/>
+      <c r="J45" s="14"/>
+      <c r="K45" s="14"/>
+      <c r="L45" s="14"/>
+      <c r="M45" s="14"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B46" s="13" t="n">
+        <f aca="false">B15-B31</f>
+        <v>1383.82</v>
+      </c>
+      <c r="C46" s="13" t="n">
+        <f aca="false">C15-C31</f>
+        <v>3413.29</v>
+      </c>
+      <c r="D46" s="13" t="n">
+        <f aca="false">D15-D31</f>
+        <v>4044.24</v>
+      </c>
+      <c r="E46" s="13" t="n">
+        <f aca="false">E15-E31</f>
+        <v>1092.48</v>
+      </c>
+      <c r="F46" s="13" t="n">
+        <f aca="false">F15-F31</f>
+        <v>1384.92</v>
+      </c>
+      <c r="G46" s="13" t="n">
+        <f aca="false">G15-G31</f>
+        <v>7210.04</v>
+      </c>
+      <c r="H46" s="13" t="n">
+        <f aca="false">H15-H31</f>
+        <v>2077</v>
+      </c>
+      <c r="I46" s="13" t="n">
+        <f aca="false">I15-I31</f>
+        <v>4229</v>
+      </c>
+      <c r="J46" s="13" t="n">
+        <f aca="false">J15-J31</f>
+        <v>3722</v>
+      </c>
+      <c r="K46" s="13" t="n">
+        <f aca="false">K15-K31</f>
+        <v>3722</v>
+      </c>
+      <c r="L46" s="13" t="n">
+        <f aca="false">L15-L31</f>
+        <v>3722</v>
+      </c>
+      <c r="M46" s="13" t="n">
+        <f aca="false">M15-M31</f>
+        <v>3722</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B47" s="13" t="n">
+        <f aca="false">B42</f>
+        <v>-938.46</v>
+      </c>
+      <c r="C47" s="13" t="n">
+        <f aca="false">C42</f>
+        <v>1288.6</v>
+      </c>
+      <c r="D47" s="13" t="n">
+        <f aca="false">D42</f>
+        <v>977.41</v>
+      </c>
+      <c r="E47" s="13" t="n">
+        <f aca="false">E42</f>
+        <v>-1963.46</v>
+      </c>
+      <c r="F47" s="13" t="n">
+        <f aca="false">F42</f>
+        <v>-1398.5</v>
+      </c>
+      <c r="G47" s="13" t="n">
+        <f aca="false">G42</f>
+        <v>3908.84</v>
+      </c>
+      <c r="H47" s="13" t="n">
+        <f aca="false">H42</f>
+        <v>-2705</v>
+      </c>
+      <c r="I47" s="13" t="n">
+        <f aca="false">I42</f>
+        <v>277</v>
+      </c>
+      <c r="J47" s="13" t="n">
+        <f aca="false">J42</f>
+        <v>1270</v>
+      </c>
+      <c r="K47" s="13" t="n">
+        <f aca="false">K42</f>
+        <v>1270</v>
+      </c>
+      <c r="L47" s="13" t="n">
+        <f aca="false">L42</f>
+        <v>1270</v>
+      </c>
+      <c r="M47" s="13" t="n">
+        <f aca="false">M42</f>
+        <v>1270</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A16:M16"/>
+    <mergeCell ref="A32:M32"/>
+    <mergeCell ref="A45:M45"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -962,7 +3051,7 @@
       <c r="O1" s="15"/>
       <c r="P1" s="15"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
         <v>61</v>
       </c>
@@ -982,7 +3071,7 @@
       <c r="O2" s="16"/>
       <c r="P2" s="16"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
         <v>62</v>
       </c>
@@ -1026,33 +3115,33 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
         <v>76</v>
       </c>
       <c r="B5" s="20" t="n">
-        <v>659</v>
+        <v>79</v>
       </c>
       <c r="C5" s="20" t="n">
-        <v>344.8</v>
+        <v>184.8</v>
       </c>
       <c r="D5" s="20" t="n">
-        <v>1153.54</v>
+        <v>432.6</v>
       </c>
       <c r="E5" s="20" t="n">
-        <v>1008.59</v>
+        <v>167</v>
       </c>
       <c r="F5" s="20" t="n">
-        <v>276.83</v>
+        <v>20.4</v>
       </c>
       <c r="G5" s="20" t="n">
-        <v>602.55</v>
+        <v>74.3</v>
       </c>
       <c r="H5" s="20" t="n">
-        <v>954</v>
+        <v>559</v>
       </c>
       <c r="I5" s="20" t="n">
-        <v>1835</v>
+        <v>335</v>
       </c>
       <c r="J5" s="20" t="n">
         <v>335</v>
@@ -1068,622 +3157,673 @@
       </c>
       <c r="N5" s="21" t="n">
         <f aca="false">SUM(B5:M5)</f>
-        <v>8174.31</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+        <v>3192.1</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="B6" s="20" t="n">
-        <v>449.19</v>
-      </c>
-      <c r="C6" s="20" t="n">
-        <v>296.37</v>
-      </c>
-      <c r="D6" s="20" t="n">
-        <v>675.97</v>
-      </c>
-      <c r="E6" s="20" t="n">
-        <v>774.49</v>
-      </c>
-      <c r="F6" s="20" t="n">
-        <v>601.75</v>
-      </c>
-      <c r="G6" s="20" t="n">
-        <v>589.87</v>
-      </c>
-      <c r="H6" s="20" t="n">
-        <v>1380</v>
-      </c>
-      <c r="I6" s="20" t="n">
-        <v>688</v>
-      </c>
-      <c r="J6" s="20" t="n">
-        <v>688</v>
-      </c>
-      <c r="K6" s="20" t="n">
-        <v>688</v>
-      </c>
-      <c r="L6" s="20" t="n">
-        <v>688</v>
-      </c>
-      <c r="M6" s="20" t="n">
-        <v>688</v>
-      </c>
-      <c r="N6" s="21" t="n">
+      <c r="B6" s="23" t="n">
+        <v>580</v>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>160</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>720.94</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <v>841.59</v>
+      </c>
+      <c r="F6" s="23" t="n">
+        <v>256.43</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>528.25</v>
+      </c>
+      <c r="H6" s="23" t="n">
+        <v>395</v>
+      </c>
+      <c r="I6" s="23" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="24" t="n">
         <f aca="false">SUM(B6:M6)</f>
-        <v>8207.64</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>4982.21</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
         <v>78</v>
       </c>
       <c r="B7" s="20" t="n">
-        <v>368.94</v>
+        <v>449.19</v>
       </c>
       <c r="C7" s="20" t="n">
-        <v>465.14</v>
+        <v>296.37</v>
       </c>
       <c r="D7" s="20" t="n">
-        <v>593.81</v>
+        <v>675.97</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>508.92</v>
+        <v>774.49</v>
       </c>
       <c r="F7" s="20" t="n">
-        <v>1003.27</v>
+        <v>601.75</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>1089.35</v>
+        <v>589.87</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>876</v>
+        <v>1380</v>
       </c>
       <c r="I7" s="20" t="n">
-        <v>593</v>
+        <v>688</v>
       </c>
       <c r="J7" s="20" t="n">
-        <v>593</v>
+        <v>688</v>
       </c>
       <c r="K7" s="20" t="n">
-        <v>593</v>
+        <v>688</v>
       </c>
       <c r="L7" s="20" t="n">
-        <v>593</v>
+        <v>688</v>
       </c>
       <c r="M7" s="20" t="n">
-        <v>593</v>
+        <v>688</v>
       </c>
       <c r="N7" s="21" t="n">
         <f aca="false">SUM(B7:M7)</f>
-        <v>7870.43</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>8207.64</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
         <v>79</v>
       </c>
       <c r="B8" s="20" t="n">
-        <v>635.87</v>
+        <v>368.94</v>
       </c>
       <c r="C8" s="20" t="n">
-        <v>417.84</v>
+        <v>465.14</v>
       </c>
       <c r="D8" s="20" t="n">
-        <v>428.22</v>
+        <v>593.81</v>
       </c>
       <c r="E8" s="20" t="n">
-        <v>266.49</v>
+        <v>508.92</v>
       </c>
       <c r="F8" s="20" t="n">
-        <v>420.31</v>
+        <v>1003.27</v>
       </c>
       <c r="G8" s="20" t="n">
-        <v>326.99</v>
+        <v>1089.35</v>
       </c>
       <c r="H8" s="20" t="n">
-        <v>265</v>
+        <v>876</v>
       </c>
       <c r="I8" s="20" t="n">
-        <v>264</v>
+        <v>593</v>
       </c>
       <c r="J8" s="20" t="n">
-        <v>264</v>
+        <v>593</v>
       </c>
       <c r="K8" s="20" t="n">
-        <v>264</v>
+        <v>593</v>
       </c>
       <c r="L8" s="20" t="n">
-        <v>264</v>
+        <v>593</v>
       </c>
       <c r="M8" s="20" t="n">
-        <v>264</v>
+        <v>593</v>
       </c>
       <c r="N8" s="21" t="n">
         <f aca="false">SUM(B8:M8)</f>
-        <v>4080.72</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>7870.43</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
         <v>80</v>
       </c>
       <c r="B9" s="20" t="n">
-        <v>142.41</v>
+        <v>544.73</v>
       </c>
       <c r="C9" s="20" t="n">
-        <v>642</v>
+        <v>334.39</v>
       </c>
       <c r="D9" s="20" t="n">
-        <v>126.42</v>
+        <v>344.77</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>377</v>
+        <v>182.45</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>276.85</v>
+        <v>336.27</v>
       </c>
       <c r="G9" s="20" t="n">
-        <v>337.13</v>
+        <v>231.12</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>287</v>
+        <v>180.96</v>
       </c>
       <c r="I9" s="20" t="n">
-        <v>316</v>
+        <v>184.7</v>
       </c>
       <c r="J9" s="20" t="n">
-        <v>316</v>
+        <v>184.7</v>
       </c>
       <c r="K9" s="20" t="n">
-        <v>316</v>
+        <v>184.7</v>
       </c>
       <c r="L9" s="20" t="n">
-        <v>316</v>
+        <v>184.7</v>
       </c>
       <c r="M9" s="20" t="n">
-        <v>316</v>
+        <v>184.7</v>
       </c>
       <c r="N9" s="21" t="n">
         <f aca="false">SUM(B9:M9)</f>
-        <v>3768.81</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3078.19</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
         <v>81</v>
       </c>
       <c r="B10" s="20" t="n">
-        <v>401</v>
+        <v>933.55</v>
       </c>
       <c r="C10" s="20" t="n">
-        <v>401</v>
+        <v>725.45</v>
       </c>
       <c r="D10" s="20" t="n">
-        <v>401</v>
+        <v>209.87</v>
       </c>
       <c r="E10" s="20" t="n">
-        <v>401</v>
+        <v>1861.04</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>401</v>
+        <v>360.89</v>
       </c>
       <c r="G10" s="20" t="n">
-        <v>401</v>
+        <v>1433</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>401</v>
+        <v>375.04</v>
       </c>
       <c r="I10" s="20" t="n">
-        <v>401</v>
+        <v>395.3</v>
       </c>
       <c r="J10" s="20" t="n">
-        <v>401</v>
+        <v>395.3</v>
       </c>
       <c r="K10" s="20" t="n">
-        <v>401</v>
+        <v>395.3</v>
       </c>
       <c r="L10" s="20" t="n">
-        <v>401</v>
+        <v>395.3</v>
       </c>
       <c r="M10" s="20" t="n">
-        <v>401</v>
+        <v>395.3</v>
       </c>
       <c r="N10" s="21" t="n">
         <f aca="false">SUM(B10:M10)</f>
-        <v>4812</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>7875.34</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
         <v>82</v>
       </c>
       <c r="B11" s="20" t="n">
-        <v>224</v>
+        <v>401</v>
       </c>
       <c r="C11" s="20" t="n">
-        <v>342</v>
+        <v>401</v>
       </c>
       <c r="D11" s="20" t="n">
-        <v>342</v>
+        <v>401</v>
       </c>
       <c r="E11" s="20" t="n">
-        <v>836</v>
+        <v>401</v>
       </c>
       <c r="F11" s="20" t="n">
-        <v>686</v>
+        <v>401</v>
       </c>
       <c r="G11" s="20" t="n">
-        <v>526</v>
+        <v>401</v>
       </c>
       <c r="H11" s="20" t="n">
-        <v>163</v>
-      </c>
-      <c r="I11" s="20"/>
+        <v>401</v>
+      </c>
+      <c r="I11" s="20" t="n">
+        <v>401</v>
+      </c>
       <c r="J11" s="20" t="n">
-        <v>507</v>
+        <v>401</v>
       </c>
       <c r="K11" s="20" t="n">
-        <v>507</v>
+        <v>401</v>
       </c>
       <c r="L11" s="20" t="n">
-        <v>507</v>
+        <v>401</v>
       </c>
       <c r="M11" s="20" t="n">
-        <v>507</v>
+        <v>401</v>
       </c>
       <c r="N11" s="21" t="n">
         <f aca="false">SUM(B11:M11)</f>
-        <v>5147</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>4812</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
         <v>83</v>
       </c>
       <c r="B12" s="20" t="n">
-        <v>700</v>
-      </c>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
+        <v>224</v>
+      </c>
+      <c r="C12" s="20" t="n">
+        <v>342</v>
+      </c>
+      <c r="D12" s="20" t="n">
+        <v>342</v>
+      </c>
       <c r="E12" s="20" t="n">
-        <v>2936.99</v>
+        <v>836</v>
       </c>
       <c r="F12" s="20" t="n">
-        <v>226.78</v>
+        <v>686</v>
       </c>
       <c r="G12" s="20" t="n">
-        <v>1021.6</v>
+        <v>526</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>4</v>
+        <v>163</v>
       </c>
       <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
-      <c r="L12" s="20"/>
-      <c r="M12" s="20"/>
+      <c r="J12" s="20" t="n">
+        <v>507</v>
+      </c>
+      <c r="K12" s="20" t="n">
+        <v>507</v>
+      </c>
+      <c r="L12" s="20" t="n">
+        <v>507</v>
+      </c>
+      <c r="M12" s="20" t="n">
+        <v>507</v>
+      </c>
       <c r="N12" s="21" t="n">
         <f aca="false">SUM(B12:M12)</f>
-        <v>4889.37</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>5147</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="20" t="n">
-        <v>258.89</v>
-      </c>
-      <c r="C13" s="20" t="n">
-        <v>265.08</v>
-      </c>
-      <c r="D13" s="20" t="n">
-        <v>172.99</v>
-      </c>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
       <c r="E13" s="20" t="n">
-        <v>227.98</v>
+        <v>1536.99</v>
       </c>
       <c r="F13" s="20" t="n">
-        <v>217.99</v>
+        <v>226.78</v>
       </c>
       <c r="G13" s="20" t="n">
-        <v>194.99</v>
-      </c>
-      <c r="H13" s="20" t="n">
-        <v>190</v>
-      </c>
-      <c r="I13" s="20" t="n">
-        <v>161</v>
-      </c>
-      <c r="J13" s="20" t="n">
-        <v>161</v>
-      </c>
-      <c r="K13" s="20" t="n">
-        <v>161</v>
-      </c>
-      <c r="L13" s="20" t="n">
-        <v>161</v>
-      </c>
-      <c r="M13" s="20" t="n">
-        <v>161</v>
-      </c>
+        <v>21.6</v>
+      </c>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="20"/>
+      <c r="L13" s="20"/>
+      <c r="M13" s="20"/>
       <c r="N13" s="21" t="n">
         <f aca="false">SUM(B13:M13)</f>
-        <v>2332.92</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1785.37</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
         <v>85</v>
       </c>
       <c r="B14" s="20" t="n">
-        <v>100</v>
+        <v>258.89</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>372.27</v>
+        <v>265.08</v>
       </c>
       <c r="D14" s="20" t="n">
-        <v>200</v>
-      </c>
-      <c r="E14" s="20"/>
+        <v>172.99</v>
+      </c>
+      <c r="E14" s="20" t="n">
+        <v>227.98</v>
+      </c>
       <c r="F14" s="20" t="n">
-        <v>150</v>
+        <v>217.99</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>242</v>
-      </c>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
-      <c r="K14" s="20"/>
-      <c r="L14" s="20"/>
-      <c r="M14" s="20"/>
+        <v>194.99</v>
+      </c>
+      <c r="H14" s="20" t="n">
+        <v>190</v>
+      </c>
+      <c r="I14" s="20" t="n">
+        <v>161</v>
+      </c>
+      <c r="J14" s="20" t="n">
+        <v>161</v>
+      </c>
+      <c r="K14" s="20" t="n">
+        <v>161</v>
+      </c>
+      <c r="L14" s="20" t="n">
+        <v>161</v>
+      </c>
+      <c r="M14" s="20" t="n">
+        <v>161</v>
+      </c>
       <c r="N14" s="21" t="n">
         <f aca="false">SUM(B14:M14)</f>
-        <v>1064.27</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2332.92</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
         <v>86</v>
       </c>
       <c r="B15" s="20" t="n">
-        <v>188.29</v>
+        <v>100</v>
       </c>
       <c r="C15" s="20" t="n">
-        <v>13.92</v>
-      </c>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20" t="n">
-        <v>160</v>
-      </c>
+        <v>372.27</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <v>200</v>
+      </c>
+      <c r="E15" s="20"/>
       <c r="F15" s="20" t="n">
-        <v>190.08</v>
+        <v>150</v>
       </c>
       <c r="G15" s="20" t="n">
-        <v>37.9</v>
-      </c>
-      <c r="H15" s="20" t="n">
-        <v>44</v>
-      </c>
-      <c r="I15" s="20" t="n">
-        <v>111</v>
-      </c>
-      <c r="J15" s="20" t="n">
-        <v>111</v>
-      </c>
-      <c r="K15" s="20" t="n">
-        <v>111</v>
-      </c>
-      <c r="L15" s="20" t="n">
-        <v>111</v>
-      </c>
-      <c r="M15" s="20" t="n">
-        <v>111</v>
-      </c>
+        <v>242</v>
+      </c>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="20"/>
+      <c r="M15" s="20"/>
       <c r="N15" s="21" t="n">
         <f aca="false">SUM(B15:M15)</f>
-        <v>1189.19</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1064.27</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
         <v>87</v>
       </c>
       <c r="B16" s="20" t="n">
-        <v>13.96</v>
+        <v>188.29</v>
       </c>
       <c r="C16" s="20" t="n">
-        <v>24.05</v>
-      </c>
-      <c r="D16" s="20" t="n">
-        <v>18.29</v>
-      </c>
+        <v>13.92</v>
+      </c>
+      <c r="D16" s="20"/>
       <c r="E16" s="20" t="n">
-        <v>13.55</v>
+        <v>160</v>
       </c>
       <c r="F16" s="20" t="n">
-        <v>14.25</v>
+        <v>190.08</v>
       </c>
       <c r="G16" s="20" t="n">
-        <v>18.78</v>
-      </c>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
-      <c r="L16" s="20"/>
-      <c r="M16" s="20"/>
+        <v>37.9</v>
+      </c>
+      <c r="H16" s="20" t="n">
+        <v>44</v>
+      </c>
+      <c r="I16" s="20" t="n">
+        <v>111</v>
+      </c>
+      <c r="J16" s="20" t="n">
+        <v>111</v>
+      </c>
+      <c r="K16" s="20" t="n">
+        <v>111</v>
+      </c>
+      <c r="L16" s="20" t="n">
+        <v>111</v>
+      </c>
+      <c r="M16" s="20" t="n">
+        <v>111</v>
+      </c>
       <c r="N16" s="21" t="n">
         <f aca="false">SUM(B16:M16)</f>
-        <v>102.88</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1189.19</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
         <v>88</v>
       </c>
       <c r="B17" s="20" t="n">
-        <v>142.69</v>
+        <v>13.96</v>
       </c>
       <c r="C17" s="20" t="n">
-        <v>316.27</v>
+        <v>24.05</v>
       </c>
       <c r="D17" s="20" t="n">
-        <v>227.88</v>
+        <v>18.29</v>
       </c>
       <c r="E17" s="20" t="n">
-        <v>393.48</v>
+        <v>13.55</v>
       </c>
       <c r="F17" s="20" t="n">
-        <v>49.56</v>
+        <v>14.25</v>
       </c>
       <c r="G17" s="20" t="n">
-        <v>427.82</v>
-      </c>
-      <c r="H17" s="20" t="n">
-        <v>1528</v>
-      </c>
-      <c r="I17" s="20" t="n">
-        <v>725</v>
-      </c>
-      <c r="J17" s="20" t="n">
-        <v>725</v>
-      </c>
-      <c r="K17" s="20" t="n">
-        <v>725</v>
-      </c>
-      <c r="L17" s="20" t="n">
-        <v>725</v>
-      </c>
-      <c r="M17" s="20" t="n">
-        <v>725</v>
-      </c>
+        <v>18.78</v>
+      </c>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
+      <c r="L17" s="20"/>
+      <c r="M17" s="20"/>
       <c r="N17" s="21" t="n">
         <f aca="false">SUM(B17:M17)</f>
-        <v>6710.7</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>102.88</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="B18" s="20"/>
+      <c r="B18" s="20" t="n">
+        <v>142.69</v>
+      </c>
       <c r="C18" s="20" t="n">
-        <v>95</v>
-      </c>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
+        <v>316.27</v>
+      </c>
+      <c r="D18" s="20" t="n">
+        <v>227.88</v>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>393.48</v>
+      </c>
+      <c r="F18" s="20" t="n">
+        <v>49.56</v>
+      </c>
       <c r="G18" s="20" t="n">
-        <v>57</v>
-      </c>
-      <c r="H18" s="20"/>
-      <c r="I18" s="20"/>
-      <c r="J18" s="20"/>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
-      <c r="M18" s="20"/>
+        <v>427.82</v>
+      </c>
+      <c r="H18" s="20" t="n">
+        <v>1528</v>
+      </c>
+      <c r="I18" s="20" t="n">
+        <v>725</v>
+      </c>
+      <c r="J18" s="20" t="n">
+        <v>725</v>
+      </c>
+      <c r="K18" s="20" t="n">
+        <v>725</v>
+      </c>
+      <c r="L18" s="20" t="n">
+        <v>725</v>
+      </c>
+      <c r="M18" s="20" t="n">
+        <v>725</v>
+      </c>
       <c r="N18" s="21" t="n">
         <f aca="false">SUM(B18:M18)</f>
+        <v>6710.7</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20" t="n">
+        <v>95</v>
+      </c>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20" t="n">
+        <v>57</v>
+      </c>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="20"/>
+      <c r="K19" s="20"/>
+      <c r="L19" s="20"/>
+      <c r="M19" s="20"/>
+      <c r="N19" s="21" t="n">
+        <f aca="false">SUM(B19:M19)</f>
         <v>152</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B19" s="23" t="n">
-        <f aca="false">SUM(B5:B18)</f>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="B20" s="26" t="n">
+        <f aca="false">SUM(B5:B19)</f>
         <v>4284.24</v>
       </c>
-      <c r="C19" s="23" t="n">
-        <f aca="false">SUM(C5:C18)</f>
+      <c r="C20" s="26" t="n">
+        <f aca="false">SUM(C5:C19)</f>
         <v>3995.74</v>
       </c>
-      <c r="D19" s="23" t="n">
-        <f aca="false">SUM(D5:D18)</f>
+      <c r="D20" s="26" t="n">
+        <f aca="false">SUM(D5:D19)</f>
         <v>4340.12</v>
       </c>
-      <c r="E19" s="23" t="n">
-        <f aca="false">SUM(E5:E18)</f>
+      <c r="E20" s="26" t="n">
+        <f aca="false">SUM(E5:E19)</f>
         <v>7904.49</v>
       </c>
-      <c r="F19" s="23" t="n">
-        <f aca="false">SUM(F5:F18)</f>
+      <c r="F20" s="26" t="n">
+        <f aca="false">SUM(F5:F19)</f>
         <v>4514.67</v>
       </c>
-      <c r="G19" s="23" t="n">
-        <f aca="false">SUM(G5:G18)</f>
+      <c r="G20" s="26" t="n">
+        <f aca="false">SUM(G5:G19)</f>
         <v>5872.98</v>
       </c>
-      <c r="H19" s="23" t="n">
-        <f aca="false">SUM(H5:H18)</f>
+      <c r="H20" s="26" t="n">
+        <f aca="false">SUM(H5:H19)</f>
         <v>6092</v>
       </c>
-      <c r="I19" s="23" t="n">
-        <f aca="false">SUM(I5:I18)</f>
+      <c r="I20" s="26" t="n">
+        <f aca="false">SUM(I5:I19)</f>
         <v>5094</v>
       </c>
-      <c r="J19" s="23" t="n">
-        <f aca="false">SUM(J5:J18)</f>
+      <c r="J20" s="26" t="n">
+        <f aca="false">SUM(J5:J19)</f>
         <v>4101</v>
       </c>
-      <c r="K19" s="23" t="n">
-        <f aca="false">SUM(K5:K18)</f>
+      <c r="K20" s="26" t="n">
+        <f aca="false">SUM(K5:K19)</f>
         <v>4101</v>
       </c>
-      <c r="L19" s="23" t="n">
-        <f aca="false">SUM(L5:L18)</f>
+      <c r="L20" s="26" t="n">
+        <f aca="false">SUM(L5:L19)</f>
         <v>4101</v>
       </c>
-      <c r="M19" s="23" t="n">
-        <f aca="false">SUM(M5:M18)</f>
+      <c r="M20" s="26" t="n">
+        <f aca="false">SUM(M5:M19)</f>
         <v>4101</v>
       </c>
-      <c r="N19" s="23" t="n">
-        <f aca="false">SUM(N5:N18)</f>
+      <c r="N20" s="26" t="n">
+        <f aca="false">SUM(N5:N19)</f>
         <v>58502.24</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="24" t="s">
-        <v>91</v>
-      </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24"/>
-      <c r="I21" s="24"/>
-      <c r="J21" s="24"/>
-      <c r="K21" s="24"/>
-      <c r="L21" s="24"/>
-      <c r="M21" s="24"/>
-      <c r="N21" s="24"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="27"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="27"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="B22" s="16"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="16"/>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="16"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="28"/>
+      <c r="J22" s="28"/>
+      <c r="K22" s="28"/>
+      <c r="L22" s="28"/>
+      <c r="M22" s="28"/>
+      <c r="N22" s="28"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="29" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="30" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="30" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="30" t="s">
+        <v>96</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>